<commit_message>
Added mining mastery via Mason trades (better pickaxes have better drop percentages)
</commit_message>
<xml_diff>
--- a/spoilers/conversations.xlsx
+++ b/spoilers/conversations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MYDATA\_GIT_REPOS\mcu4\spoilers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17D3BD67-77DE-4F54-910D-6FCEBFC3D53D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9CECD17-485C-455B-9951-B8304764D94E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="11964" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="191">
   <si>
     <t>Game-Level Conversation List</t>
   </si>
@@ -239,9 +239,6 @@
     <t>Welcomer: MOST of the day, Moongates will take you back to your stone circle!</t>
   </si>
   <si>
-    <t>Moongate Books!</t>
-  </si>
-  <si>
     <t>Question</t>
   </si>
   <si>
@@ -440,9 +437,6 @@
     <t>Pepper: The Rune is at the end of a Hallway!</t>
   </si>
   <si>
-    <t>Shepherd ("Bard"). Blocked pending predicate fix.</t>
-  </si>
-  <si>
     <t>Winston A.</t>
   </si>
   <si>
@@ -452,12 +446,6 @@
     <t>Shalimar and Cricket say the mantra.</t>
   </si>
   <si>
-    <t>Winston A.: Shalimar and Cricket say the mantra.</t>
-  </si>
-  <si>
-    <t>Blocked pending predicate fix.</t>
-  </si>
-  <si>
     <t>Winston T.</t>
   </si>
   <si>
@@ -467,33 +455,18 @@
     <t>The mantra is in Iolo's poem.</t>
   </si>
   <si>
-    <t>Winston T.: The mantra is in Iolo's poem.</t>
-  </si>
-  <si>
     <t>Winston L.</t>
   </si>
   <si>
     <t>Leatherworker</t>
   </si>
   <si>
-    <t>The Armorer loves to lie.</t>
-  </si>
-  <si>
-    <t>Winston L.: The Armorer loves to lie.</t>
-  </si>
-  <si>
     <t>Winston W.</t>
   </si>
   <si>
     <t>Weaponsmith</t>
   </si>
   <si>
-    <t>The Toolsmith loves to tell the truth.</t>
-  </si>
-  <si>
-    <t>Winston W.: The Toolsmith loves to tell the truth.</t>
-  </si>
-  <si>
     <t>Would you like to know more of potions?</t>
   </si>
   <si>
@@ -515,9 +488,6 @@
     <t>…MOST of the day will take you back to your stone circle!</t>
   </si>
   <si>
-    <t>…educate you on the LORE. I will trade you for one!</t>
-  </si>
-  <si>
     <t>Sebastian: Vegans show compassion in how they eat.</t>
   </si>
   <si>
@@ -567,6 +537,63 @@
   </si>
   <si>
     <t>Trades for a Secret..?</t>
+  </si>
+  <si>
+    <t>The Armorer loves to tell the truth.</t>
+  </si>
+  <si>
+    <t>The Toolsmith loves to lie.</t>
+  </si>
+  <si>
+    <t>Winston L.: The Toolsmith loves to lie.</t>
+  </si>
+  <si>
+    <t>Winston W.: The Armorer loves to tell the truth.</t>
+  </si>
+  <si>
+    <t>Metallurgy…</t>
+  </si>
+  <si>
+    <t>You can see that iron ingots aren't so easy to make, eh?</t>
+  </si>
+  <si>
+    <t>Iron Smelting…</t>
+  </si>
+  <si>
+    <t>L3 Trade or Above</t>
+  </si>
+  <si>
+    <t>Until you KNOW iron, you're not fit to hold ingots!</t>
+  </si>
+  <si>
+    <t>Towns…</t>
+  </si>
+  <si>
+    <t>Librarian Books…</t>
+  </si>
+  <si>
+    <t>Welcomer: BOOKS educate you on the LORE. I can trade you for one!</t>
+  </si>
+  <si>
+    <t>…educate you on the LORE. I can trade you for one!</t>
+  </si>
+  <si>
+    <t>Welcomer: This Land has 8 virtuous towns across 5 biomes!</t>
+  </si>
+  <si>
+    <t>…This land has 8 virtuous towns across 5 biomes!</t>
+  </si>
+  <si>
+    <t>Winston M.</t>
+  </si>
+  <si>
+    <t>Mason</t>
+  </si>
+  <si>
+    <t>I'm a Master Mason</t>
+  </si>
+  <si>
+    <t>I can teach you how to mine cobblestones!</t>
   </si>
 </sst>
 </file>
@@ -1243,7 +1270,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:O400"/>
+  <dimension ref="A1:O402"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1333,10 +1360,10 @@
       </c>
       <c r="H2" s="5"/>
       <c r="I2" s="8">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="K2" s="9" t="s">
         <v>64</v>
@@ -1346,7 +1373,7 @@
       </c>
       <c r="M2" s="5"/>
       <c r="N2" s="5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O2" s="5" t="s">
         <v>66</v>
@@ -1376,10 +1403,10 @@
       </c>
       <c r="H3" s="5"/>
       <c r="I3" s="8">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="K3" s="9" t="s">
         <v>68</v>
@@ -1389,7 +1416,7 @@
       </c>
       <c r="M3" s="5"/>
       <c r="N3" s="5">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O3" s="5"/>
     </row>
@@ -1420,17 +1447,17 @@
         <v>15</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>160</v>
+        <v>181</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>161</v>
+        <v>186</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>70</v>
+        <v>185</v>
       </c>
       <c r="M4" s="5"/>
       <c r="N4" s="5">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="O4" s="5"/>
     </row>
@@ -1461,17 +1488,17 @@
         <v>15</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>163</v>
+        <v>152</v>
       </c>
       <c r="L5" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="M5" s="5"/>
       <c r="N5" s="5">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="O5" s="5"/>
     </row>
@@ -1502,22 +1529,21 @@
         <v>15</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>72</v>
+        <v>153</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="L6" s="9" t="str">
-        <f>B6&amp;": "&amp;K6</f>
-        <v>Welcomer: …educate you on the LORE. I will trade you for one!</v>
+        <v>154</v>
+      </c>
+      <c r="L6" s="9" t="s">
+        <v>71</v>
       </c>
       <c r="M6" s="5"/>
       <c r="N6" s="5">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="O6" s="5"/>
     </row>
-    <row r="7" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>58</v>
       </c>
@@ -1536,35 +1562,29 @@
       <c r="F7" s="5">
         <v>-1</v>
       </c>
-      <c r="G7" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="I7" s="7">
-        <v>15</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="L7" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="M7" s="5">
-        <v>1</v>
-      </c>
+      <c r="G7" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="H7" s="5"/>
+      <c r="I7" s="8">
+        <v>10</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="K7" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="L7" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="M7" s="5"/>
       <c r="N7" s="5">
         <v>5</v>
       </c>
-      <c r="O7" s="5" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="O7" s="5"/>
+    </row>
+    <row r="8" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>58</v>
       </c>
@@ -1584,28 +1604,32 @@
         <v>-1</v>
       </c>
       <c r="G8" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="H8" s="7" t="s">
         <v>73</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>78</v>
       </c>
       <c r="I8" s="7">
         <v>15</v>
       </c>
       <c r="J8" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="L8" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="K8" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="L8" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="M8" s="5"/>
+      <c r="M8" s="5">
+        <v>1</v>
+      </c>
       <c r="N8" s="5">
-        <v>-5</v>
-      </c>
-      <c r="O8" s="5"/>
+        <v>5</v>
+      </c>
+      <c r="O8" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="9" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
@@ -1618,35 +1642,37 @@
         <v>60</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="F9" s="5">
         <v>-1</v>
       </c>
-      <c r="G9" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
+      <c r="G9" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="I9" s="7">
+        <v>15</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>74</v>
+      </c>
       <c r="K9" s="5" t="s">
-        <v>83</v>
+        <v>148</v>
       </c>
       <c r="L9" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="M9" s="5">
-        <v>10</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="M9" s="5"/>
       <c r="N9" s="5">
-        <v>4</v>
-      </c>
-      <c r="O9" s="5" t="s">
-        <v>85</v>
-      </c>
+        <v>-50</v>
+      </c>
+      <c r="O9" s="5"/>
     </row>
     <row r="10" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
@@ -1659,36 +1685,34 @@
         <v>60</v>
       </c>
       <c r="D10" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>80</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>86</v>
       </c>
       <c r="F10" s="5">
         <v>-1</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
-      <c r="J10" s="5" t="s">
-        <v>87</v>
-      </c>
+      <c r="J10" s="5"/>
       <c r="K10" s="5" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="L10" s="5" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="M10" s="5">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="N10" s="5">
         <v>4</v>
       </c>
       <c r="O10" s="5" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
@@ -1696,122 +1720,124 @@
         <v>58</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>91</v>
+        <v>59</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>102</v>
+        <v>85</v>
       </c>
       <c r="F11" s="5">
         <v>-1</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
       <c r="J11" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="L11" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="M11" s="5">
+        <v>1</v>
+      </c>
+      <c r="N11" s="5">
+        <v>4</v>
+      </c>
+      <c r="O11" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A12" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="F12" s="5">
+        <v>-1</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="K12" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="K11" s="5" t="s">
+      <c r="L12" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="M12" s="5"/>
+      <c r="N12" s="5">
+        <v>5</v>
+      </c>
+      <c r="O12" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="L11" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5">
-        <v>5</v>
-      </c>
-      <c r="O11" s="5" t="s">
+    </row>
+    <row r="13" spans="1:15" s="10" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" s="10" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="B12" s="7" t="s">
+      <c r="C13" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="D13" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E13" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="D12" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="E12" s="7" t="s">
+      <c r="F13" s="7">
+        <v>-1</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="K13" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="M13" s="7"/>
+      <c r="N13" s="7">
+        <v>20</v>
+      </c>
+      <c r="O13" s="7" t="s">
         <v>98</v>
-      </c>
-      <c r="F12" s="7">
-        <v>-1</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
-      <c r="J12" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="K12" s="7" t="s">
-        <v>168</v>
-      </c>
-      <c r="L12" s="7" t="s">
-        <v>167</v>
-      </c>
-      <c r="M12" s="7"/>
-      <c r="N12" s="7">
-        <v>20</v>
-      </c>
-      <c r="O12" s="7" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="F13" s="5">
-        <v>-1</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="K13" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="L13" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5">
-        <v>5</v>
-      </c>
-      <c r="O13" s="5" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
@@ -1819,249 +1845,249 @@
         <v>58</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F14" s="5">
         <v>-1</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
       <c r="J14" s="5" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="L14" s="7" t="s">
-        <v>165</v>
+        <v>103</v>
+      </c>
+      <c r="L14" s="5" t="s">
+        <v>104</v>
       </c>
       <c r="M14" s="5"/>
       <c r="N14" s="5">
         <v>5</v>
       </c>
       <c r="O14" s="5" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>58</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="F15" s="5">
         <v>-1</v>
       </c>
-      <c r="G15" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="I15" s="7"/>
-      <c r="J15" s="7" t="s">
-        <v>75</v>
+      <c r="G15" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="H15" s="5"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5" t="s">
+        <v>107</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="L15" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="M15" s="5">
-        <v>5</v>
-      </c>
+        <v>108</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="M15" s="5"/>
       <c r="N15" s="5">
         <v>5</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>58</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F16" s="5">
         <v>-1</v>
       </c>
       <c r="G16" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="H16" s="7" t="s">
         <v>73</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>78</v>
       </c>
       <c r="I16" s="7"/>
       <c r="J16" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K16" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="L16" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="L16" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="M16" s="5"/>
+      <c r="M16" s="5">
+        <v>5</v>
+      </c>
       <c r="N16" s="5">
-        <v>-5</v>
-      </c>
-      <c r="O16" s="5"/>
-    </row>
-    <row r="17" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+      <c r="O16" s="5" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>58</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>117</v>
+        <v>91</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="F17" s="5">
         <v>-1</v>
       </c>
-      <c r="G17" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5" t="s">
-        <v>118</v>
+      <c r="G17" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7" t="s">
+        <v>74</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L17" s="5" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="M17" s="5"/>
       <c r="N17" s="5">
-        <v>5</v>
-      </c>
-      <c r="O17" s="5" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+        <v>-5</v>
+      </c>
+      <c r="O17" s="5"/>
+    </row>
+    <row r="18" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>58</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F18" s="5">
         <v>-1</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H18" s="5"/>
       <c r="I18" s="5"/>
       <c r="J18" s="5" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="L18" s="5" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="M18" s="5"/>
       <c r="N18" s="5">
         <v>5</v>
       </c>
       <c r="O18" s="5" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>58</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F19" s="5">
         <v>-1</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H19" s="5"/>
       <c r="I19" s="5"/>
-      <c r="J19" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K19" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="L19" s="7" t="s">
-        <v>172</v>
+      <c r="J19" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="L19" s="5" t="s">
+        <v>124</v>
       </c>
       <c r="M19" s="5"/>
       <c r="N19" s="5">
         <v>5</v>
       </c>
       <c r="O19" s="5" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
     </row>
     <row r="20" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
@@ -2069,40 +2095,40 @@
         <v>58</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F20" s="5">
         <v>-1</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
       <c r="J20" s="7" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="M20" s="5"/>
       <c r="N20" s="5">
         <v>5</v>
       </c>
       <c r="O20" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="21" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
@@ -2110,415 +2136,482 @@
         <v>58</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F21" s="5">
         <v>-1</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H21" s="5"/>
       <c r="I21" s="5"/>
-      <c r="J21" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="K21" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="L21" s="5" t="s">
-        <v>134</v>
+      <c r="J21" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="K21" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="L21" s="7" t="s">
+        <v>163</v>
       </c>
       <c r="M21" s="5"/>
       <c r="N21" s="5">
         <v>5</v>
       </c>
-      <c r="O21" s="5"/>
+      <c r="O21" s="5" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="22" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>58</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="F22" s="5">
         <v>-1</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H22" s="5"/>
       <c r="I22" s="5"/>
       <c r="J22" s="5" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="L22" s="5" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="M22" s="5"/>
       <c r="N22" s="5">
         <v>5</v>
       </c>
-      <c r="O22" s="5" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="O22" s="5"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>58</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D23" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E23" s="5" t="s">
         <v>80</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>98</v>
       </c>
       <c r="F23" s="5">
         <v>-1</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H23" s="5"/>
       <c r="I23" s="5"/>
       <c r="J23" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="L23" s="5" t="s">
         <v>143</v>
+      </c>
+      <c r="L23" s="5" t="str">
+        <f>B23&amp;": "&amp;K23</f>
+        <v>Winston A.: The mantra is in Iolo's poem.</v>
       </c>
       <c r="M23" s="5"/>
       <c r="N23" s="5">
         <v>5</v>
       </c>
-      <c r="O23" s="5" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="O23" s="5"/>
+    </row>
+    <row r="24" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>58</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="F24" s="5">
         <v>-1</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
       <c r="J24" s="5" t="s">
-        <v>136</v>
+        <v>178</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="L24" s="5" t="s">
-        <v>148</v>
+        <v>177</v>
+      </c>
+      <c r="L24" s="5" t="str">
+        <f>B24&amp;": "&amp;K24</f>
+        <v>Winston A.: You can see that iron ingots aren't so easy to make, eh?</v>
       </c>
       <c r="M24" s="5"/>
       <c r="N24" s="5">
         <v>5</v>
       </c>
-      <c r="O24" s="5" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="O24" s="5"/>
+    </row>
+    <row r="25" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>58</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>150</v>
+        <v>139</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>98</v>
+        <v>179</v>
       </c>
       <c r="F25" s="5">
         <v>-1</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H25" s="5"/>
       <c r="I25" s="5"/>
       <c r="J25" s="5" t="s">
-        <v>136</v>
+        <v>176</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="L25" s="5" t="s">
-        <v>152</v>
+        <v>180</v>
+      </c>
+      <c r="L25" s="5" t="str">
+        <f>B25&amp;": "&amp;K25</f>
+        <v>Winston A.: Until you KNOW iron, you're not fit to hold ingots!</v>
       </c>
       <c r="M25" s="5"/>
       <c r="N25" s="5">
         <v>5</v>
       </c>
-      <c r="O25" s="5" t="s">
-        <v>144</v>
-      </c>
+      <c r="O25" s="5"/>
     </row>
     <row r="26" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>58</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F26" s="5">
         <v>-1</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
       <c r="J26" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="L26" s="5" t="s">
-        <v>156</v>
+        <v>140</v>
+      </c>
+      <c r="L26" s="5" t="str">
+        <f>B26&amp;": "&amp;K26</f>
+        <v>Winston T.: Shalimar and Cricket say the mantra.</v>
       </c>
       <c r="M26" s="5"/>
       <c r="N26" s="5">
         <v>5</v>
       </c>
-      <c r="O26" s="5" t="s">
+      <c r="O26" s="5"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A27" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B27" s="5" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="27" spans="1:15" s="12" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A27" s="8" t="s">
+      <c r="C27" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="F27" s="5">
+        <v>-1</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="H27" s="5"/>
+      <c r="I27" s="5"/>
+      <c r="J27" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="K27" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="L27" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="M27" s="5"/>
+      <c r="N27" s="5">
+        <v>5</v>
+      </c>
+      <c r="O27" s="5"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A28" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="D27" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="E27" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="F27" s="8">
+      <c r="B28" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="F28" s="5">
         <v>-1</v>
       </c>
-      <c r="G27" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="H27" s="8"/>
-      <c r="I27" s="8"/>
-      <c r="J27" s="8" t="s">
+      <c r="G28" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="H28" s="5"/>
+      <c r="I28" s="5"/>
+      <c r="J28" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="K28" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="L28" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="K27" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="L27" s="8" t="s">
-        <v>177</v>
-      </c>
-      <c r="M27" s="8"/>
-      <c r="N27" s="8">
+      <c r="M28" s="5"/>
+      <c r="N28" s="5">
         <v>5</v>
       </c>
-      <c r="O27" s="8" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" s="10" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B28" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="C28" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="D28" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="F28" s="13">
-        <v>-1</v>
-      </c>
-      <c r="G28" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="H28" s="11"/>
-      <c r="I28" s="11"/>
-      <c r="J28" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="K28" s="11" t="s">
-        <v>180</v>
-      </c>
-      <c r="L28" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="M28" s="11"/>
-      <c r="N28" s="8">
-        <v>5</v>
-      </c>
-      <c r="O28" s="11"/>
+      <c r="O28" s="5"/>
     </row>
     <row r="29" spans="1:15" s="12" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="B29" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="D29" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="E29" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="F29" s="15">
+      <c r="B29" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="F29" s="8">
         <v>-1</v>
       </c>
-      <c r="G29" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="H29" s="9"/>
-      <c r="J29" s="9" t="s">
-        <v>178</v>
-      </c>
-      <c r="K29" s="12" t="s">
-        <v>137</v>
-      </c>
-      <c r="L29" s="12" t="s">
-        <v>137</v>
-      </c>
-      <c r="M29" s="9"/>
+      <c r="G29" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="H29" s="8"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="K29" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="L29" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="M29" s="8"/>
       <c r="N29" s="8">
         <v>5</v>
       </c>
-      <c r="O29" s="12" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A30" s="6"/>
-      <c r="B30" s="6"/>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="6"/>
-      <c r="F30" s="6"/>
-      <c r="G30" s="6"/>
-      <c r="H30" s="6"/>
-      <c r="I30" s="6"/>
-      <c r="J30" s="6"/>
-      <c r="K30" s="6"/>
-      <c r="L30" s="6"/>
-      <c r="M30" s="6"/>
-      <c r="N30" s="6"/>
-      <c r="O30" s="6"/>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A31" s="6"/>
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
-      <c r="G31" s="6"/>
-      <c r="H31" s="6"/>
-      <c r="I31" s="6"/>
-      <c r="J31" s="6"/>
-      <c r="K31" s="6"/>
-      <c r="L31" s="6"/>
-      <c r="M31" s="6"/>
-      <c r="N31" s="6"/>
-      <c r="O31" s="6"/>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A32" s="6"/>
-      <c r="B32" s="6"/>
-      <c r="C32" s="6"/>
-      <c r="D32" s="6"/>
-      <c r="E32" s="6"/>
-      <c r="F32" s="6"/>
-      <c r="G32" s="6"/>
-      <c r="H32" s="6"/>
-      <c r="I32" s="6"/>
-      <c r="J32" s="6"/>
-      <c r="K32" s="6"/>
-      <c r="L32" s="6"/>
+      <c r="O29" s="8" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="F30" s="13">
+        <v>3</v>
+      </c>
+      <c r="G30" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="H30" s="11"/>
+      <c r="I30" s="11"/>
+      <c r="J30" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="K30" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="L30" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="M30" s="11"/>
+      <c r="N30" s="8">
+        <v>5</v>
+      </c>
+      <c r="O30" s="12" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" s="12" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A31" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="F31" s="15">
+        <v>-1</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H31" s="9"/>
+      <c r="J31" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="K31" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="L31" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="M31" s="9"/>
+      <c r="N31" s="8">
+        <v>5</v>
+      </c>
+      <c r="O31" s="12" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A32" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="F32" s="7">
+        <v>3</v>
+      </c>
+      <c r="G32" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="H32" s="7"/>
+      <c r="I32" s="7"/>
+      <c r="J32" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="K32" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="L32" s="7" t="str">
+        <f>B32&amp;": "&amp;K32</f>
+        <v>Winston M.: I can teach you how to mine cobblestones!</v>
+      </c>
       <c r="M32" s="6"/>
-      <c r="N32" s="6"/>
-      <c r="O32" s="6"/>
+      <c r="N32" s="5">
+        <v>10</v>
+      </c>
+      <c r="O32" s="5" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33" s="6"/>
@@ -2531,7 +2624,7 @@
       <c r="H33" s="6"/>
       <c r="I33" s="6"/>
       <c r="J33" s="6"/>
-      <c r="K33" s="6"/>
+      <c r="K33" s="5"/>
       <c r="L33" s="6"/>
       <c r="M33" s="6"/>
       <c r="N33" s="6"/>
@@ -8776,16 +8869,50 @@
       <c r="N400" s="6"/>
       <c r="O400" s="6"/>
     </row>
+    <row r="401" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A401" s="6"/>
+      <c r="B401" s="6"/>
+      <c r="C401" s="6"/>
+      <c r="D401" s="6"/>
+      <c r="E401" s="6"/>
+      <c r="F401" s="6"/>
+      <c r="G401" s="6"/>
+      <c r="H401" s="6"/>
+      <c r="I401" s="6"/>
+      <c r="J401" s="6"/>
+      <c r="K401" s="6"/>
+      <c r="L401" s="6"/>
+      <c r="M401" s="6"/>
+      <c r="N401" s="6"/>
+      <c r="O401" s="6"/>
+    </row>
+    <row r="402" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A402" s="6"/>
+      <c r="B402" s="6"/>
+      <c r="C402" s="6"/>
+      <c r="D402" s="6"/>
+      <c r="E402" s="6"/>
+      <c r="F402" s="6"/>
+      <c r="G402" s="6"/>
+      <c r="H402" s="6"/>
+      <c r="I402" s="6"/>
+      <c r="J402" s="6"/>
+      <c r="K402" s="6"/>
+      <c r="L402" s="6"/>
+      <c r="M402" s="6"/>
+      <c r="N402" s="6"/>
+      <c r="O402" s="6"/>
+    </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" sqref="D2:D400" xr:uid="{00000000-0002-0000-0100-000000000000}">
-      <formula1>"Proximity,Trade-completion,Level-reached"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="G30:G400 G2:G27" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="G2:G29 G32:G402" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Statement,Question,Statement-Roll"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="G28:G29" xr:uid="{978F0CFC-32AF-4B55-9CBC-7DF8E8F9C2A9}">
+    <dataValidation type="list" allowBlank="1" sqref="G30:G31" xr:uid="{978F0CFC-32AF-4B55-9CBC-7DF8E8F9C2A9}">
       <formula1>"Statement,Question-YN,Question-MultiChoice"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="D2:D402" xr:uid="{00000000-0002-0000-0100-000000000000}">
+      <formula1>"Proximity,Trade-completion,Level-reached"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mining Mastery (both loot drops for different pickaxe types) and Mining advcmt tab - tested OK
</commit_message>
<xml_diff>
--- a/spoilers/conversations.xlsx
+++ b/spoilers/conversations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MYDATA\_GIT_REPOS\mcu4\spoilers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9CECD17-485C-455B-9951-B8304764D94E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63A9CDAB-F85F-4A87-8F7C-D4407FEFD149}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="11964" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="189">
   <si>
     <t>Game-Level Conversation List</t>
   </si>
@@ -275,9 +275,6 @@
     <t>Welcomer: "Much obliged."</t>
   </si>
   <si>
-    <t>Blocked — trade-completion predicate not yet confirmed working, not built.</t>
-  </si>
-  <si>
     <t>L2 Trade</t>
   </si>
   <si>
@@ -288,9 +285,6 @@
   </si>
   <si>
     <t>Welcomer: This potion will teleport you back to our portal!</t>
-  </si>
-  <si>
-    <t>Blocked — same reason as above.</t>
   </si>
   <si>
     <t>Shapero</t>
@@ -1363,7 +1357,7 @@
         <v>15</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="K2" s="9" t="s">
         <v>64</v>
@@ -1406,7 +1400,7 @@
         <v>15</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="K3" s="9" t="s">
         <v>68</v>
@@ -1447,13 +1441,13 @@
         <v>15</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="M4" s="5"/>
       <c r="N4" s="5">
@@ -1488,10 +1482,10 @@
         <v>15</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="L5" s="9" t="s">
         <v>70</v>
@@ -1529,10 +1523,10 @@
         <v>15</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="L6" s="9" t="s">
         <v>71</v>
@@ -1570,13 +1564,13 @@
         <v>10</v>
       </c>
       <c r="J7" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="K7" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="K7" s="9" t="s">
-        <v>184</v>
-      </c>
       <c r="L7" s="9" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="M7" s="5"/>
       <c r="N7" s="5">
@@ -1616,7 +1610,7 @@
         <v>74</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="L8" s="5" t="s">
         <v>75</v>
@@ -1663,7 +1657,7 @@
         <v>74</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="L9" s="5" t="s">
         <v>78</v>
@@ -1674,7 +1668,7 @@
       </c>
       <c r="O9" s="5"/>
     </row>
-    <row r="10" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>58</v>
       </c>
@@ -1711,9 +1705,7 @@
       <c r="N10" s="5">
         <v>4</v>
       </c>
-      <c r="O10" s="5" t="s">
-        <v>84</v>
-      </c>
+      <c r="O10" s="5"/>
     </row>
     <row r="11" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
@@ -1729,7 +1721,7 @@
         <v>79</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F11" s="5">
         <v>-1</v>
@@ -1740,13 +1732,13 @@
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
       <c r="J11" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="K11" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="K11" s="5" t="s">
+      <c r="L11" s="5" t="s">
         <v>87</v>
-      </c>
-      <c r="L11" s="5" t="s">
-        <v>88</v>
       </c>
       <c r="M11" s="5">
         <v>1</v>
@@ -1754,25 +1746,23 @@
       <c r="N11" s="5">
         <v>4</v>
       </c>
-      <c r="O11" s="5" t="s">
-        <v>89</v>
-      </c>
+      <c r="O11" s="5"/>
     </row>
     <row r="12" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>58</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F12" s="5">
         <v>-1</v>
@@ -1783,20 +1773,20 @@
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
       <c r="J12" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="L12" s="5" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="M12" s="5"/>
       <c r="N12" s="5">
         <v>5</v>
       </c>
       <c r="O12" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:15" s="10" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
@@ -1804,16 +1794,16 @@
         <v>58</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>79</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F13" s="7">
         <v>-1</v>
@@ -1827,17 +1817,17 @@
         <v>67</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="M13" s="7"/>
       <c r="N13" s="7">
         <v>20</v>
       </c>
       <c r="O13" s="7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
@@ -1845,16 +1835,16 @@
         <v>58</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F14" s="5">
         <v>-1</v>
@@ -1865,20 +1855,20 @@
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
       <c r="J14" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="L14" s="5" t="s">
         <v>102</v>
-      </c>
-      <c r="K14" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="L14" s="5" t="s">
-        <v>104</v>
       </c>
       <c r="M14" s="5"/>
       <c r="N14" s="5">
         <v>5</v>
       </c>
       <c r="O14" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="15" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
@@ -1886,16 +1876,16 @@
         <v>58</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F15" s="5">
         <v>-1</v>
@@ -1906,20 +1896,20 @@
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
       <c r="J15" s="5" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="M15" s="5"/>
       <c r="N15" s="5">
         <v>5</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="16" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
@@ -1927,16 +1917,16 @@
         <v>58</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>79</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F16" s="5">
         <v>-1</v>
@@ -1952,10 +1942,10 @@
         <v>74</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="L16" s="5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="M16" s="5">
         <v>5</v>
@@ -1964,7 +1954,7 @@
         <v>5</v>
       </c>
       <c r="O16" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
@@ -1972,16 +1962,16 @@
         <v>58</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>79</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F17" s="5">
         <v>-1</v>
@@ -1997,10 +1987,10 @@
         <v>74</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="L17" s="5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="M17" s="5"/>
       <c r="N17" s="5">
@@ -2013,16 +2003,16 @@
         <v>58</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F18" s="5">
         <v>-1</v>
@@ -2033,20 +2023,20 @@
       <c r="H18" s="5"/>
       <c r="I18" s="5"/>
       <c r="J18" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="K18" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="L18" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="K18" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="L18" s="5" t="s">
-        <v>119</v>
       </c>
       <c r="M18" s="5"/>
       <c r="N18" s="5">
         <v>5</v>
       </c>
       <c r="O18" s="5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
@@ -2054,16 +2044,16 @@
         <v>58</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F19" s="5">
         <v>-1</v>
@@ -2074,20 +2064,20 @@
       <c r="H19" s="5"/>
       <c r="I19" s="5"/>
       <c r="J19" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="L19" s="5" t="s">
         <v>122</v>
-      </c>
-      <c r="K19" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="L19" s="5" t="s">
-        <v>124</v>
       </c>
       <c r="M19" s="5"/>
       <c r="N19" s="5">
         <v>5</v>
       </c>
       <c r="O19" s="5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
@@ -2095,16 +2085,16 @@
         <v>58</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F20" s="5">
         <v>-1</v>
@@ -2115,20 +2105,20 @@
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
       <c r="J20" s="7" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="M20" s="5"/>
       <c r="N20" s="5">
         <v>5</v>
       </c>
       <c r="O20" s="5" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="21" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
@@ -2136,16 +2126,16 @@
         <v>58</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F21" s="5">
         <v>-1</v>
@@ -2156,20 +2146,20 @@
       <c r="H21" s="5"/>
       <c r="I21" s="5"/>
       <c r="J21" s="7" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K21" s="7" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="L21" s="7" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="M21" s="5"/>
       <c r="N21" s="5">
         <v>5</v>
       </c>
       <c r="O21" s="5" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="22" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
@@ -2177,16 +2167,16 @@
         <v>58</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F22" s="5">
         <v>-1</v>
@@ -2197,13 +2187,13 @@
       <c r="H22" s="5"/>
       <c r="I22" s="5"/>
       <c r="J22" s="5" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="L22" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="M22" s="5"/>
       <c r="N22" s="5">
@@ -2216,10 +2206,10 @@
         <v>58</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>79</v>
@@ -2236,10 +2226,10 @@
       <c r="H23" s="5"/>
       <c r="I23" s="5"/>
       <c r="J23" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="L23" s="5" t="str">
         <f>B23&amp;": "&amp;K23</f>
@@ -2256,16 +2246,16 @@
         <v>58</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>79</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F24" s="5">
         <v>-1</v>
@@ -2276,10 +2266,10 @@
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
       <c r="J24" s="5" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="L24" s="5" t="str">
         <f>B24&amp;": "&amp;K24</f>
@@ -2296,16 +2286,16 @@
         <v>58</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>79</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F25" s="5">
         <v>-1</v>
@@ -2316,10 +2306,10 @@
       <c r="H25" s="5"/>
       <c r="I25" s="5"/>
       <c r="J25" s="5" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="L25" s="5" t="str">
         <f>B25&amp;": "&amp;K25</f>
@@ -2336,16 +2326,16 @@
         <v>58</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>79</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F26" s="5">
         <v>-1</v>
@@ -2356,10 +2346,10 @@
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
       <c r="J26" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="L26" s="5" t="str">
         <f>B26&amp;": "&amp;K26</f>
@@ -2376,16 +2366,16 @@
         <v>58</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>79</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F27" s="5">
         <v>-1</v>
@@ -2396,13 +2386,13 @@
       <c r="H27" s="5"/>
       <c r="I27" s="5"/>
       <c r="J27" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="L27" s="5" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="M27" s="5"/>
       <c r="N27" s="5">
@@ -2415,16 +2405,16 @@
         <v>58</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>79</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F28" s="5">
         <v>-1</v>
@@ -2435,13 +2425,13 @@
       <c r="H28" s="5"/>
       <c r="I28" s="5"/>
       <c r="J28" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="L28" s="5" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="M28" s="5"/>
       <c r="N28" s="5">
@@ -2454,16 +2444,16 @@
         <v>58</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D29" s="8" t="s">
         <v>61</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="F29" s="8">
         <v>-1</v>
@@ -2474,20 +2464,20 @@
       <c r="H29" s="8"/>
       <c r="I29" s="8"/>
       <c r="J29" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="K29" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="L29" s="8" t="s">
         <v>165</v>
-      </c>
-      <c r="K29" s="8" t="s">
-        <v>166</v>
-      </c>
-      <c r="L29" s="8" t="s">
-        <v>167</v>
       </c>
       <c r="M29" s="8"/>
       <c r="N29" s="8">
         <v>5</v>
       </c>
       <c r="O29" s="8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="30" spans="1:15" s="10" customFormat="1" x14ac:dyDescent="0.3">
@@ -2495,16 +2485,16 @@
         <v>58</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D30" s="8" t="s">
         <v>61</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="F30" s="13">
         <v>3</v>
@@ -2515,20 +2505,20 @@
       <c r="H30" s="11"/>
       <c r="I30" s="11"/>
       <c r="J30" s="11" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="K30" s="11" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="L30" s="11" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="M30" s="11"/>
       <c r="N30" s="8">
         <v>5</v>
       </c>
       <c r="O30" s="12" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="31" spans="1:15" s="12" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
@@ -2536,16 +2526,16 @@
         <v>58</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D31" s="14" t="s">
         <v>79</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F31" s="15">
         <v>-1</v>
@@ -2555,20 +2545,20 @@
       </c>
       <c r="H31" s="9"/>
       <c r="J31" s="9" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="K31" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="L31" s="7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="M31" s="9"/>
       <c r="N31" s="8">
         <v>5</v>
       </c>
       <c r="O31" s="12" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="32" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
@@ -2576,16 +2566,16 @@
         <v>58</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D32" s="7" t="s">
         <v>61</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="F32" s="7">
         <v>3</v>
@@ -2596,10 +2586,10 @@
       <c r="H32" s="7"/>
       <c r="I32" s="7"/>
       <c r="J32" s="7" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="K32" s="7" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="L32" s="7" t="str">
         <f>B32&amp;": "&amp;K32</f>
@@ -2610,7 +2600,7 @@
         <v>10</v>
       </c>
       <c r="O32" s="5" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Tested conversational L1 and L2 trades with Welcomer and potion related chatter to be consistent with Celest.
</commit_message>
<xml_diff>
--- a/spoilers/conversations.xlsx
+++ b/spoilers/conversations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MYDATA\_GIT_REPOS\mcu4\spoilers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63A9CDAB-F85F-4A87-8F7C-D4407FEFD149}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18B8D48C-9BE8-40C0-81E9-CEE35A79F3BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="11964" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -278,15 +278,6 @@
     <t>L2 Trade</t>
   </si>
   <si>
-    <t>About this Potion...</t>
-  </si>
-  <si>
-    <t>This potion will teleport you back to our portal!</t>
-  </si>
-  <si>
-    <t>Welcomer: This potion will teleport you back to our portal!</t>
-  </si>
-  <si>
     <t>Shapero</t>
   </si>
   <si>
@@ -588,6 +579,15 @@
   </si>
   <si>
     <t>I can teach you how to mine cobblestones!</t>
+  </si>
+  <si>
+    <t>About this bottle…</t>
+  </si>
+  <si>
+    <t>Fill it with water and trade with Celest!</t>
+  </si>
+  <si>
+    <t>Welcomer: Fill it with water and trade with Celest!</t>
   </si>
 </sst>
 </file>
@@ -1357,7 +1357,7 @@
         <v>15</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="K2" s="9" t="s">
         <v>64</v>
@@ -1400,7 +1400,7 @@
         <v>15</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="K3" s="9" t="s">
         <v>68</v>
@@ -1441,13 +1441,13 @@
         <v>15</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="M4" s="5"/>
       <c r="N4" s="5">
@@ -1482,10 +1482,10 @@
         <v>15</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="L5" s="9" t="s">
         <v>70</v>
@@ -1523,10 +1523,10 @@
         <v>15</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="L6" s="9" t="s">
         <v>71</v>
@@ -1564,13 +1564,13 @@
         <v>10</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="L7" s="9" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="M7" s="5"/>
       <c r="N7" s="5">
@@ -1610,7 +1610,7 @@
         <v>74</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="L8" s="5" t="s">
         <v>75</v>
@@ -1657,7 +1657,7 @@
         <v>74</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="L9" s="5" t="s">
         <v>78</v>
@@ -1732,13 +1732,13 @@
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
       <c r="J11" s="5" t="s">
-        <v>85</v>
+        <v>186</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>86</v>
+        <v>187</v>
       </c>
       <c r="L11" s="5" t="s">
-        <v>87</v>
+        <v>188</v>
       </c>
       <c r="M11" s="5">
         <v>1</v>
@@ -1753,16 +1753,16 @@
         <v>58</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F12" s="5">
         <v>-1</v>
@@ -1773,20 +1773,20 @@
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
       <c r="J12" s="5" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="L12" s="5" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="M12" s="5"/>
       <c r="N12" s="5">
         <v>5</v>
       </c>
       <c r="O12" s="5" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="1:15" s="10" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
@@ -1794,16 +1794,16 @@
         <v>58</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>79</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="F13" s="7">
         <v>-1</v>
@@ -1817,17 +1817,17 @@
         <v>67</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="M13" s="7"/>
       <c r="N13" s="7">
         <v>20</v>
       </c>
       <c r="O13" s="7" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
@@ -1835,16 +1835,16 @@
         <v>58</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F14" s="5">
         <v>-1</v>
@@ -1855,20 +1855,20 @@
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
       <c r="J14" s="5" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="L14" s="5" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="M14" s="5"/>
       <c r="N14" s="5">
         <v>5</v>
       </c>
       <c r="O14" s="5" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
@@ -1876,16 +1876,16 @@
         <v>58</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F15" s="5">
         <v>-1</v>
@@ -1896,20 +1896,20 @@
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
       <c r="J15" s="5" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="M15" s="5"/>
       <c r="N15" s="5">
         <v>5</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
@@ -1917,16 +1917,16 @@
         <v>58</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>79</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="F16" s="5">
         <v>-1</v>
@@ -1942,10 +1942,10 @@
         <v>74</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="L16" s="5" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="M16" s="5">
         <v>5</v>
@@ -1954,7 +1954,7 @@
         <v>5</v>
       </c>
       <c r="O16" s="5" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
@@ -1962,16 +1962,16 @@
         <v>58</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>79</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="F17" s="5">
         <v>-1</v>
@@ -1987,10 +1987,10 @@
         <v>74</v>
       </c>
       <c r="K17" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="L17" s="5" t="s">
         <v>109</v>
-      </c>
-      <c r="L17" s="5" t="s">
-        <v>112</v>
       </c>
       <c r="M17" s="5"/>
       <c r="N17" s="5">
@@ -2003,16 +2003,16 @@
         <v>58</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F18" s="5">
         <v>-1</v>
@@ -2023,20 +2023,20 @@
       <c r="H18" s="5"/>
       <c r="I18" s="5"/>
       <c r="J18" s="5" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="L18" s="5" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="M18" s="5"/>
       <c r="N18" s="5">
         <v>5</v>
       </c>
       <c r="O18" s="5" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
@@ -2044,16 +2044,16 @@
         <v>58</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F19" s="5">
         <v>-1</v>
@@ -2064,20 +2064,20 @@
       <c r="H19" s="5"/>
       <c r="I19" s="5"/>
       <c r="J19" s="5" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="L19" s="5" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="M19" s="5"/>
       <c r="N19" s="5">
         <v>5</v>
       </c>
       <c r="O19" s="5" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="20" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
@@ -2085,16 +2085,16 @@
         <v>58</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F20" s="5">
         <v>-1</v>
@@ -2105,20 +2105,20 @@
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
       <c r="J20" s="7" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="M20" s="5"/>
       <c r="N20" s="5">
         <v>5</v>
       </c>
       <c r="O20" s="5" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="21" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
@@ -2126,16 +2126,16 @@
         <v>58</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F21" s="5">
         <v>-1</v>
@@ -2146,20 +2146,20 @@
       <c r="H21" s="5"/>
       <c r="I21" s="5"/>
       <c r="J21" s="7" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="K21" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="L21" s="7" t="s">
         <v>158</v>
-      </c>
-      <c r="L21" s="7" t="s">
-        <v>161</v>
       </c>
       <c r="M21" s="5"/>
       <c r="N21" s="5">
         <v>5</v>
       </c>
       <c r="O21" s="5" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="22" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
@@ -2167,16 +2167,16 @@
         <v>58</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F22" s="5">
         <v>-1</v>
@@ -2187,13 +2187,13 @@
       <c r="H22" s="5"/>
       <c r="I22" s="5"/>
       <c r="J22" s="5" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="L22" s="5" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="M22" s="5"/>
       <c r="N22" s="5">
@@ -2206,10 +2206,10 @@
         <v>58</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>79</v>
@@ -2226,10 +2226,10 @@
       <c r="H23" s="5"/>
       <c r="I23" s="5"/>
       <c r="J23" s="5" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="L23" s="5" t="str">
         <f>B23&amp;": "&amp;K23</f>
@@ -2246,10 +2246,10 @@
         <v>58</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>79</v>
@@ -2266,10 +2266,10 @@
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
       <c r="J24" s="5" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="L24" s="5" t="str">
         <f>B24&amp;": "&amp;K24</f>
@@ -2286,16 +2286,16 @@
         <v>58</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>79</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="F25" s="5">
         <v>-1</v>
@@ -2306,10 +2306,10 @@
       <c r="H25" s="5"/>
       <c r="I25" s="5"/>
       <c r="J25" s="5" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="L25" s="5" t="str">
         <f>B25&amp;": "&amp;K25</f>
@@ -2326,16 +2326,16 @@
         <v>58</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>79</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="F26" s="5">
         <v>-1</v>
@@ -2346,10 +2346,10 @@
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
       <c r="J26" s="5" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="L26" s="5" t="str">
         <f>B26&amp;": "&amp;K26</f>
@@ -2366,16 +2366,16 @@
         <v>58</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>79</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="F27" s="5">
         <v>-1</v>
@@ -2386,13 +2386,13 @@
       <c r="H27" s="5"/>
       <c r="I27" s="5"/>
       <c r="J27" s="5" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="L27" s="5" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="M27" s="5"/>
       <c r="N27" s="5">
@@ -2405,16 +2405,16 @@
         <v>58</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>79</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="F28" s="5">
         <v>-1</v>
@@ -2425,13 +2425,13 @@
       <c r="H28" s="5"/>
       <c r="I28" s="5"/>
       <c r="J28" s="5" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="K28" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="L28" s="5" t="s">
         <v>170</v>
-      </c>
-      <c r="L28" s="5" t="s">
-        <v>173</v>
       </c>
       <c r="M28" s="5"/>
       <c r="N28" s="5">
@@ -2444,16 +2444,16 @@
         <v>58</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D29" s="8" t="s">
         <v>61</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="F29" s="8">
         <v>-1</v>
@@ -2464,20 +2464,20 @@
       <c r="H29" s="8"/>
       <c r="I29" s="8"/>
       <c r="J29" s="8" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="K29" s="8" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="L29" s="8" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="M29" s="8"/>
       <c r="N29" s="8">
         <v>5</v>
       </c>
       <c r="O29" s="8" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="30" spans="1:15" s="10" customFormat="1" x14ac:dyDescent="0.3">
@@ -2485,16 +2485,16 @@
         <v>58</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D30" s="8" t="s">
         <v>61</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="F30" s="13">
         <v>3</v>
@@ -2505,20 +2505,20 @@
       <c r="H30" s="11"/>
       <c r="I30" s="11"/>
       <c r="J30" s="11" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="K30" s="11" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="L30" s="11" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="M30" s="11"/>
       <c r="N30" s="8">
         <v>5</v>
       </c>
       <c r="O30" s="12" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="31" spans="1:15" s="12" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
@@ -2526,16 +2526,16 @@
         <v>58</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D31" s="14" t="s">
         <v>79</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="F31" s="15">
         <v>-1</v>
@@ -2545,20 +2545,20 @@
       </c>
       <c r="H31" s="9"/>
       <c r="J31" s="9" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="K31" s="12" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="L31" s="7" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="M31" s="9"/>
       <c r="N31" s="8">
         <v>5</v>
       </c>
       <c r="O31" s="12" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="32" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
@@ -2566,16 +2566,16 @@
         <v>58</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D32" s="7" t="s">
         <v>61</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="F32" s="7">
         <v>3</v>
@@ -2586,10 +2586,10 @@
       <c r="H32" s="7"/>
       <c r="I32" s="7"/>
       <c r="J32" s="7" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="K32" s="7" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="L32" s="7" t="str">
         <f>B32&amp;": "&amp;K32</f>
@@ -2600,7 +2600,7 @@
         <v>10</v>
       </c>
       <c r="O32" s="5" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Helmet function working. Added SWEN riddles to conversations xlsx
</commit_message>
<xml_diff>
--- a/spoilers/conversations.xlsx
+++ b/spoilers/conversations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MYDATA\_GIT_REPOS\mcu4\spoilers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18B8D48C-9BE8-40C0-81E9-CEE35A79F3BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{996C5A6C-AC91-428B-877C-4B5EB2B81D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="11964" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="204">
   <si>
     <t>Game-Level Conversation List</t>
   </si>
@@ -588,13 +588,58 @@
   </si>
   <si>
     <t>Welcomer: Fill it with water and trade with Celest!</t>
+  </si>
+  <si>
+    <t>Jhelom</t>
+  </si>
+  <si>
+    <t>Swen</t>
+  </si>
+  <si>
+    <t>I love Johnny Cash!</t>
+  </si>
+  <si>
+    <t>Hi, my name is SWEN!</t>
+  </si>
+  <si>
+    <t>It'll come in handy at least once, around here.</t>
+  </si>
+  <si>
+    <t>I love the Doors</t>
+  </si>
+  <si>
+    <t>Here's the end of my riddle</t>
+  </si>
+  <si>
+    <t>Here's the start of my riddle</t>
+  </si>
+  <si>
+    <t>A zillion keys but no matching door.</t>
+  </si>
+  <si>
+    <t>A zillion doors with no matching key...</t>
+  </si>
+  <si>
+    <t>Cuz I've been "everywhere", man...in Jhelom!</t>
+  </si>
+  <si>
+    <t>Not the band, but all the doors in Jhelom</t>
+  </si>
+  <si>
+    <t>I love all the doors in Jhelom</t>
+  </si>
+  <si>
+    <t>Riddle 2 there's a zillion keys with no matching door</t>
+  </si>
+  <si>
+    <t>Riddle 1 there's a zillion doors with no matching key</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -641,6 +686,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -690,7 +741,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -716,13 +767,25 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1272,7 +1335,7 @@
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="6" max="6" width="10" style="18" customWidth="1"/>
     <col min="7" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
     <col min="10" max="10" width="20" customWidth="1"/>
@@ -1299,7 +1362,7 @@
       <c r="E1" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="16" t="s">
         <v>48</v>
       </c>
       <c r="G1" s="4" t="s">
@@ -1346,7 +1409,7 @@
       <c r="E2" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="14">
         <v>-1</v>
       </c>
       <c r="G2" s="5" t="s">
@@ -1389,7 +1452,7 @@
       <c r="E3" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="14">
         <v>-1</v>
       </c>
       <c r="G3" s="5" t="s">
@@ -1430,7 +1493,7 @@
       <c r="E4" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="14">
         <v>-1</v>
       </c>
       <c r="G4" s="5" t="s">
@@ -1471,7 +1534,7 @@
       <c r="E5" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="14">
         <v>-1</v>
       </c>
       <c r="G5" s="5" t="s">
@@ -1512,7 +1575,7 @@
       <c r="E6" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="14">
         <v>-1</v>
       </c>
       <c r="G6" s="5" t="s">
@@ -1553,7 +1616,7 @@
       <c r="E7" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="14">
         <v>-1</v>
       </c>
       <c r="G7" s="5" t="s">
@@ -1594,7 +1657,7 @@
       <c r="E8" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="14">
         <v>-1</v>
       </c>
       <c r="G8" s="7" t="s">
@@ -1641,7 +1704,7 @@
       <c r="E9" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="14">
         <v>-1</v>
       </c>
       <c r="G9" s="7" t="s">
@@ -1684,7 +1747,7 @@
       <c r="E10" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="14">
         <v>-1</v>
       </c>
       <c r="G10" s="5" t="s">
@@ -1723,7 +1786,7 @@
       <c r="E11" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="F11" s="5">
+      <c r="F11" s="14">
         <v>-1</v>
       </c>
       <c r="G11" s="5" t="s">
@@ -1764,7 +1827,7 @@
       <c r="E12" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="F12" s="5">
+      <c r="F12" s="14">
         <v>-1</v>
       </c>
       <c r="G12" s="5" t="s">
@@ -1805,7 +1868,7 @@
       <c r="E13" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="F13" s="7">
+      <c r="F13" s="14">
         <v>-1</v>
       </c>
       <c r="G13" s="7" t="s">
@@ -1846,7 +1909,7 @@
       <c r="E14" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="14">
         <v>-1</v>
       </c>
       <c r="G14" s="5" t="s">
@@ -1887,7 +1950,7 @@
       <c r="E15" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="14">
         <v>-1</v>
       </c>
       <c r="G15" s="5" t="s">
@@ -1928,7 +1991,7 @@
       <c r="E16" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="F16" s="5">
+      <c r="F16" s="14">
         <v>-1</v>
       </c>
       <c r="G16" s="7" t="s">
@@ -1973,7 +2036,7 @@
       <c r="E17" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="F17" s="5">
+      <c r="F17" s="14">
         <v>-1</v>
       </c>
       <c r="G17" s="7" t="s">
@@ -2014,7 +2077,7 @@
       <c r="E18" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="F18" s="5">
+      <c r="F18" s="14">
         <v>-1</v>
       </c>
       <c r="G18" s="5" t="s">
@@ -2055,7 +2118,7 @@
       <c r="E19" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="F19" s="5">
+      <c r="F19" s="14">
         <v>-1</v>
       </c>
       <c r="G19" s="5" t="s">
@@ -2096,7 +2159,7 @@
       <c r="E20" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="F20" s="5">
+      <c r="F20" s="14">
         <v>-1</v>
       </c>
       <c r="G20" s="5" t="s">
@@ -2137,7 +2200,7 @@
       <c r="E21" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="F21" s="5">
+      <c r="F21" s="14">
         <v>-1</v>
       </c>
       <c r="G21" s="5" t="s">
@@ -2178,7 +2241,7 @@
       <c r="E22" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="F22" s="5">
+      <c r="F22" s="14">
         <v>-1</v>
       </c>
       <c r="G22" s="5" t="s">
@@ -2217,7 +2280,7 @@
       <c r="E23" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="F23" s="5">
+      <c r="F23" s="14">
         <v>-1</v>
       </c>
       <c r="G23" s="5" t="s">
@@ -2257,7 +2320,7 @@
       <c r="E24" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="F24" s="5">
+      <c r="F24" s="14">
         <v>-1</v>
       </c>
       <c r="G24" s="5" t="s">
@@ -2297,7 +2360,7 @@
       <c r="E25" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="F25" s="5">
+      <c r="F25" s="14">
         <v>-1</v>
       </c>
       <c r="G25" s="5" t="s">
@@ -2337,7 +2400,7 @@
       <c r="E26" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="F26" s="5">
+      <c r="F26" s="14">
         <v>-1</v>
       </c>
       <c r="G26" s="5" t="s">
@@ -2377,7 +2440,7 @@
       <c r="E27" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="F27" s="5">
+      <c r="F27" s="14">
         <v>-1</v>
       </c>
       <c r="G27" s="5" t="s">
@@ -2416,7 +2479,7 @@
       <c r="E28" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="F28" s="5">
+      <c r="F28" s="14">
         <v>-1</v>
       </c>
       <c r="G28" s="5" t="s">
@@ -2455,7 +2518,7 @@
       <c r="E29" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="F29" s="8">
+      <c r="F29" s="17">
         <v>-1</v>
       </c>
       <c r="G29" s="8" t="s">
@@ -2496,7 +2559,7 @@
       <c r="E30" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="F30" s="13">
+      <c r="F30" s="18">
         <v>3</v>
       </c>
       <c r="G30" s="11" t="s">
@@ -2531,13 +2594,13 @@
       <c r="C31" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="D31" s="14" t="s">
+      <c r="D31" s="13" t="s">
         <v>79</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="F31" s="15">
+      <c r="F31" s="19">
         <v>-1</v>
       </c>
       <c r="G31" s="9" t="s">
@@ -2577,7 +2640,7 @@
       <c r="E32" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="F32" s="7">
+      <c r="F32" s="14">
         <v>3</v>
       </c>
       <c r="G32" s="7" t="s">
@@ -2604,89 +2667,215 @@
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A33" s="6"/>
-      <c r="B33" s="6"/>
-      <c r="C33" s="6"/>
-      <c r="D33" s="6"/>
-      <c r="E33" s="6"/>
-      <c r="F33" s="6"/>
-      <c r="G33" s="6"/>
-      <c r="H33" s="6"/>
-      <c r="I33" s="6"/>
-      <c r="J33" s="6"/>
-      <c r="K33" s="5"/>
+      <c r="A33" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F33" s="14">
+        <v>-1</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="H33" s="5"/>
+      <c r="I33" s="8">
+        <v>20</v>
+      </c>
+      <c r="J33" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>193</v>
+      </c>
       <c r="L33" s="6"/>
       <c r="M33" s="6"/>
-      <c r="N33" s="6"/>
-      <c r="O33" s="6"/>
+      <c r="N33" s="6">
+        <v>0</v>
+      </c>
+      <c r="O33" s="6" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A34" s="6"/>
-      <c r="B34" s="6"/>
-      <c r="C34" s="6"/>
-      <c r="D34" s="6"/>
-      <c r="E34" s="6"/>
-      <c r="F34" s="6"/>
-      <c r="G34" s="6"/>
-      <c r="H34" s="6"/>
-      <c r="I34" s="6"/>
-      <c r="J34" s="6"/>
-      <c r="K34" s="6"/>
+      <c r="A34" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F34" s="14">
+        <v>-1</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="H34" s="5"/>
+      <c r="I34" s="8">
+        <v>20</v>
+      </c>
+      <c r="J34" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>199</v>
+      </c>
       <c r="L34" s="6"/>
       <c r="M34" s="6"/>
-      <c r="N34" s="6"/>
-      <c r="O34" s="6"/>
+      <c r="N34" s="6">
+        <v>0</v>
+      </c>
+      <c r="O34" s="6" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A35" s="6"/>
-      <c r="B35" s="6"/>
-      <c r="C35" s="6"/>
-      <c r="D35" s="6"/>
-      <c r="E35" s="6"/>
-      <c r="F35" s="6"/>
-      <c r="G35" s="6"/>
-      <c r="H35" s="6"/>
-      <c r="I35" s="6"/>
-      <c r="J35" s="6"/>
-      <c r="K35" s="6"/>
-      <c r="L35" s="6"/>
+      <c r="A35" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F35" s="14">
+        <v>-1</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="H35" s="5"/>
+      <c r="I35" s="8">
+        <v>20</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="K35" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="L35" s="6" t="s">
+        <v>201</v>
+      </c>
       <c r="M35" s="6"/>
-      <c r="N35" s="6"/>
-      <c r="O35" s="6"/>
+      <c r="N35" s="6">
+        <v>0</v>
+      </c>
+      <c r="O35" s="6" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A36" s="6"/>
-      <c r="B36" s="6"/>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6"/>
-      <c r="I36" s="6"/>
-      <c r="J36" s="6"/>
-      <c r="K36" s="6"/>
-      <c r="L36" s="6"/>
+      <c r="A36" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F36" s="14">
+        <v>-1</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="H36" s="5"/>
+      <c r="I36" s="8">
+        <v>20</v>
+      </c>
+      <c r="J36" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="K36" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="L36" s="6" t="s">
+        <v>203</v>
+      </c>
       <c r="M36" s="6"/>
-      <c r="N36" s="6"/>
-      <c r="O36" s="6"/>
+      <c r="N36" s="6">
+        <v>10</v>
+      </c>
+      <c r="O36" s="6" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A37" s="6"/>
-      <c r="B37" s="6"/>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
-      <c r="E37" s="6"/>
-      <c r="F37" s="6"/>
-      <c r="G37" s="6"/>
-      <c r="H37" s="6"/>
-      <c r="I37" s="6"/>
-      <c r="J37" s="6"/>
-      <c r="K37" s="6"/>
-      <c r="L37" s="6"/>
+      <c r="A37" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F37" s="14">
+        <v>-1</v>
+      </c>
+      <c r="G37" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="H37" s="5"/>
+      <c r="I37" s="8">
+        <v>20</v>
+      </c>
+      <c r="J37" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="L37" s="6" t="s">
+        <v>202</v>
+      </c>
       <c r="M37" s="6"/>
-      <c r="N37" s="6"/>
-      <c r="O37" s="6"/>
+      <c r="N37" s="6">
+        <v>10</v>
+      </c>
+      <c r="O37" s="6" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38" s="6"/>
@@ -2694,12 +2883,10 @@
       <c r="C38" s="6"/>
       <c r="D38" s="6"/>
       <c r="E38" s="6"/>
-      <c r="F38" s="6"/>
+      <c r="F38" s="15"/>
       <c r="G38" s="6"/>
       <c r="H38" s="6"/>
       <c r="I38" s="6"/>
-      <c r="J38" s="6"/>
-      <c r="K38" s="6"/>
       <c r="L38" s="6"/>
       <c r="M38" s="6"/>
       <c r="N38" s="6"/>
@@ -2711,7 +2898,7 @@
       <c r="C39" s="6"/>
       <c r="D39" s="6"/>
       <c r="E39" s="6"/>
-      <c r="F39" s="6"/>
+      <c r="F39" s="15"/>
       <c r="G39" s="6"/>
       <c r="H39" s="6"/>
       <c r="I39" s="6"/>
@@ -2728,7 +2915,7 @@
       <c r="C40" s="6"/>
       <c r="D40" s="6"/>
       <c r="E40" s="6"/>
-      <c r="F40" s="6"/>
+      <c r="F40" s="15"/>
       <c r="G40" s="6"/>
       <c r="H40" s="6"/>
       <c r="I40" s="6"/>
@@ -2745,7 +2932,7 @@
       <c r="C41" s="6"/>
       <c r="D41" s="6"/>
       <c r="E41" s="6"/>
-      <c r="F41" s="6"/>
+      <c r="F41" s="15"/>
       <c r="G41" s="6"/>
       <c r="H41" s="6"/>
       <c r="I41" s="6"/>
@@ -2762,7 +2949,7 @@
       <c r="C42" s="6"/>
       <c r="D42" s="6"/>
       <c r="E42" s="6"/>
-      <c r="F42" s="6"/>
+      <c r="F42" s="15"/>
       <c r="G42" s="6"/>
       <c r="H42" s="6"/>
       <c r="I42" s="6"/>
@@ -2779,7 +2966,7 @@
       <c r="C43" s="6"/>
       <c r="D43" s="6"/>
       <c r="E43" s="6"/>
-      <c r="F43" s="6"/>
+      <c r="F43" s="15"/>
       <c r="G43" s="6"/>
       <c r="H43" s="6"/>
       <c r="I43" s="6"/>
@@ -2796,7 +2983,7 @@
       <c r="C44" s="6"/>
       <c r="D44" s="6"/>
       <c r="E44" s="6"/>
-      <c r="F44" s="6"/>
+      <c r="F44" s="15"/>
       <c r="G44" s="6"/>
       <c r="H44" s="6"/>
       <c r="I44" s="6"/>
@@ -2813,7 +3000,7 @@
       <c r="C45" s="6"/>
       <c r="D45" s="6"/>
       <c r="E45" s="6"/>
-      <c r="F45" s="6"/>
+      <c r="F45" s="15"/>
       <c r="G45" s="6"/>
       <c r="H45" s="6"/>
       <c r="I45" s="6"/>
@@ -2830,7 +3017,7 @@
       <c r="C46" s="6"/>
       <c r="D46" s="6"/>
       <c r="E46" s="6"/>
-      <c r="F46" s="6"/>
+      <c r="F46" s="15"/>
       <c r="G46" s="6"/>
       <c r="H46" s="6"/>
       <c r="I46" s="6"/>
@@ -2847,7 +3034,7 @@
       <c r="C47" s="6"/>
       <c r="D47" s="6"/>
       <c r="E47" s="6"/>
-      <c r="F47" s="6"/>
+      <c r="F47" s="15"/>
       <c r="G47" s="6"/>
       <c r="H47" s="6"/>
       <c r="I47" s="6"/>
@@ -2864,7 +3051,7 @@
       <c r="C48" s="6"/>
       <c r="D48" s="6"/>
       <c r="E48" s="6"/>
-      <c r="F48" s="6"/>
+      <c r="F48" s="15"/>
       <c r="G48" s="6"/>
       <c r="H48" s="6"/>
       <c r="I48" s="6"/>
@@ -2881,7 +3068,7 @@
       <c r="C49" s="6"/>
       <c r="D49" s="6"/>
       <c r="E49" s="6"/>
-      <c r="F49" s="6"/>
+      <c r="F49" s="15"/>
       <c r="G49" s="6"/>
       <c r="H49" s="6"/>
       <c r="I49" s="6"/>
@@ -2898,7 +3085,7 @@
       <c r="C50" s="6"/>
       <c r="D50" s="6"/>
       <c r="E50" s="6"/>
-      <c r="F50" s="6"/>
+      <c r="F50" s="15"/>
       <c r="G50" s="6"/>
       <c r="H50" s="6"/>
       <c r="I50" s="6"/>
@@ -2915,7 +3102,7 @@
       <c r="C51" s="6"/>
       <c r="D51" s="6"/>
       <c r="E51" s="6"/>
-      <c r="F51" s="6"/>
+      <c r="F51" s="15"/>
       <c r="G51" s="6"/>
       <c r="H51" s="6"/>
       <c r="I51" s="6"/>
@@ -2932,7 +3119,7 @@
       <c r="C52" s="6"/>
       <c r="D52" s="6"/>
       <c r="E52" s="6"/>
-      <c r="F52" s="6"/>
+      <c r="F52" s="15"/>
       <c r="G52" s="6"/>
       <c r="H52" s="6"/>
       <c r="I52" s="6"/>
@@ -2949,7 +3136,7 @@
       <c r="C53" s="6"/>
       <c r="D53" s="6"/>
       <c r="E53" s="6"/>
-      <c r="F53" s="6"/>
+      <c r="F53" s="15"/>
       <c r="G53" s="6"/>
       <c r="H53" s="6"/>
       <c r="I53" s="6"/>
@@ -2966,7 +3153,7 @@
       <c r="C54" s="6"/>
       <c r="D54" s="6"/>
       <c r="E54" s="6"/>
-      <c r="F54" s="6"/>
+      <c r="F54" s="15"/>
       <c r="G54" s="6"/>
       <c r="H54" s="6"/>
       <c r="I54" s="6"/>
@@ -2983,7 +3170,7 @@
       <c r="C55" s="6"/>
       <c r="D55" s="6"/>
       <c r="E55" s="6"/>
-      <c r="F55" s="6"/>
+      <c r="F55" s="15"/>
       <c r="G55" s="6"/>
       <c r="H55" s="6"/>
       <c r="I55" s="6"/>
@@ -3000,7 +3187,7 @@
       <c r="C56" s="6"/>
       <c r="D56" s="6"/>
       <c r="E56" s="6"/>
-      <c r="F56" s="6"/>
+      <c r="F56" s="15"/>
       <c r="G56" s="6"/>
       <c r="H56" s="6"/>
       <c r="I56" s="6"/>
@@ -3017,7 +3204,7 @@
       <c r="C57" s="6"/>
       <c r="D57" s="6"/>
       <c r="E57" s="6"/>
-      <c r="F57" s="6"/>
+      <c r="F57" s="15"/>
       <c r="G57" s="6"/>
       <c r="H57" s="6"/>
       <c r="I57" s="6"/>
@@ -3034,7 +3221,7 @@
       <c r="C58" s="6"/>
       <c r="D58" s="6"/>
       <c r="E58" s="6"/>
-      <c r="F58" s="6"/>
+      <c r="F58" s="15"/>
       <c r="G58" s="6"/>
       <c r="H58" s="6"/>
       <c r="I58" s="6"/>
@@ -3051,7 +3238,7 @@
       <c r="C59" s="6"/>
       <c r="D59" s="6"/>
       <c r="E59" s="6"/>
-      <c r="F59" s="6"/>
+      <c r="F59" s="15"/>
       <c r="G59" s="6"/>
       <c r="H59" s="6"/>
       <c r="I59" s="6"/>
@@ -3068,7 +3255,7 @@
       <c r="C60" s="6"/>
       <c r="D60" s="6"/>
       <c r="E60" s="6"/>
-      <c r="F60" s="6"/>
+      <c r="F60" s="15"/>
       <c r="G60" s="6"/>
       <c r="H60" s="6"/>
       <c r="I60" s="6"/>
@@ -3085,7 +3272,7 @@
       <c r="C61" s="6"/>
       <c r="D61" s="6"/>
       <c r="E61" s="6"/>
-      <c r="F61" s="6"/>
+      <c r="F61" s="15"/>
       <c r="G61" s="6"/>
       <c r="H61" s="6"/>
       <c r="I61" s="6"/>
@@ -3102,7 +3289,7 @@
       <c r="C62" s="6"/>
       <c r="D62" s="6"/>
       <c r="E62" s="6"/>
-      <c r="F62" s="6"/>
+      <c r="F62" s="15"/>
       <c r="G62" s="6"/>
       <c r="H62" s="6"/>
       <c r="I62" s="6"/>
@@ -3119,7 +3306,7 @@
       <c r="C63" s="6"/>
       <c r="D63" s="6"/>
       <c r="E63" s="6"/>
-      <c r="F63" s="6"/>
+      <c r="F63" s="15"/>
       <c r="G63" s="6"/>
       <c r="H63" s="6"/>
       <c r="I63" s="6"/>
@@ -3136,7 +3323,7 @@
       <c r="C64" s="6"/>
       <c r="D64" s="6"/>
       <c r="E64" s="6"/>
-      <c r="F64" s="6"/>
+      <c r="F64" s="15"/>
       <c r="G64" s="6"/>
       <c r="H64" s="6"/>
       <c r="I64" s="6"/>
@@ -3153,7 +3340,7 @@
       <c r="C65" s="6"/>
       <c r="D65" s="6"/>
       <c r="E65" s="6"/>
-      <c r="F65" s="6"/>
+      <c r="F65" s="15"/>
       <c r="G65" s="6"/>
       <c r="H65" s="6"/>
       <c r="I65" s="6"/>
@@ -3170,7 +3357,7 @@
       <c r="C66" s="6"/>
       <c r="D66" s="6"/>
       <c r="E66" s="6"/>
-      <c r="F66" s="6"/>
+      <c r="F66" s="15"/>
       <c r="G66" s="6"/>
       <c r="H66" s="6"/>
       <c r="I66" s="6"/>
@@ -3187,7 +3374,7 @@
       <c r="C67" s="6"/>
       <c r="D67" s="6"/>
       <c r="E67" s="6"/>
-      <c r="F67" s="6"/>
+      <c r="F67" s="15"/>
       <c r="G67" s="6"/>
       <c r="H67" s="6"/>
       <c r="I67" s="6"/>
@@ -3204,7 +3391,7 @@
       <c r="C68" s="6"/>
       <c r="D68" s="6"/>
       <c r="E68" s="6"/>
-      <c r="F68" s="6"/>
+      <c r="F68" s="15"/>
       <c r="G68" s="6"/>
       <c r="H68" s="6"/>
       <c r="I68" s="6"/>
@@ -3221,7 +3408,7 @@
       <c r="C69" s="6"/>
       <c r="D69" s="6"/>
       <c r="E69" s="6"/>
-      <c r="F69" s="6"/>
+      <c r="F69" s="15"/>
       <c r="G69" s="6"/>
       <c r="H69" s="6"/>
       <c r="I69" s="6"/>
@@ -3238,7 +3425,7 @@
       <c r="C70" s="6"/>
       <c r="D70" s="6"/>
       <c r="E70" s="6"/>
-      <c r="F70" s="6"/>
+      <c r="F70" s="15"/>
       <c r="G70" s="6"/>
       <c r="H70" s="6"/>
       <c r="I70" s="6"/>
@@ -3255,7 +3442,7 @@
       <c r="C71" s="6"/>
       <c r="D71" s="6"/>
       <c r="E71" s="6"/>
-      <c r="F71" s="6"/>
+      <c r="F71" s="15"/>
       <c r="G71" s="6"/>
       <c r="H71" s="6"/>
       <c r="I71" s="6"/>
@@ -3272,7 +3459,7 @@
       <c r="C72" s="6"/>
       <c r="D72" s="6"/>
       <c r="E72" s="6"/>
-      <c r="F72" s="6"/>
+      <c r="F72" s="15"/>
       <c r="G72" s="6"/>
       <c r="H72" s="6"/>
       <c r="I72" s="6"/>
@@ -3289,7 +3476,7 @@
       <c r="C73" s="6"/>
       <c r="D73" s="6"/>
       <c r="E73" s="6"/>
-      <c r="F73" s="6"/>
+      <c r="F73" s="15"/>
       <c r="G73" s="6"/>
       <c r="H73" s="6"/>
       <c r="I73" s="6"/>
@@ -3306,7 +3493,7 @@
       <c r="C74" s="6"/>
       <c r="D74" s="6"/>
       <c r="E74" s="6"/>
-      <c r="F74" s="6"/>
+      <c r="F74" s="15"/>
       <c r="G74" s="6"/>
       <c r="H74" s="6"/>
       <c r="I74" s="6"/>
@@ -3323,7 +3510,7 @@
       <c r="C75" s="6"/>
       <c r="D75" s="6"/>
       <c r="E75" s="6"/>
-      <c r="F75" s="6"/>
+      <c r="F75" s="15"/>
       <c r="G75" s="6"/>
       <c r="H75" s="6"/>
       <c r="I75" s="6"/>
@@ -3340,7 +3527,7 @@
       <c r="C76" s="6"/>
       <c r="D76" s="6"/>
       <c r="E76" s="6"/>
-      <c r="F76" s="6"/>
+      <c r="F76" s="15"/>
       <c r="G76" s="6"/>
       <c r="H76" s="6"/>
       <c r="I76" s="6"/>
@@ -3357,7 +3544,7 @@
       <c r="C77" s="6"/>
       <c r="D77" s="6"/>
       <c r="E77" s="6"/>
-      <c r="F77" s="6"/>
+      <c r="F77" s="15"/>
       <c r="G77" s="6"/>
       <c r="H77" s="6"/>
       <c r="I77" s="6"/>
@@ -3374,7 +3561,7 @@
       <c r="C78" s="6"/>
       <c r="D78" s="6"/>
       <c r="E78" s="6"/>
-      <c r="F78" s="6"/>
+      <c r="F78" s="15"/>
       <c r="G78" s="6"/>
       <c r="H78" s="6"/>
       <c r="I78" s="6"/>
@@ -3391,7 +3578,7 @@
       <c r="C79" s="6"/>
       <c r="D79" s="6"/>
       <c r="E79" s="6"/>
-      <c r="F79" s="6"/>
+      <c r="F79" s="15"/>
       <c r="G79" s="6"/>
       <c r="H79" s="6"/>
       <c r="I79" s="6"/>
@@ -3408,7 +3595,7 @@
       <c r="C80" s="6"/>
       <c r="D80" s="6"/>
       <c r="E80" s="6"/>
-      <c r="F80" s="6"/>
+      <c r="F80" s="15"/>
       <c r="G80" s="6"/>
       <c r="H80" s="6"/>
       <c r="I80" s="6"/>
@@ -3425,7 +3612,7 @@
       <c r="C81" s="6"/>
       <c r="D81" s="6"/>
       <c r="E81" s="6"/>
-      <c r="F81" s="6"/>
+      <c r="F81" s="15"/>
       <c r="G81" s="6"/>
       <c r="H81" s="6"/>
       <c r="I81" s="6"/>
@@ -3442,7 +3629,7 @@
       <c r="C82" s="6"/>
       <c r="D82" s="6"/>
       <c r="E82" s="6"/>
-      <c r="F82" s="6"/>
+      <c r="F82" s="15"/>
       <c r="G82" s="6"/>
       <c r="H82" s="6"/>
       <c r="I82" s="6"/>
@@ -3459,7 +3646,7 @@
       <c r="C83" s="6"/>
       <c r="D83" s="6"/>
       <c r="E83" s="6"/>
-      <c r="F83" s="6"/>
+      <c r="F83" s="15"/>
       <c r="G83" s="6"/>
       <c r="H83" s="6"/>
       <c r="I83" s="6"/>
@@ -3476,7 +3663,7 @@
       <c r="C84" s="6"/>
       <c r="D84" s="6"/>
       <c r="E84" s="6"/>
-      <c r="F84" s="6"/>
+      <c r="F84" s="15"/>
       <c r="G84" s="6"/>
       <c r="H84" s="6"/>
       <c r="I84" s="6"/>
@@ -3493,7 +3680,7 @@
       <c r="C85" s="6"/>
       <c r="D85" s="6"/>
       <c r="E85" s="6"/>
-      <c r="F85" s="6"/>
+      <c r="F85" s="15"/>
       <c r="G85" s="6"/>
       <c r="H85" s="6"/>
       <c r="I85" s="6"/>
@@ -3510,7 +3697,7 @@
       <c r="C86" s="6"/>
       <c r="D86" s="6"/>
       <c r="E86" s="6"/>
-      <c r="F86" s="6"/>
+      <c r="F86" s="15"/>
       <c r="G86" s="6"/>
       <c r="H86" s="6"/>
       <c r="I86" s="6"/>
@@ -3527,7 +3714,7 @@
       <c r="C87" s="6"/>
       <c r="D87" s="6"/>
       <c r="E87" s="6"/>
-      <c r="F87" s="6"/>
+      <c r="F87" s="15"/>
       <c r="G87" s="6"/>
       <c r="H87" s="6"/>
       <c r="I87" s="6"/>
@@ -3544,7 +3731,7 @@
       <c r="C88" s="6"/>
       <c r="D88" s="6"/>
       <c r="E88" s="6"/>
-      <c r="F88" s="6"/>
+      <c r="F88" s="15"/>
       <c r="G88" s="6"/>
       <c r="H88" s="6"/>
       <c r="I88" s="6"/>
@@ -3561,7 +3748,7 @@
       <c r="C89" s="6"/>
       <c r="D89" s="6"/>
       <c r="E89" s="6"/>
-      <c r="F89" s="6"/>
+      <c r="F89" s="15"/>
       <c r="G89" s="6"/>
       <c r="H89" s="6"/>
       <c r="I89" s="6"/>
@@ -3578,7 +3765,7 @@
       <c r="C90" s="6"/>
       <c r="D90" s="6"/>
       <c r="E90" s="6"/>
-      <c r="F90" s="6"/>
+      <c r="F90" s="15"/>
       <c r="G90" s="6"/>
       <c r="H90" s="6"/>
       <c r="I90" s="6"/>
@@ -3595,7 +3782,7 @@
       <c r="C91" s="6"/>
       <c r="D91" s="6"/>
       <c r="E91" s="6"/>
-      <c r="F91" s="6"/>
+      <c r="F91" s="15"/>
       <c r="G91" s="6"/>
       <c r="H91" s="6"/>
       <c r="I91" s="6"/>
@@ -3612,7 +3799,7 @@
       <c r="C92" s="6"/>
       <c r="D92" s="6"/>
       <c r="E92" s="6"/>
-      <c r="F92" s="6"/>
+      <c r="F92" s="15"/>
       <c r="G92" s="6"/>
       <c r="H92" s="6"/>
       <c r="I92" s="6"/>
@@ -3629,7 +3816,7 @@
       <c r="C93" s="6"/>
       <c r="D93" s="6"/>
       <c r="E93" s="6"/>
-      <c r="F93" s="6"/>
+      <c r="F93" s="15"/>
       <c r="G93" s="6"/>
       <c r="H93" s="6"/>
       <c r="I93" s="6"/>
@@ -3646,7 +3833,7 @@
       <c r="C94" s="6"/>
       <c r="D94" s="6"/>
       <c r="E94" s="6"/>
-      <c r="F94" s="6"/>
+      <c r="F94" s="15"/>
       <c r="G94" s="6"/>
       <c r="H94" s="6"/>
       <c r="I94" s="6"/>
@@ -3663,7 +3850,7 @@
       <c r="C95" s="6"/>
       <c r="D95" s="6"/>
       <c r="E95" s="6"/>
-      <c r="F95" s="6"/>
+      <c r="F95" s="15"/>
       <c r="G95" s="6"/>
       <c r="H95" s="6"/>
       <c r="I95" s="6"/>
@@ -3680,7 +3867,7 @@
       <c r="C96" s="6"/>
       <c r="D96" s="6"/>
       <c r="E96" s="6"/>
-      <c r="F96" s="6"/>
+      <c r="F96" s="15"/>
       <c r="G96" s="6"/>
       <c r="H96" s="6"/>
       <c r="I96" s="6"/>
@@ -3697,7 +3884,7 @@
       <c r="C97" s="6"/>
       <c r="D97" s="6"/>
       <c r="E97" s="6"/>
-      <c r="F97" s="6"/>
+      <c r="F97" s="15"/>
       <c r="G97" s="6"/>
       <c r="H97" s="6"/>
       <c r="I97" s="6"/>
@@ -3714,7 +3901,7 @@
       <c r="C98" s="6"/>
       <c r="D98" s="6"/>
       <c r="E98" s="6"/>
-      <c r="F98" s="6"/>
+      <c r="F98" s="15"/>
       <c r="G98" s="6"/>
       <c r="H98" s="6"/>
       <c r="I98" s="6"/>
@@ -3731,7 +3918,7 @@
       <c r="C99" s="6"/>
       <c r="D99" s="6"/>
       <c r="E99" s="6"/>
-      <c r="F99" s="6"/>
+      <c r="F99" s="15"/>
       <c r="G99" s="6"/>
       <c r="H99" s="6"/>
       <c r="I99" s="6"/>
@@ -3748,7 +3935,7 @@
       <c r="C100" s="6"/>
       <c r="D100" s="6"/>
       <c r="E100" s="6"/>
-      <c r="F100" s="6"/>
+      <c r="F100" s="15"/>
       <c r="G100" s="6"/>
       <c r="H100" s="6"/>
       <c r="I100" s="6"/>
@@ -3765,7 +3952,7 @@
       <c r="C101" s="6"/>
       <c r="D101" s="6"/>
       <c r="E101" s="6"/>
-      <c r="F101" s="6"/>
+      <c r="F101" s="15"/>
       <c r="G101" s="6"/>
       <c r="H101" s="6"/>
       <c r="I101" s="6"/>
@@ -3782,7 +3969,7 @@
       <c r="C102" s="6"/>
       <c r="D102" s="6"/>
       <c r="E102" s="6"/>
-      <c r="F102" s="6"/>
+      <c r="F102" s="15"/>
       <c r="G102" s="6"/>
       <c r="H102" s="6"/>
       <c r="I102" s="6"/>
@@ -3799,7 +3986,7 @@
       <c r="C103" s="6"/>
       <c r="D103" s="6"/>
       <c r="E103" s="6"/>
-      <c r="F103" s="6"/>
+      <c r="F103" s="15"/>
       <c r="G103" s="6"/>
       <c r="H103" s="6"/>
       <c r="I103" s="6"/>
@@ -3816,7 +4003,7 @@
       <c r="C104" s="6"/>
       <c r="D104" s="6"/>
       <c r="E104" s="6"/>
-      <c r="F104" s="6"/>
+      <c r="F104" s="15"/>
       <c r="G104" s="6"/>
       <c r="H104" s="6"/>
       <c r="I104" s="6"/>
@@ -3833,7 +4020,7 @@
       <c r="C105" s="6"/>
       <c r="D105" s="6"/>
       <c r="E105" s="6"/>
-      <c r="F105" s="6"/>
+      <c r="F105" s="15"/>
       <c r="G105" s="6"/>
       <c r="H105" s="6"/>
       <c r="I105" s="6"/>
@@ -3850,7 +4037,7 @@
       <c r="C106" s="6"/>
       <c r="D106" s="6"/>
       <c r="E106" s="6"/>
-      <c r="F106" s="6"/>
+      <c r="F106" s="15"/>
       <c r="G106" s="6"/>
       <c r="H106" s="6"/>
       <c r="I106" s="6"/>
@@ -3867,7 +4054,7 @@
       <c r="C107" s="6"/>
       <c r="D107" s="6"/>
       <c r="E107" s="6"/>
-      <c r="F107" s="6"/>
+      <c r="F107" s="15"/>
       <c r="G107" s="6"/>
       <c r="H107" s="6"/>
       <c r="I107" s="6"/>
@@ -3884,7 +4071,7 @@
       <c r="C108" s="6"/>
       <c r="D108" s="6"/>
       <c r="E108" s="6"/>
-      <c r="F108" s="6"/>
+      <c r="F108" s="15"/>
       <c r="G108" s="6"/>
       <c r="H108" s="6"/>
       <c r="I108" s="6"/>
@@ -3901,7 +4088,7 @@
       <c r="C109" s="6"/>
       <c r="D109" s="6"/>
       <c r="E109" s="6"/>
-      <c r="F109" s="6"/>
+      <c r="F109" s="15"/>
       <c r="G109" s="6"/>
       <c r="H109" s="6"/>
       <c r="I109" s="6"/>
@@ -3918,7 +4105,7 @@
       <c r="C110" s="6"/>
       <c r="D110" s="6"/>
       <c r="E110" s="6"/>
-      <c r="F110" s="6"/>
+      <c r="F110" s="15"/>
       <c r="G110" s="6"/>
       <c r="H110" s="6"/>
       <c r="I110" s="6"/>
@@ -3935,7 +4122,7 @@
       <c r="C111" s="6"/>
       <c r="D111" s="6"/>
       <c r="E111" s="6"/>
-      <c r="F111" s="6"/>
+      <c r="F111" s="15"/>
       <c r="G111" s="6"/>
       <c r="H111" s="6"/>
       <c r="I111" s="6"/>
@@ -3952,7 +4139,7 @@
       <c r="C112" s="6"/>
       <c r="D112" s="6"/>
       <c r="E112" s="6"/>
-      <c r="F112" s="6"/>
+      <c r="F112" s="15"/>
       <c r="G112" s="6"/>
       <c r="H112" s="6"/>
       <c r="I112" s="6"/>
@@ -3969,7 +4156,7 @@
       <c r="C113" s="6"/>
       <c r="D113" s="6"/>
       <c r="E113" s="6"/>
-      <c r="F113" s="6"/>
+      <c r="F113" s="15"/>
       <c r="G113" s="6"/>
       <c r="H113" s="6"/>
       <c r="I113" s="6"/>
@@ -3986,7 +4173,7 @@
       <c r="C114" s="6"/>
       <c r="D114" s="6"/>
       <c r="E114" s="6"/>
-      <c r="F114" s="6"/>
+      <c r="F114" s="15"/>
       <c r="G114" s="6"/>
       <c r="H114" s="6"/>
       <c r="I114" s="6"/>
@@ -4003,7 +4190,7 @@
       <c r="C115" s="6"/>
       <c r="D115" s="6"/>
       <c r="E115" s="6"/>
-      <c r="F115" s="6"/>
+      <c r="F115" s="15"/>
       <c r="G115" s="6"/>
       <c r="H115" s="6"/>
       <c r="I115" s="6"/>
@@ -4020,7 +4207,7 @@
       <c r="C116" s="6"/>
       <c r="D116" s="6"/>
       <c r="E116" s="6"/>
-      <c r="F116" s="6"/>
+      <c r="F116" s="15"/>
       <c r="G116" s="6"/>
       <c r="H116" s="6"/>
       <c r="I116" s="6"/>
@@ -4037,7 +4224,7 @@
       <c r="C117" s="6"/>
       <c r="D117" s="6"/>
       <c r="E117" s="6"/>
-      <c r="F117" s="6"/>
+      <c r="F117" s="15"/>
       <c r="G117" s="6"/>
       <c r="H117" s="6"/>
       <c r="I117" s="6"/>
@@ -4054,7 +4241,7 @@
       <c r="C118" s="6"/>
       <c r="D118" s="6"/>
       <c r="E118" s="6"/>
-      <c r="F118" s="6"/>
+      <c r="F118" s="15"/>
       <c r="G118" s="6"/>
       <c r="H118" s="6"/>
       <c r="I118" s="6"/>
@@ -4071,7 +4258,7 @@
       <c r="C119" s="6"/>
       <c r="D119" s="6"/>
       <c r="E119" s="6"/>
-      <c r="F119" s="6"/>
+      <c r="F119" s="15"/>
       <c r="G119" s="6"/>
       <c r="H119" s="6"/>
       <c r="I119" s="6"/>
@@ -4088,7 +4275,7 @@
       <c r="C120" s="6"/>
       <c r="D120" s="6"/>
       <c r="E120" s="6"/>
-      <c r="F120" s="6"/>
+      <c r="F120" s="15"/>
       <c r="G120" s="6"/>
       <c r="H120" s="6"/>
       <c r="I120" s="6"/>
@@ -4105,7 +4292,7 @@
       <c r="C121" s="6"/>
       <c r="D121" s="6"/>
       <c r="E121" s="6"/>
-      <c r="F121" s="6"/>
+      <c r="F121" s="15"/>
       <c r="G121" s="6"/>
       <c r="H121" s="6"/>
       <c r="I121" s="6"/>
@@ -4122,7 +4309,7 @@
       <c r="C122" s="6"/>
       <c r="D122" s="6"/>
       <c r="E122" s="6"/>
-      <c r="F122" s="6"/>
+      <c r="F122" s="15"/>
       <c r="G122" s="6"/>
       <c r="H122" s="6"/>
       <c r="I122" s="6"/>
@@ -4139,7 +4326,7 @@
       <c r="C123" s="6"/>
       <c r="D123" s="6"/>
       <c r="E123" s="6"/>
-      <c r="F123" s="6"/>
+      <c r="F123" s="15"/>
       <c r="G123" s="6"/>
       <c r="H123" s="6"/>
       <c r="I123" s="6"/>
@@ -4156,7 +4343,7 @@
       <c r="C124" s="6"/>
       <c r="D124" s="6"/>
       <c r="E124" s="6"/>
-      <c r="F124" s="6"/>
+      <c r="F124" s="15"/>
       <c r="G124" s="6"/>
       <c r="H124" s="6"/>
       <c r="I124" s="6"/>
@@ -4173,7 +4360,7 @@
       <c r="C125" s="6"/>
       <c r="D125" s="6"/>
       <c r="E125" s="6"/>
-      <c r="F125" s="6"/>
+      <c r="F125" s="15"/>
       <c r="G125" s="6"/>
       <c r="H125" s="6"/>
       <c r="I125" s="6"/>
@@ -4190,7 +4377,7 @@
       <c r="C126" s="6"/>
       <c r="D126" s="6"/>
       <c r="E126" s="6"/>
-      <c r="F126" s="6"/>
+      <c r="F126" s="15"/>
       <c r="G126" s="6"/>
       <c r="H126" s="6"/>
       <c r="I126" s="6"/>
@@ -4207,7 +4394,7 @@
       <c r="C127" s="6"/>
       <c r="D127" s="6"/>
       <c r="E127" s="6"/>
-      <c r="F127" s="6"/>
+      <c r="F127" s="15"/>
       <c r="G127" s="6"/>
       <c r="H127" s="6"/>
       <c r="I127" s="6"/>
@@ -4224,7 +4411,7 @@
       <c r="C128" s="6"/>
       <c r="D128" s="6"/>
       <c r="E128" s="6"/>
-      <c r="F128" s="6"/>
+      <c r="F128" s="15"/>
       <c r="G128" s="6"/>
       <c r="H128" s="6"/>
       <c r="I128" s="6"/>
@@ -4241,7 +4428,7 @@
       <c r="C129" s="6"/>
       <c r="D129" s="6"/>
       <c r="E129" s="6"/>
-      <c r="F129" s="6"/>
+      <c r="F129" s="15"/>
       <c r="G129" s="6"/>
       <c r="H129" s="6"/>
       <c r="I129" s="6"/>
@@ -4258,7 +4445,7 @@
       <c r="C130" s="6"/>
       <c r="D130" s="6"/>
       <c r="E130" s="6"/>
-      <c r="F130" s="6"/>
+      <c r="F130" s="15"/>
       <c r="G130" s="6"/>
       <c r="H130" s="6"/>
       <c r="I130" s="6"/>
@@ -4275,7 +4462,7 @@
       <c r="C131" s="6"/>
       <c r="D131" s="6"/>
       <c r="E131" s="6"/>
-      <c r="F131" s="6"/>
+      <c r="F131" s="15"/>
       <c r="G131" s="6"/>
       <c r="H131" s="6"/>
       <c r="I131" s="6"/>
@@ -4292,7 +4479,7 @@
       <c r="C132" s="6"/>
       <c r="D132" s="6"/>
       <c r="E132" s="6"/>
-      <c r="F132" s="6"/>
+      <c r="F132" s="15"/>
       <c r="G132" s="6"/>
       <c r="H132" s="6"/>
       <c r="I132" s="6"/>
@@ -4309,7 +4496,7 @@
       <c r="C133" s="6"/>
       <c r="D133" s="6"/>
       <c r="E133" s="6"/>
-      <c r="F133" s="6"/>
+      <c r="F133" s="15"/>
       <c r="G133" s="6"/>
       <c r="H133" s="6"/>
       <c r="I133" s="6"/>
@@ -4326,7 +4513,7 @@
       <c r="C134" s="6"/>
       <c r="D134" s="6"/>
       <c r="E134" s="6"/>
-      <c r="F134" s="6"/>
+      <c r="F134" s="15"/>
       <c r="G134" s="6"/>
       <c r="H134" s="6"/>
       <c r="I134" s="6"/>
@@ -4343,7 +4530,7 @@
       <c r="C135" s="6"/>
       <c r="D135" s="6"/>
       <c r="E135" s="6"/>
-      <c r="F135" s="6"/>
+      <c r="F135" s="15"/>
       <c r="G135" s="6"/>
       <c r="H135" s="6"/>
       <c r="I135" s="6"/>
@@ -4360,7 +4547,7 @@
       <c r="C136" s="6"/>
       <c r="D136" s="6"/>
       <c r="E136" s="6"/>
-      <c r="F136" s="6"/>
+      <c r="F136" s="15"/>
       <c r="G136" s="6"/>
       <c r="H136" s="6"/>
       <c r="I136" s="6"/>
@@ -4377,7 +4564,7 @@
       <c r="C137" s="6"/>
       <c r="D137" s="6"/>
       <c r="E137" s="6"/>
-      <c r="F137" s="6"/>
+      <c r="F137" s="15"/>
       <c r="G137" s="6"/>
       <c r="H137" s="6"/>
       <c r="I137" s="6"/>
@@ -4394,7 +4581,7 @@
       <c r="C138" s="6"/>
       <c r="D138" s="6"/>
       <c r="E138" s="6"/>
-      <c r="F138" s="6"/>
+      <c r="F138" s="15"/>
       <c r="G138" s="6"/>
       <c r="H138" s="6"/>
       <c r="I138" s="6"/>
@@ -4411,7 +4598,7 @@
       <c r="C139" s="6"/>
       <c r="D139" s="6"/>
       <c r="E139" s="6"/>
-      <c r="F139" s="6"/>
+      <c r="F139" s="15"/>
       <c r="G139" s="6"/>
       <c r="H139" s="6"/>
       <c r="I139" s="6"/>
@@ -4428,7 +4615,7 @@
       <c r="C140" s="6"/>
       <c r="D140" s="6"/>
       <c r="E140" s="6"/>
-      <c r="F140" s="6"/>
+      <c r="F140" s="15"/>
       <c r="G140" s="6"/>
       <c r="H140" s="6"/>
       <c r="I140" s="6"/>
@@ -4445,7 +4632,7 @@
       <c r="C141" s="6"/>
       <c r="D141" s="6"/>
       <c r="E141" s="6"/>
-      <c r="F141" s="6"/>
+      <c r="F141" s="15"/>
       <c r="G141" s="6"/>
       <c r="H141" s="6"/>
       <c r="I141" s="6"/>
@@ -4462,7 +4649,7 @@
       <c r="C142" s="6"/>
       <c r="D142" s="6"/>
       <c r="E142" s="6"/>
-      <c r="F142" s="6"/>
+      <c r="F142" s="15"/>
       <c r="G142" s="6"/>
       <c r="H142" s="6"/>
       <c r="I142" s="6"/>
@@ -4479,7 +4666,7 @@
       <c r="C143" s="6"/>
       <c r="D143" s="6"/>
       <c r="E143" s="6"/>
-      <c r="F143" s="6"/>
+      <c r="F143" s="15"/>
       <c r="G143" s="6"/>
       <c r="H143" s="6"/>
       <c r="I143" s="6"/>
@@ -4496,7 +4683,7 @@
       <c r="C144" s="6"/>
       <c r="D144" s="6"/>
       <c r="E144" s="6"/>
-      <c r="F144" s="6"/>
+      <c r="F144" s="15"/>
       <c r="G144" s="6"/>
       <c r="H144" s="6"/>
       <c r="I144" s="6"/>
@@ -4513,7 +4700,7 @@
       <c r="C145" s="6"/>
       <c r="D145" s="6"/>
       <c r="E145" s="6"/>
-      <c r="F145" s="6"/>
+      <c r="F145" s="15"/>
       <c r="G145" s="6"/>
       <c r="H145" s="6"/>
       <c r="I145" s="6"/>
@@ -4530,7 +4717,7 @@
       <c r="C146" s="6"/>
       <c r="D146" s="6"/>
       <c r="E146" s="6"/>
-      <c r="F146" s="6"/>
+      <c r="F146" s="15"/>
       <c r="G146" s="6"/>
       <c r="H146" s="6"/>
       <c r="I146" s="6"/>
@@ -4547,7 +4734,7 @@
       <c r="C147" s="6"/>
       <c r="D147" s="6"/>
       <c r="E147" s="6"/>
-      <c r="F147" s="6"/>
+      <c r="F147" s="15"/>
       <c r="G147" s="6"/>
       <c r="H147" s="6"/>
       <c r="I147" s="6"/>
@@ -4564,7 +4751,7 @@
       <c r="C148" s="6"/>
       <c r="D148" s="6"/>
       <c r="E148" s="6"/>
-      <c r="F148" s="6"/>
+      <c r="F148" s="15"/>
       <c r="G148" s="6"/>
       <c r="H148" s="6"/>
       <c r="I148" s="6"/>
@@ -4581,7 +4768,7 @@
       <c r="C149" s="6"/>
       <c r="D149" s="6"/>
       <c r="E149" s="6"/>
-      <c r="F149" s="6"/>
+      <c r="F149" s="15"/>
       <c r="G149" s="6"/>
       <c r="H149" s="6"/>
       <c r="I149" s="6"/>
@@ -4598,7 +4785,7 @@
       <c r="C150" s="6"/>
       <c r="D150" s="6"/>
       <c r="E150" s="6"/>
-      <c r="F150" s="6"/>
+      <c r="F150" s="15"/>
       <c r="G150" s="6"/>
       <c r="H150" s="6"/>
       <c r="I150" s="6"/>
@@ -4615,7 +4802,7 @@
       <c r="C151" s="6"/>
       <c r="D151" s="6"/>
       <c r="E151" s="6"/>
-      <c r="F151" s="6"/>
+      <c r="F151" s="15"/>
       <c r="G151" s="6"/>
       <c r="H151" s="6"/>
       <c r="I151" s="6"/>
@@ -4632,7 +4819,7 @@
       <c r="C152" s="6"/>
       <c r="D152" s="6"/>
       <c r="E152" s="6"/>
-      <c r="F152" s="6"/>
+      <c r="F152" s="15"/>
       <c r="G152" s="6"/>
       <c r="H152" s="6"/>
       <c r="I152" s="6"/>
@@ -4649,7 +4836,7 @@
       <c r="C153" s="6"/>
       <c r="D153" s="6"/>
       <c r="E153" s="6"/>
-      <c r="F153" s="6"/>
+      <c r="F153" s="15"/>
       <c r="G153" s="6"/>
       <c r="H153" s="6"/>
       <c r="I153" s="6"/>
@@ -4666,7 +4853,7 @@
       <c r="C154" s="6"/>
       <c r="D154" s="6"/>
       <c r="E154" s="6"/>
-      <c r="F154" s="6"/>
+      <c r="F154" s="15"/>
       <c r="G154" s="6"/>
       <c r="H154" s="6"/>
       <c r="I154" s="6"/>
@@ -4683,7 +4870,7 @@
       <c r="C155" s="6"/>
       <c r="D155" s="6"/>
       <c r="E155" s="6"/>
-      <c r="F155" s="6"/>
+      <c r="F155" s="15"/>
       <c r="G155" s="6"/>
       <c r="H155" s="6"/>
       <c r="I155" s="6"/>
@@ -4700,7 +4887,7 @@
       <c r="C156" s="6"/>
       <c r="D156" s="6"/>
       <c r="E156" s="6"/>
-      <c r="F156" s="6"/>
+      <c r="F156" s="15"/>
       <c r="G156" s="6"/>
       <c r="H156" s="6"/>
       <c r="I156" s="6"/>
@@ -4717,7 +4904,7 @@
       <c r="C157" s="6"/>
       <c r="D157" s="6"/>
       <c r="E157" s="6"/>
-      <c r="F157" s="6"/>
+      <c r="F157" s="15"/>
       <c r="G157" s="6"/>
       <c r="H157" s="6"/>
       <c r="I157" s="6"/>
@@ -4734,7 +4921,7 @@
       <c r="C158" s="6"/>
       <c r="D158" s="6"/>
       <c r="E158" s="6"/>
-      <c r="F158" s="6"/>
+      <c r="F158" s="15"/>
       <c r="G158" s="6"/>
       <c r="H158" s="6"/>
       <c r="I158" s="6"/>
@@ -4751,7 +4938,7 @@
       <c r="C159" s="6"/>
       <c r="D159" s="6"/>
       <c r="E159" s="6"/>
-      <c r="F159" s="6"/>
+      <c r="F159" s="15"/>
       <c r="G159" s="6"/>
       <c r="H159" s="6"/>
       <c r="I159" s="6"/>
@@ -4768,7 +4955,7 @@
       <c r="C160" s="6"/>
       <c r="D160" s="6"/>
       <c r="E160" s="6"/>
-      <c r="F160" s="6"/>
+      <c r="F160" s="15"/>
       <c r="G160" s="6"/>
       <c r="H160" s="6"/>
       <c r="I160" s="6"/>
@@ -4785,7 +4972,7 @@
       <c r="C161" s="6"/>
       <c r="D161" s="6"/>
       <c r="E161" s="6"/>
-      <c r="F161" s="6"/>
+      <c r="F161" s="15"/>
       <c r="G161" s="6"/>
       <c r="H161" s="6"/>
       <c r="I161" s="6"/>
@@ -4802,7 +4989,7 @@
       <c r="C162" s="6"/>
       <c r="D162" s="6"/>
       <c r="E162" s="6"/>
-      <c r="F162" s="6"/>
+      <c r="F162" s="15"/>
       <c r="G162" s="6"/>
       <c r="H162" s="6"/>
       <c r="I162" s="6"/>
@@ -4819,7 +5006,7 @@
       <c r="C163" s="6"/>
       <c r="D163" s="6"/>
       <c r="E163" s="6"/>
-      <c r="F163" s="6"/>
+      <c r="F163" s="15"/>
       <c r="G163" s="6"/>
       <c r="H163" s="6"/>
       <c r="I163" s="6"/>
@@ -4836,7 +5023,7 @@
       <c r="C164" s="6"/>
       <c r="D164" s="6"/>
       <c r="E164" s="6"/>
-      <c r="F164" s="6"/>
+      <c r="F164" s="15"/>
       <c r="G164" s="6"/>
       <c r="H164" s="6"/>
       <c r="I164" s="6"/>
@@ -4853,7 +5040,7 @@
       <c r="C165" s="6"/>
       <c r="D165" s="6"/>
       <c r="E165" s="6"/>
-      <c r="F165" s="6"/>
+      <c r="F165" s="15"/>
       <c r="G165" s="6"/>
       <c r="H165" s="6"/>
       <c r="I165" s="6"/>
@@ -4870,7 +5057,7 @@
       <c r="C166" s="6"/>
       <c r="D166" s="6"/>
       <c r="E166" s="6"/>
-      <c r="F166" s="6"/>
+      <c r="F166" s="15"/>
       <c r="G166" s="6"/>
       <c r="H166" s="6"/>
       <c r="I166" s="6"/>
@@ -4887,7 +5074,7 @@
       <c r="C167" s="6"/>
       <c r="D167" s="6"/>
       <c r="E167" s="6"/>
-      <c r="F167" s="6"/>
+      <c r="F167" s="15"/>
       <c r="G167" s="6"/>
       <c r="H167" s="6"/>
       <c r="I167" s="6"/>
@@ -4904,7 +5091,7 @@
       <c r="C168" s="6"/>
       <c r="D168" s="6"/>
       <c r="E168" s="6"/>
-      <c r="F168" s="6"/>
+      <c r="F168" s="15"/>
       <c r="G168" s="6"/>
       <c r="H168" s="6"/>
       <c r="I168" s="6"/>
@@ -4921,7 +5108,7 @@
       <c r="C169" s="6"/>
       <c r="D169" s="6"/>
       <c r="E169" s="6"/>
-      <c r="F169" s="6"/>
+      <c r="F169" s="15"/>
       <c r="G169" s="6"/>
       <c r="H169" s="6"/>
       <c r="I169" s="6"/>
@@ -4938,7 +5125,7 @@
       <c r="C170" s="6"/>
       <c r="D170" s="6"/>
       <c r="E170" s="6"/>
-      <c r="F170" s="6"/>
+      <c r="F170" s="15"/>
       <c r="G170" s="6"/>
       <c r="H170" s="6"/>
       <c r="I170" s="6"/>
@@ -4955,7 +5142,7 @@
       <c r="C171" s="6"/>
       <c r="D171" s="6"/>
       <c r="E171" s="6"/>
-      <c r="F171" s="6"/>
+      <c r="F171" s="15"/>
       <c r="G171" s="6"/>
       <c r="H171" s="6"/>
       <c r="I171" s="6"/>
@@ -4972,7 +5159,7 @@
       <c r="C172" s="6"/>
       <c r="D172" s="6"/>
       <c r="E172" s="6"/>
-      <c r="F172" s="6"/>
+      <c r="F172" s="15"/>
       <c r="G172" s="6"/>
       <c r="H172" s="6"/>
       <c r="I172" s="6"/>
@@ -4989,7 +5176,7 @@
       <c r="C173" s="6"/>
       <c r="D173" s="6"/>
       <c r="E173" s="6"/>
-      <c r="F173" s="6"/>
+      <c r="F173" s="15"/>
       <c r="G173" s="6"/>
       <c r="H173" s="6"/>
       <c r="I173" s="6"/>
@@ -5006,7 +5193,7 @@
       <c r="C174" s="6"/>
       <c r="D174" s="6"/>
       <c r="E174" s="6"/>
-      <c r="F174" s="6"/>
+      <c r="F174" s="15"/>
       <c r="G174" s="6"/>
       <c r="H174" s="6"/>
       <c r="I174" s="6"/>
@@ -5023,7 +5210,7 @@
       <c r="C175" s="6"/>
       <c r="D175" s="6"/>
       <c r="E175" s="6"/>
-      <c r="F175" s="6"/>
+      <c r="F175" s="15"/>
       <c r="G175" s="6"/>
       <c r="H175" s="6"/>
       <c r="I175" s="6"/>
@@ -5040,7 +5227,7 @@
       <c r="C176" s="6"/>
       <c r="D176" s="6"/>
       <c r="E176" s="6"/>
-      <c r="F176" s="6"/>
+      <c r="F176" s="15"/>
       <c r="G176" s="6"/>
       <c r="H176" s="6"/>
       <c r="I176" s="6"/>
@@ -5057,7 +5244,7 @@
       <c r="C177" s="6"/>
       <c r="D177" s="6"/>
       <c r="E177" s="6"/>
-      <c r="F177" s="6"/>
+      <c r="F177" s="15"/>
       <c r="G177" s="6"/>
       <c r="H177" s="6"/>
       <c r="I177" s="6"/>
@@ -5074,7 +5261,7 @@
       <c r="C178" s="6"/>
       <c r="D178" s="6"/>
       <c r="E178" s="6"/>
-      <c r="F178" s="6"/>
+      <c r="F178" s="15"/>
       <c r="G178" s="6"/>
       <c r="H178" s="6"/>
       <c r="I178" s="6"/>
@@ -5091,7 +5278,7 @@
       <c r="C179" s="6"/>
       <c r="D179" s="6"/>
       <c r="E179" s="6"/>
-      <c r="F179" s="6"/>
+      <c r="F179" s="15"/>
       <c r="G179" s="6"/>
       <c r="H179" s="6"/>
       <c r="I179" s="6"/>
@@ -5108,7 +5295,7 @@
       <c r="C180" s="6"/>
       <c r="D180" s="6"/>
       <c r="E180" s="6"/>
-      <c r="F180" s="6"/>
+      <c r="F180" s="15"/>
       <c r="G180" s="6"/>
       <c r="H180" s="6"/>
       <c r="I180" s="6"/>
@@ -5125,7 +5312,7 @@
       <c r="C181" s="6"/>
       <c r="D181" s="6"/>
       <c r="E181" s="6"/>
-      <c r="F181" s="6"/>
+      <c r="F181" s="15"/>
       <c r="G181" s="6"/>
       <c r="H181" s="6"/>
       <c r="I181" s="6"/>
@@ -5142,7 +5329,7 @@
       <c r="C182" s="6"/>
       <c r="D182" s="6"/>
       <c r="E182" s="6"/>
-      <c r="F182" s="6"/>
+      <c r="F182" s="15"/>
       <c r="G182" s="6"/>
       <c r="H182" s="6"/>
       <c r="I182" s="6"/>
@@ -5159,7 +5346,7 @@
       <c r="C183" s="6"/>
       <c r="D183" s="6"/>
       <c r="E183" s="6"/>
-      <c r="F183" s="6"/>
+      <c r="F183" s="15"/>
       <c r="G183" s="6"/>
       <c r="H183" s="6"/>
       <c r="I183" s="6"/>
@@ -5176,7 +5363,7 @@
       <c r="C184" s="6"/>
       <c r="D184" s="6"/>
       <c r="E184" s="6"/>
-      <c r="F184" s="6"/>
+      <c r="F184" s="15"/>
       <c r="G184" s="6"/>
       <c r="H184" s="6"/>
       <c r="I184" s="6"/>
@@ -5193,7 +5380,7 @@
       <c r="C185" s="6"/>
       <c r="D185" s="6"/>
       <c r="E185" s="6"/>
-      <c r="F185" s="6"/>
+      <c r="F185" s="15"/>
       <c r="G185" s="6"/>
       <c r="H185" s="6"/>
       <c r="I185" s="6"/>
@@ -5210,7 +5397,7 @@
       <c r="C186" s="6"/>
       <c r="D186" s="6"/>
       <c r="E186" s="6"/>
-      <c r="F186" s="6"/>
+      <c r="F186" s="15"/>
       <c r="G186" s="6"/>
       <c r="H186" s="6"/>
       <c r="I186" s="6"/>
@@ -5227,7 +5414,7 @@
       <c r="C187" s="6"/>
       <c r="D187" s="6"/>
       <c r="E187" s="6"/>
-      <c r="F187" s="6"/>
+      <c r="F187" s="15"/>
       <c r="G187" s="6"/>
       <c r="H187" s="6"/>
       <c r="I187" s="6"/>
@@ -5244,7 +5431,7 @@
       <c r="C188" s="6"/>
       <c r="D188" s="6"/>
       <c r="E188" s="6"/>
-      <c r="F188" s="6"/>
+      <c r="F188" s="15"/>
       <c r="G188" s="6"/>
       <c r="H188" s="6"/>
       <c r="I188" s="6"/>
@@ -5261,7 +5448,7 @@
       <c r="C189" s="6"/>
       <c r="D189" s="6"/>
       <c r="E189" s="6"/>
-      <c r="F189" s="6"/>
+      <c r="F189" s="15"/>
       <c r="G189" s="6"/>
       <c r="H189" s="6"/>
       <c r="I189" s="6"/>
@@ -5278,7 +5465,7 @@
       <c r="C190" s="6"/>
       <c r="D190" s="6"/>
       <c r="E190" s="6"/>
-      <c r="F190" s="6"/>
+      <c r="F190" s="15"/>
       <c r="G190" s="6"/>
       <c r="H190" s="6"/>
       <c r="I190" s="6"/>
@@ -5295,7 +5482,7 @@
       <c r="C191" s="6"/>
       <c r="D191" s="6"/>
       <c r="E191" s="6"/>
-      <c r="F191" s="6"/>
+      <c r="F191" s="15"/>
       <c r="G191" s="6"/>
       <c r="H191" s="6"/>
       <c r="I191" s="6"/>
@@ -5312,7 +5499,7 @@
       <c r="C192" s="6"/>
       <c r="D192" s="6"/>
       <c r="E192" s="6"/>
-      <c r="F192" s="6"/>
+      <c r="F192" s="15"/>
       <c r="G192" s="6"/>
       <c r="H192" s="6"/>
       <c r="I192" s="6"/>
@@ -5329,7 +5516,7 @@
       <c r="C193" s="6"/>
       <c r="D193" s="6"/>
       <c r="E193" s="6"/>
-      <c r="F193" s="6"/>
+      <c r="F193" s="15"/>
       <c r="G193" s="6"/>
       <c r="H193" s="6"/>
       <c r="I193" s="6"/>
@@ -5346,7 +5533,7 @@
       <c r="C194" s="6"/>
       <c r="D194" s="6"/>
       <c r="E194" s="6"/>
-      <c r="F194" s="6"/>
+      <c r="F194" s="15"/>
       <c r="G194" s="6"/>
       <c r="H194" s="6"/>
       <c r="I194" s="6"/>
@@ -5363,7 +5550,7 @@
       <c r="C195" s="6"/>
       <c r="D195" s="6"/>
       <c r="E195" s="6"/>
-      <c r="F195" s="6"/>
+      <c r="F195" s="15"/>
       <c r="G195" s="6"/>
       <c r="H195" s="6"/>
       <c r="I195" s="6"/>
@@ -5380,7 +5567,7 @@
       <c r="C196" s="6"/>
       <c r="D196" s="6"/>
       <c r="E196" s="6"/>
-      <c r="F196" s="6"/>
+      <c r="F196" s="15"/>
       <c r="G196" s="6"/>
       <c r="H196" s="6"/>
       <c r="I196" s="6"/>
@@ -5397,7 +5584,7 @@
       <c r="C197" s="6"/>
       <c r="D197" s="6"/>
       <c r="E197" s="6"/>
-      <c r="F197" s="6"/>
+      <c r="F197" s="15"/>
       <c r="G197" s="6"/>
       <c r="H197" s="6"/>
       <c r="I197" s="6"/>
@@ -5414,7 +5601,7 @@
       <c r="C198" s="6"/>
       <c r="D198" s="6"/>
       <c r="E198" s="6"/>
-      <c r="F198" s="6"/>
+      <c r="F198" s="15"/>
       <c r="G198" s="6"/>
       <c r="H198" s="6"/>
       <c r="I198" s="6"/>
@@ -5431,7 +5618,7 @@
       <c r="C199" s="6"/>
       <c r="D199" s="6"/>
       <c r="E199" s="6"/>
-      <c r="F199" s="6"/>
+      <c r="F199" s="15"/>
       <c r="G199" s="6"/>
       <c r="H199" s="6"/>
       <c r="I199" s="6"/>
@@ -5448,7 +5635,7 @@
       <c r="C200" s="6"/>
       <c r="D200" s="6"/>
       <c r="E200" s="6"/>
-      <c r="F200" s="6"/>
+      <c r="F200" s="15"/>
       <c r="G200" s="6"/>
       <c r="H200" s="6"/>
       <c r="I200" s="6"/>
@@ -5465,7 +5652,7 @@
       <c r="C201" s="6"/>
       <c r="D201" s="6"/>
       <c r="E201" s="6"/>
-      <c r="F201" s="6"/>
+      <c r="F201" s="15"/>
       <c r="G201" s="6"/>
       <c r="H201" s="6"/>
       <c r="I201" s="6"/>
@@ -5482,7 +5669,7 @@
       <c r="C202" s="6"/>
       <c r="D202" s="6"/>
       <c r="E202" s="6"/>
-      <c r="F202" s="6"/>
+      <c r="F202" s="15"/>
       <c r="G202" s="6"/>
       <c r="H202" s="6"/>
       <c r="I202" s="6"/>
@@ -5499,7 +5686,7 @@
       <c r="C203" s="6"/>
       <c r="D203" s="6"/>
       <c r="E203" s="6"/>
-      <c r="F203" s="6"/>
+      <c r="F203" s="15"/>
       <c r="G203" s="6"/>
       <c r="H203" s="6"/>
       <c r="I203" s="6"/>
@@ -5516,7 +5703,7 @@
       <c r="C204" s="6"/>
       <c r="D204" s="6"/>
       <c r="E204" s="6"/>
-      <c r="F204" s="6"/>
+      <c r="F204" s="15"/>
       <c r="G204" s="6"/>
       <c r="H204" s="6"/>
       <c r="I204" s="6"/>
@@ -5533,7 +5720,7 @@
       <c r="C205" s="6"/>
       <c r="D205" s="6"/>
       <c r="E205" s="6"/>
-      <c r="F205" s="6"/>
+      <c r="F205" s="15"/>
       <c r="G205" s="6"/>
       <c r="H205" s="6"/>
       <c r="I205" s="6"/>
@@ -5550,7 +5737,7 @@
       <c r="C206" s="6"/>
       <c r="D206" s="6"/>
       <c r="E206" s="6"/>
-      <c r="F206" s="6"/>
+      <c r="F206" s="15"/>
       <c r="G206" s="6"/>
       <c r="H206" s="6"/>
       <c r="I206" s="6"/>
@@ -5567,7 +5754,7 @@
       <c r="C207" s="6"/>
       <c r="D207" s="6"/>
       <c r="E207" s="6"/>
-      <c r="F207" s="6"/>
+      <c r="F207" s="15"/>
       <c r="G207" s="6"/>
       <c r="H207" s="6"/>
       <c r="I207" s="6"/>
@@ -5584,7 +5771,7 @@
       <c r="C208" s="6"/>
       <c r="D208" s="6"/>
       <c r="E208" s="6"/>
-      <c r="F208" s="6"/>
+      <c r="F208" s="15"/>
       <c r="G208" s="6"/>
       <c r="H208" s="6"/>
       <c r="I208" s="6"/>
@@ -5601,7 +5788,7 @@
       <c r="C209" s="6"/>
       <c r="D209" s="6"/>
       <c r="E209" s="6"/>
-      <c r="F209" s="6"/>
+      <c r="F209" s="15"/>
       <c r="G209" s="6"/>
       <c r="H209" s="6"/>
       <c r="I209" s="6"/>
@@ -5618,7 +5805,7 @@
       <c r="C210" s="6"/>
       <c r="D210" s="6"/>
       <c r="E210" s="6"/>
-      <c r="F210" s="6"/>
+      <c r="F210" s="15"/>
       <c r="G210" s="6"/>
       <c r="H210" s="6"/>
       <c r="I210" s="6"/>
@@ -5635,7 +5822,7 @@
       <c r="C211" s="6"/>
       <c r="D211" s="6"/>
       <c r="E211" s="6"/>
-      <c r="F211" s="6"/>
+      <c r="F211" s="15"/>
       <c r="G211" s="6"/>
       <c r="H211" s="6"/>
       <c r="I211" s="6"/>
@@ -5652,7 +5839,7 @@
       <c r="C212" s="6"/>
       <c r="D212" s="6"/>
       <c r="E212" s="6"/>
-      <c r="F212" s="6"/>
+      <c r="F212" s="15"/>
       <c r="G212" s="6"/>
       <c r="H212" s="6"/>
       <c r="I212" s="6"/>
@@ -5669,7 +5856,7 @@
       <c r="C213" s="6"/>
       <c r="D213" s="6"/>
       <c r="E213" s="6"/>
-      <c r="F213" s="6"/>
+      <c r="F213" s="15"/>
       <c r="G213" s="6"/>
       <c r="H213" s="6"/>
       <c r="I213" s="6"/>
@@ -5686,7 +5873,7 @@
       <c r="C214" s="6"/>
       <c r="D214" s="6"/>
       <c r="E214" s="6"/>
-      <c r="F214" s="6"/>
+      <c r="F214" s="15"/>
       <c r="G214" s="6"/>
       <c r="H214" s="6"/>
       <c r="I214" s="6"/>
@@ -5703,7 +5890,7 @@
       <c r="C215" s="6"/>
       <c r="D215" s="6"/>
       <c r="E215" s="6"/>
-      <c r="F215" s="6"/>
+      <c r="F215" s="15"/>
       <c r="G215" s="6"/>
       <c r="H215" s="6"/>
       <c r="I215" s="6"/>
@@ -5720,7 +5907,7 @@
       <c r="C216" s="6"/>
       <c r="D216" s="6"/>
       <c r="E216" s="6"/>
-      <c r="F216" s="6"/>
+      <c r="F216" s="15"/>
       <c r="G216" s="6"/>
       <c r="H216" s="6"/>
       <c r="I216" s="6"/>
@@ -5737,7 +5924,7 @@
       <c r="C217" s="6"/>
       <c r="D217" s="6"/>
       <c r="E217" s="6"/>
-      <c r="F217" s="6"/>
+      <c r="F217" s="15"/>
       <c r="G217" s="6"/>
       <c r="H217" s="6"/>
       <c r="I217" s="6"/>
@@ -5754,7 +5941,7 @@
       <c r="C218" s="6"/>
       <c r="D218" s="6"/>
       <c r="E218" s="6"/>
-      <c r="F218" s="6"/>
+      <c r="F218" s="15"/>
       <c r="G218" s="6"/>
       <c r="H218" s="6"/>
       <c r="I218" s="6"/>
@@ -5771,7 +5958,7 @@
       <c r="C219" s="6"/>
       <c r="D219" s="6"/>
       <c r="E219" s="6"/>
-      <c r="F219" s="6"/>
+      <c r="F219" s="15"/>
       <c r="G219" s="6"/>
       <c r="H219" s="6"/>
       <c r="I219" s="6"/>
@@ -5788,7 +5975,7 @@
       <c r="C220" s="6"/>
       <c r="D220" s="6"/>
       <c r="E220" s="6"/>
-      <c r="F220" s="6"/>
+      <c r="F220" s="15"/>
       <c r="G220" s="6"/>
       <c r="H220" s="6"/>
       <c r="I220" s="6"/>
@@ -5805,7 +5992,7 @@
       <c r="C221" s="6"/>
       <c r="D221" s="6"/>
       <c r="E221" s="6"/>
-      <c r="F221" s="6"/>
+      <c r="F221" s="15"/>
       <c r="G221" s="6"/>
       <c r="H221" s="6"/>
       <c r="I221" s="6"/>
@@ -5822,7 +6009,7 @@
       <c r="C222" s="6"/>
       <c r="D222" s="6"/>
       <c r="E222" s="6"/>
-      <c r="F222" s="6"/>
+      <c r="F222" s="15"/>
       <c r="G222" s="6"/>
       <c r="H222" s="6"/>
       <c r="I222" s="6"/>
@@ -5839,7 +6026,7 @@
       <c r="C223" s="6"/>
       <c r="D223" s="6"/>
       <c r="E223" s="6"/>
-      <c r="F223" s="6"/>
+      <c r="F223" s="15"/>
       <c r="G223" s="6"/>
       <c r="H223" s="6"/>
       <c r="I223" s="6"/>
@@ -5856,7 +6043,7 @@
       <c r="C224" s="6"/>
       <c r="D224" s="6"/>
       <c r="E224" s="6"/>
-      <c r="F224" s="6"/>
+      <c r="F224" s="15"/>
       <c r="G224" s="6"/>
       <c r="H224" s="6"/>
       <c r="I224" s="6"/>
@@ -5873,7 +6060,7 @@
       <c r="C225" s="6"/>
       <c r="D225" s="6"/>
       <c r="E225" s="6"/>
-      <c r="F225" s="6"/>
+      <c r="F225" s="15"/>
       <c r="G225" s="6"/>
       <c r="H225" s="6"/>
       <c r="I225" s="6"/>
@@ -5890,7 +6077,7 @@
       <c r="C226" s="6"/>
       <c r="D226" s="6"/>
       <c r="E226" s="6"/>
-      <c r="F226" s="6"/>
+      <c r="F226" s="15"/>
       <c r="G226" s="6"/>
       <c r="H226" s="6"/>
       <c r="I226" s="6"/>
@@ -5907,7 +6094,7 @@
       <c r="C227" s="6"/>
       <c r="D227" s="6"/>
       <c r="E227" s="6"/>
-      <c r="F227" s="6"/>
+      <c r="F227" s="15"/>
       <c r="G227" s="6"/>
       <c r="H227" s="6"/>
       <c r="I227" s="6"/>
@@ -5924,7 +6111,7 @@
       <c r="C228" s="6"/>
       <c r="D228" s="6"/>
       <c r="E228" s="6"/>
-      <c r="F228" s="6"/>
+      <c r="F228" s="15"/>
       <c r="G228" s="6"/>
       <c r="H228" s="6"/>
       <c r="I228" s="6"/>
@@ -5941,7 +6128,7 @@
       <c r="C229" s="6"/>
       <c r="D229" s="6"/>
       <c r="E229" s="6"/>
-      <c r="F229" s="6"/>
+      <c r="F229" s="15"/>
       <c r="G229" s="6"/>
       <c r="H229" s="6"/>
       <c r="I229" s="6"/>
@@ -5958,7 +6145,7 @@
       <c r="C230" s="6"/>
       <c r="D230" s="6"/>
       <c r="E230" s="6"/>
-      <c r="F230" s="6"/>
+      <c r="F230" s="15"/>
       <c r="G230" s="6"/>
       <c r="H230" s="6"/>
       <c r="I230" s="6"/>
@@ -5975,7 +6162,7 @@
       <c r="C231" s="6"/>
       <c r="D231" s="6"/>
       <c r="E231" s="6"/>
-      <c r="F231" s="6"/>
+      <c r="F231" s="15"/>
       <c r="G231" s="6"/>
       <c r="H231" s="6"/>
       <c r="I231" s="6"/>
@@ -5992,7 +6179,7 @@
       <c r="C232" s="6"/>
       <c r="D232" s="6"/>
       <c r="E232" s="6"/>
-      <c r="F232" s="6"/>
+      <c r="F232" s="15"/>
       <c r="G232" s="6"/>
       <c r="H232" s="6"/>
       <c r="I232" s="6"/>
@@ -6009,7 +6196,7 @@
       <c r="C233" s="6"/>
       <c r="D233" s="6"/>
       <c r="E233" s="6"/>
-      <c r="F233" s="6"/>
+      <c r="F233" s="15"/>
       <c r="G233" s="6"/>
       <c r="H233" s="6"/>
       <c r="I233" s="6"/>
@@ -6026,7 +6213,7 @@
       <c r="C234" s="6"/>
       <c r="D234" s="6"/>
       <c r="E234" s="6"/>
-      <c r="F234" s="6"/>
+      <c r="F234" s="15"/>
       <c r="G234" s="6"/>
       <c r="H234" s="6"/>
       <c r="I234" s="6"/>
@@ -6043,7 +6230,7 @@
       <c r="C235" s="6"/>
       <c r="D235" s="6"/>
       <c r="E235" s="6"/>
-      <c r="F235" s="6"/>
+      <c r="F235" s="15"/>
       <c r="G235" s="6"/>
       <c r="H235" s="6"/>
       <c r="I235" s="6"/>
@@ -6060,7 +6247,7 @@
       <c r="C236" s="6"/>
       <c r="D236" s="6"/>
       <c r="E236" s="6"/>
-      <c r="F236" s="6"/>
+      <c r="F236" s="15"/>
       <c r="G236" s="6"/>
       <c r="H236" s="6"/>
       <c r="I236" s="6"/>
@@ -6077,7 +6264,7 @@
       <c r="C237" s="6"/>
       <c r="D237" s="6"/>
       <c r="E237" s="6"/>
-      <c r="F237" s="6"/>
+      <c r="F237" s="15"/>
       <c r="G237" s="6"/>
       <c r="H237" s="6"/>
       <c r="I237" s="6"/>
@@ -6094,7 +6281,7 @@
       <c r="C238" s="6"/>
       <c r="D238" s="6"/>
       <c r="E238" s="6"/>
-      <c r="F238" s="6"/>
+      <c r="F238" s="15"/>
       <c r="G238" s="6"/>
       <c r="H238" s="6"/>
       <c r="I238" s="6"/>
@@ -6111,7 +6298,7 @@
       <c r="C239" s="6"/>
       <c r="D239" s="6"/>
       <c r="E239" s="6"/>
-      <c r="F239" s="6"/>
+      <c r="F239" s="15"/>
       <c r="G239" s="6"/>
       <c r="H239" s="6"/>
       <c r="I239" s="6"/>
@@ -6128,7 +6315,7 @@
       <c r="C240" s="6"/>
       <c r="D240" s="6"/>
       <c r="E240" s="6"/>
-      <c r="F240" s="6"/>
+      <c r="F240" s="15"/>
       <c r="G240" s="6"/>
       <c r="H240" s="6"/>
       <c r="I240" s="6"/>
@@ -6145,7 +6332,7 @@
       <c r="C241" s="6"/>
       <c r="D241" s="6"/>
       <c r="E241" s="6"/>
-      <c r="F241" s="6"/>
+      <c r="F241" s="15"/>
       <c r="G241" s="6"/>
       <c r="H241" s="6"/>
       <c r="I241" s="6"/>
@@ -6162,7 +6349,7 @@
       <c r="C242" s="6"/>
       <c r="D242" s="6"/>
       <c r="E242" s="6"/>
-      <c r="F242" s="6"/>
+      <c r="F242" s="15"/>
       <c r="G242" s="6"/>
       <c r="H242" s="6"/>
       <c r="I242" s="6"/>
@@ -6179,7 +6366,7 @@
       <c r="C243" s="6"/>
       <c r="D243" s="6"/>
       <c r="E243" s="6"/>
-      <c r="F243" s="6"/>
+      <c r="F243" s="15"/>
       <c r="G243" s="6"/>
       <c r="H243" s="6"/>
       <c r="I243" s="6"/>
@@ -6196,7 +6383,7 @@
       <c r="C244" s="6"/>
       <c r="D244" s="6"/>
       <c r="E244" s="6"/>
-      <c r="F244" s="6"/>
+      <c r="F244" s="15"/>
       <c r="G244" s="6"/>
       <c r="H244" s="6"/>
       <c r="I244" s="6"/>
@@ -6213,7 +6400,7 @@
       <c r="C245" s="6"/>
       <c r="D245" s="6"/>
       <c r="E245" s="6"/>
-      <c r="F245" s="6"/>
+      <c r="F245" s="15"/>
       <c r="G245" s="6"/>
       <c r="H245" s="6"/>
       <c r="I245" s="6"/>
@@ -6230,7 +6417,7 @@
       <c r="C246" s="6"/>
       <c r="D246" s="6"/>
       <c r="E246" s="6"/>
-      <c r="F246" s="6"/>
+      <c r="F246" s="15"/>
       <c r="G246" s="6"/>
       <c r="H246" s="6"/>
       <c r="I246" s="6"/>
@@ -6247,7 +6434,7 @@
       <c r="C247" s="6"/>
       <c r="D247" s="6"/>
       <c r="E247" s="6"/>
-      <c r="F247" s="6"/>
+      <c r="F247" s="15"/>
       <c r="G247" s="6"/>
       <c r="H247" s="6"/>
       <c r="I247" s="6"/>
@@ -6264,7 +6451,7 @@
       <c r="C248" s="6"/>
       <c r="D248" s="6"/>
       <c r="E248" s="6"/>
-      <c r="F248" s="6"/>
+      <c r="F248" s="15"/>
       <c r="G248" s="6"/>
       <c r="H248" s="6"/>
       <c r="I248" s="6"/>
@@ -6281,7 +6468,7 @@
       <c r="C249" s="6"/>
       <c r="D249" s="6"/>
       <c r="E249" s="6"/>
-      <c r="F249" s="6"/>
+      <c r="F249" s="15"/>
       <c r="G249" s="6"/>
       <c r="H249" s="6"/>
       <c r="I249" s="6"/>
@@ -6298,7 +6485,7 @@
       <c r="C250" s="6"/>
       <c r="D250" s="6"/>
       <c r="E250" s="6"/>
-      <c r="F250" s="6"/>
+      <c r="F250" s="15"/>
       <c r="G250" s="6"/>
       <c r="H250" s="6"/>
       <c r="I250" s="6"/>
@@ -6315,7 +6502,7 @@
       <c r="C251" s="6"/>
       <c r="D251" s="6"/>
       <c r="E251" s="6"/>
-      <c r="F251" s="6"/>
+      <c r="F251" s="15"/>
       <c r="G251" s="6"/>
       <c r="H251" s="6"/>
       <c r="I251" s="6"/>
@@ -6332,7 +6519,7 @@
       <c r="C252" s="6"/>
       <c r="D252" s="6"/>
       <c r="E252" s="6"/>
-      <c r="F252" s="6"/>
+      <c r="F252" s="15"/>
       <c r="G252" s="6"/>
       <c r="H252" s="6"/>
       <c r="I252" s="6"/>
@@ -6349,7 +6536,7 @@
       <c r="C253" s="6"/>
       <c r="D253" s="6"/>
       <c r="E253" s="6"/>
-      <c r="F253" s="6"/>
+      <c r="F253" s="15"/>
       <c r="G253" s="6"/>
       <c r="H253" s="6"/>
       <c r="I253" s="6"/>
@@ -6366,7 +6553,7 @@
       <c r="C254" s="6"/>
       <c r="D254" s="6"/>
       <c r="E254" s="6"/>
-      <c r="F254" s="6"/>
+      <c r="F254" s="15"/>
       <c r="G254" s="6"/>
       <c r="H254" s="6"/>
       <c r="I254" s="6"/>
@@ -6383,7 +6570,7 @@
       <c r="C255" s="6"/>
       <c r="D255" s="6"/>
       <c r="E255" s="6"/>
-      <c r="F255" s="6"/>
+      <c r="F255" s="15"/>
       <c r="G255" s="6"/>
       <c r="H255" s="6"/>
       <c r="I255" s="6"/>
@@ -6400,7 +6587,7 @@
       <c r="C256" s="6"/>
       <c r="D256" s="6"/>
       <c r="E256" s="6"/>
-      <c r="F256" s="6"/>
+      <c r="F256" s="15"/>
       <c r="G256" s="6"/>
       <c r="H256" s="6"/>
       <c r="I256" s="6"/>
@@ -6417,7 +6604,7 @@
       <c r="C257" s="6"/>
       <c r="D257" s="6"/>
       <c r="E257" s="6"/>
-      <c r="F257" s="6"/>
+      <c r="F257" s="15"/>
       <c r="G257" s="6"/>
       <c r="H257" s="6"/>
       <c r="I257" s="6"/>
@@ -6434,7 +6621,7 @@
       <c r="C258" s="6"/>
       <c r="D258" s="6"/>
       <c r="E258" s="6"/>
-      <c r="F258" s="6"/>
+      <c r="F258" s="15"/>
       <c r="G258" s="6"/>
       <c r="H258" s="6"/>
       <c r="I258" s="6"/>
@@ -6451,7 +6638,7 @@
       <c r="C259" s="6"/>
       <c r="D259" s="6"/>
       <c r="E259" s="6"/>
-      <c r="F259" s="6"/>
+      <c r="F259" s="15"/>
       <c r="G259" s="6"/>
       <c r="H259" s="6"/>
       <c r="I259" s="6"/>
@@ -6468,7 +6655,7 @@
       <c r="C260" s="6"/>
       <c r="D260" s="6"/>
       <c r="E260" s="6"/>
-      <c r="F260" s="6"/>
+      <c r="F260" s="15"/>
       <c r="G260" s="6"/>
       <c r="H260" s="6"/>
       <c r="I260" s="6"/>
@@ -6485,7 +6672,7 @@
       <c r="C261" s="6"/>
       <c r="D261" s="6"/>
       <c r="E261" s="6"/>
-      <c r="F261" s="6"/>
+      <c r="F261" s="15"/>
       <c r="G261" s="6"/>
       <c r="H261" s="6"/>
       <c r="I261" s="6"/>
@@ -6502,7 +6689,7 @@
       <c r="C262" s="6"/>
       <c r="D262" s="6"/>
       <c r="E262" s="6"/>
-      <c r="F262" s="6"/>
+      <c r="F262" s="15"/>
       <c r="G262" s="6"/>
       <c r="H262" s="6"/>
       <c r="I262" s="6"/>
@@ -6519,7 +6706,7 @@
       <c r="C263" s="6"/>
       <c r="D263" s="6"/>
       <c r="E263" s="6"/>
-      <c r="F263" s="6"/>
+      <c r="F263" s="15"/>
       <c r="G263" s="6"/>
       <c r="H263" s="6"/>
       <c r="I263" s="6"/>
@@ -6536,7 +6723,7 @@
       <c r="C264" s="6"/>
       <c r="D264" s="6"/>
       <c r="E264" s="6"/>
-      <c r="F264" s="6"/>
+      <c r="F264" s="15"/>
       <c r="G264" s="6"/>
       <c r="H264" s="6"/>
       <c r="I264" s="6"/>
@@ -6553,7 +6740,7 @@
       <c r="C265" s="6"/>
       <c r="D265" s="6"/>
       <c r="E265" s="6"/>
-      <c r="F265" s="6"/>
+      <c r="F265" s="15"/>
       <c r="G265" s="6"/>
       <c r="H265" s="6"/>
       <c r="I265" s="6"/>
@@ -6570,7 +6757,7 @@
       <c r="C266" s="6"/>
       <c r="D266" s="6"/>
       <c r="E266" s="6"/>
-      <c r="F266" s="6"/>
+      <c r="F266" s="15"/>
       <c r="G266" s="6"/>
       <c r="H266" s="6"/>
       <c r="I266" s="6"/>
@@ -6587,7 +6774,7 @@
       <c r="C267" s="6"/>
       <c r="D267" s="6"/>
       <c r="E267" s="6"/>
-      <c r="F267" s="6"/>
+      <c r="F267" s="15"/>
       <c r="G267" s="6"/>
       <c r="H267" s="6"/>
       <c r="I267" s="6"/>
@@ -6604,7 +6791,7 @@
       <c r="C268" s="6"/>
       <c r="D268" s="6"/>
       <c r="E268" s="6"/>
-      <c r="F268" s="6"/>
+      <c r="F268" s="15"/>
       <c r="G268" s="6"/>
       <c r="H268" s="6"/>
       <c r="I268" s="6"/>
@@ -6621,7 +6808,7 @@
       <c r="C269" s="6"/>
       <c r="D269" s="6"/>
       <c r="E269" s="6"/>
-      <c r="F269" s="6"/>
+      <c r="F269" s="15"/>
       <c r="G269" s="6"/>
       <c r="H269" s="6"/>
       <c r="I269" s="6"/>
@@ -6638,7 +6825,7 @@
       <c r="C270" s="6"/>
       <c r="D270" s="6"/>
       <c r="E270" s="6"/>
-      <c r="F270" s="6"/>
+      <c r="F270" s="15"/>
       <c r="G270" s="6"/>
       <c r="H270" s="6"/>
       <c r="I270" s="6"/>
@@ -6655,7 +6842,7 @@
       <c r="C271" s="6"/>
       <c r="D271" s="6"/>
       <c r="E271" s="6"/>
-      <c r="F271" s="6"/>
+      <c r="F271" s="15"/>
       <c r="G271" s="6"/>
       <c r="H271" s="6"/>
       <c r="I271" s="6"/>
@@ -6672,7 +6859,7 @@
       <c r="C272" s="6"/>
       <c r="D272" s="6"/>
       <c r="E272" s="6"/>
-      <c r="F272" s="6"/>
+      <c r="F272" s="15"/>
       <c r="G272" s="6"/>
       <c r="H272" s="6"/>
       <c r="I272" s="6"/>
@@ -6689,7 +6876,7 @@
       <c r="C273" s="6"/>
       <c r="D273" s="6"/>
       <c r="E273" s="6"/>
-      <c r="F273" s="6"/>
+      <c r="F273" s="15"/>
       <c r="G273" s="6"/>
       <c r="H273" s="6"/>
       <c r="I273" s="6"/>
@@ -6706,7 +6893,7 @@
       <c r="C274" s="6"/>
       <c r="D274" s="6"/>
       <c r="E274" s="6"/>
-      <c r="F274" s="6"/>
+      <c r="F274" s="15"/>
       <c r="G274" s="6"/>
       <c r="H274" s="6"/>
       <c r="I274" s="6"/>
@@ -6723,7 +6910,7 @@
       <c r="C275" s="6"/>
       <c r="D275" s="6"/>
       <c r="E275" s="6"/>
-      <c r="F275" s="6"/>
+      <c r="F275" s="15"/>
       <c r="G275" s="6"/>
       <c r="H275" s="6"/>
       <c r="I275" s="6"/>
@@ -6740,7 +6927,7 @@
       <c r="C276" s="6"/>
       <c r="D276" s="6"/>
       <c r="E276" s="6"/>
-      <c r="F276" s="6"/>
+      <c r="F276" s="15"/>
       <c r="G276" s="6"/>
       <c r="H276" s="6"/>
       <c r="I276" s="6"/>
@@ -6757,7 +6944,7 @@
       <c r="C277" s="6"/>
       <c r="D277" s="6"/>
       <c r="E277" s="6"/>
-      <c r="F277" s="6"/>
+      <c r="F277" s="15"/>
       <c r="G277" s="6"/>
       <c r="H277" s="6"/>
       <c r="I277" s="6"/>
@@ -6774,7 +6961,7 @@
       <c r="C278" s="6"/>
       <c r="D278" s="6"/>
       <c r="E278" s="6"/>
-      <c r="F278" s="6"/>
+      <c r="F278" s="15"/>
       <c r="G278" s="6"/>
       <c r="H278" s="6"/>
       <c r="I278" s="6"/>
@@ -6791,7 +6978,7 @@
       <c r="C279" s="6"/>
       <c r="D279" s="6"/>
       <c r="E279" s="6"/>
-      <c r="F279" s="6"/>
+      <c r="F279" s="15"/>
       <c r="G279" s="6"/>
       <c r="H279" s="6"/>
       <c r="I279" s="6"/>
@@ -6808,7 +6995,7 @@
       <c r="C280" s="6"/>
       <c r="D280" s="6"/>
       <c r="E280" s="6"/>
-      <c r="F280" s="6"/>
+      <c r="F280" s="15"/>
       <c r="G280" s="6"/>
       <c r="H280" s="6"/>
       <c r="I280" s="6"/>
@@ -6825,7 +7012,7 @@
       <c r="C281" s="6"/>
       <c r="D281" s="6"/>
       <c r="E281" s="6"/>
-      <c r="F281" s="6"/>
+      <c r="F281" s="15"/>
       <c r="G281" s="6"/>
       <c r="H281" s="6"/>
       <c r="I281" s="6"/>
@@ -6842,7 +7029,7 @@
       <c r="C282" s="6"/>
       <c r="D282" s="6"/>
       <c r="E282" s="6"/>
-      <c r="F282" s="6"/>
+      <c r="F282" s="15"/>
       <c r="G282" s="6"/>
       <c r="H282" s="6"/>
       <c r="I282" s="6"/>
@@ -6859,7 +7046,7 @@
       <c r="C283" s="6"/>
       <c r="D283" s="6"/>
       <c r="E283" s="6"/>
-      <c r="F283" s="6"/>
+      <c r="F283" s="15"/>
       <c r="G283" s="6"/>
       <c r="H283" s="6"/>
       <c r="I283" s="6"/>
@@ -6876,7 +7063,7 @@
       <c r="C284" s="6"/>
       <c r="D284" s="6"/>
       <c r="E284" s="6"/>
-      <c r="F284" s="6"/>
+      <c r="F284" s="15"/>
       <c r="G284" s="6"/>
       <c r="H284" s="6"/>
       <c r="I284" s="6"/>
@@ -6893,7 +7080,7 @@
       <c r="C285" s="6"/>
       <c r="D285" s="6"/>
       <c r="E285" s="6"/>
-      <c r="F285" s="6"/>
+      <c r="F285" s="15"/>
       <c r="G285" s="6"/>
       <c r="H285" s="6"/>
       <c r="I285" s="6"/>
@@ -6910,7 +7097,7 @@
       <c r="C286" s="6"/>
       <c r="D286" s="6"/>
       <c r="E286" s="6"/>
-      <c r="F286" s="6"/>
+      <c r="F286" s="15"/>
       <c r="G286" s="6"/>
       <c r="H286" s="6"/>
       <c r="I286" s="6"/>
@@ -6927,7 +7114,7 @@
       <c r="C287" s="6"/>
       <c r="D287" s="6"/>
       <c r="E287" s="6"/>
-      <c r="F287" s="6"/>
+      <c r="F287" s="15"/>
       <c r="G287" s="6"/>
       <c r="H287" s="6"/>
       <c r="I287" s="6"/>
@@ -6944,7 +7131,7 @@
       <c r="C288" s="6"/>
       <c r="D288" s="6"/>
       <c r="E288" s="6"/>
-      <c r="F288" s="6"/>
+      <c r="F288" s="15"/>
       <c r="G288" s="6"/>
       <c r="H288" s="6"/>
       <c r="I288" s="6"/>
@@ -6961,7 +7148,7 @@
       <c r="C289" s="6"/>
       <c r="D289" s="6"/>
       <c r="E289" s="6"/>
-      <c r="F289" s="6"/>
+      <c r="F289" s="15"/>
       <c r="G289" s="6"/>
       <c r="H289" s="6"/>
       <c r="I289" s="6"/>
@@ -6978,7 +7165,7 @@
       <c r="C290" s="6"/>
       <c r="D290" s="6"/>
       <c r="E290" s="6"/>
-      <c r="F290" s="6"/>
+      <c r="F290" s="15"/>
       <c r="G290" s="6"/>
       <c r="H290" s="6"/>
       <c r="I290" s="6"/>
@@ -6995,7 +7182,7 @@
       <c r="C291" s="6"/>
       <c r="D291" s="6"/>
       <c r="E291" s="6"/>
-      <c r="F291" s="6"/>
+      <c r="F291" s="15"/>
       <c r="G291" s="6"/>
       <c r="H291" s="6"/>
       <c r="I291" s="6"/>
@@ -7012,7 +7199,7 @@
       <c r="C292" s="6"/>
       <c r="D292" s="6"/>
       <c r="E292" s="6"/>
-      <c r="F292" s="6"/>
+      <c r="F292" s="15"/>
       <c r="G292" s="6"/>
       <c r="H292" s="6"/>
       <c r="I292" s="6"/>
@@ -7029,7 +7216,7 @@
       <c r="C293" s="6"/>
       <c r="D293" s="6"/>
       <c r="E293" s="6"/>
-      <c r="F293" s="6"/>
+      <c r="F293" s="15"/>
       <c r="G293" s="6"/>
       <c r="H293" s="6"/>
       <c r="I293" s="6"/>
@@ -7046,7 +7233,7 @@
       <c r="C294" s="6"/>
       <c r="D294" s="6"/>
       <c r="E294" s="6"/>
-      <c r="F294" s="6"/>
+      <c r="F294" s="15"/>
       <c r="G294" s="6"/>
       <c r="H294" s="6"/>
       <c r="I294" s="6"/>
@@ -7063,7 +7250,7 @@
       <c r="C295" s="6"/>
       <c r="D295" s="6"/>
       <c r="E295" s="6"/>
-      <c r="F295" s="6"/>
+      <c r="F295" s="15"/>
       <c r="G295" s="6"/>
       <c r="H295" s="6"/>
       <c r="I295" s="6"/>
@@ -7080,7 +7267,7 @@
       <c r="C296" s="6"/>
       <c r="D296" s="6"/>
       <c r="E296" s="6"/>
-      <c r="F296" s="6"/>
+      <c r="F296" s="15"/>
       <c r="G296" s="6"/>
       <c r="H296" s="6"/>
       <c r="I296" s="6"/>
@@ -7097,7 +7284,7 @@
       <c r="C297" s="6"/>
       <c r="D297" s="6"/>
       <c r="E297" s="6"/>
-      <c r="F297" s="6"/>
+      <c r="F297" s="15"/>
       <c r="G297" s="6"/>
       <c r="H297" s="6"/>
       <c r="I297" s="6"/>
@@ -7114,7 +7301,7 @@
       <c r="C298" s="6"/>
       <c r="D298" s="6"/>
       <c r="E298" s="6"/>
-      <c r="F298" s="6"/>
+      <c r="F298" s="15"/>
       <c r="G298" s="6"/>
       <c r="H298" s="6"/>
       <c r="I298" s="6"/>
@@ -7131,7 +7318,7 @@
       <c r="C299" s="6"/>
       <c r="D299" s="6"/>
       <c r="E299" s="6"/>
-      <c r="F299" s="6"/>
+      <c r="F299" s="15"/>
       <c r="G299" s="6"/>
       <c r="H299" s="6"/>
       <c r="I299" s="6"/>
@@ -7148,7 +7335,7 @@
       <c r="C300" s="6"/>
       <c r="D300" s="6"/>
       <c r="E300" s="6"/>
-      <c r="F300" s="6"/>
+      <c r="F300" s="15"/>
       <c r="G300" s="6"/>
       <c r="H300" s="6"/>
       <c r="I300" s="6"/>
@@ -7165,7 +7352,7 @@
       <c r="C301" s="6"/>
       <c r="D301" s="6"/>
       <c r="E301" s="6"/>
-      <c r="F301" s="6"/>
+      <c r="F301" s="15"/>
       <c r="G301" s="6"/>
       <c r="H301" s="6"/>
       <c r="I301" s="6"/>
@@ -7182,7 +7369,7 @@
       <c r="C302" s="6"/>
       <c r="D302" s="6"/>
       <c r="E302" s="6"/>
-      <c r="F302" s="6"/>
+      <c r="F302" s="15"/>
       <c r="G302" s="6"/>
       <c r="H302" s="6"/>
       <c r="I302" s="6"/>
@@ -7199,7 +7386,7 @@
       <c r="C303" s="6"/>
       <c r="D303" s="6"/>
       <c r="E303" s="6"/>
-      <c r="F303" s="6"/>
+      <c r="F303" s="15"/>
       <c r="G303" s="6"/>
       <c r="H303" s="6"/>
       <c r="I303" s="6"/>
@@ -7216,7 +7403,7 @@
       <c r="C304" s="6"/>
       <c r="D304" s="6"/>
       <c r="E304" s="6"/>
-      <c r="F304" s="6"/>
+      <c r="F304" s="15"/>
       <c r="G304" s="6"/>
       <c r="H304" s="6"/>
       <c r="I304" s="6"/>
@@ -7233,7 +7420,7 @@
       <c r="C305" s="6"/>
       <c r="D305" s="6"/>
       <c r="E305" s="6"/>
-      <c r="F305" s="6"/>
+      <c r="F305" s="15"/>
       <c r="G305" s="6"/>
       <c r="H305" s="6"/>
       <c r="I305" s="6"/>
@@ -7250,7 +7437,7 @@
       <c r="C306" s="6"/>
       <c r="D306" s="6"/>
       <c r="E306" s="6"/>
-      <c r="F306" s="6"/>
+      <c r="F306" s="15"/>
       <c r="G306" s="6"/>
       <c r="H306" s="6"/>
       <c r="I306" s="6"/>
@@ -7267,7 +7454,7 @@
       <c r="C307" s="6"/>
       <c r="D307" s="6"/>
       <c r="E307" s="6"/>
-      <c r="F307" s="6"/>
+      <c r="F307" s="15"/>
       <c r="G307" s="6"/>
       <c r="H307" s="6"/>
       <c r="I307" s="6"/>
@@ -7284,7 +7471,7 @@
       <c r="C308" s="6"/>
       <c r="D308" s="6"/>
       <c r="E308" s="6"/>
-      <c r="F308" s="6"/>
+      <c r="F308" s="15"/>
       <c r="G308" s="6"/>
       <c r="H308" s="6"/>
       <c r="I308" s="6"/>
@@ -7301,7 +7488,7 @@
       <c r="C309" s="6"/>
       <c r="D309" s="6"/>
       <c r="E309" s="6"/>
-      <c r="F309" s="6"/>
+      <c r="F309" s="15"/>
       <c r="G309" s="6"/>
       <c r="H309" s="6"/>
       <c r="I309" s="6"/>
@@ -7318,7 +7505,7 @@
       <c r="C310" s="6"/>
       <c r="D310" s="6"/>
       <c r="E310" s="6"/>
-      <c r="F310" s="6"/>
+      <c r="F310" s="15"/>
       <c r="G310" s="6"/>
       <c r="H310" s="6"/>
       <c r="I310" s="6"/>
@@ -7335,7 +7522,7 @@
       <c r="C311" s="6"/>
       <c r="D311" s="6"/>
       <c r="E311" s="6"/>
-      <c r="F311" s="6"/>
+      <c r="F311" s="15"/>
       <c r="G311" s="6"/>
       <c r="H311" s="6"/>
       <c r="I311" s="6"/>
@@ -7352,7 +7539,7 @@
       <c r="C312" s="6"/>
       <c r="D312" s="6"/>
       <c r="E312" s="6"/>
-      <c r="F312" s="6"/>
+      <c r="F312" s="15"/>
       <c r="G312" s="6"/>
       <c r="H312" s="6"/>
       <c r="I312" s="6"/>
@@ -7369,7 +7556,7 @@
       <c r="C313" s="6"/>
       <c r="D313" s="6"/>
       <c r="E313" s="6"/>
-      <c r="F313" s="6"/>
+      <c r="F313" s="15"/>
       <c r="G313" s="6"/>
       <c r="H313" s="6"/>
       <c r="I313" s="6"/>
@@ -7386,7 +7573,7 @@
       <c r="C314" s="6"/>
       <c r="D314" s="6"/>
       <c r="E314" s="6"/>
-      <c r="F314" s="6"/>
+      <c r="F314" s="15"/>
       <c r="G314" s="6"/>
       <c r="H314" s="6"/>
       <c r="I314" s="6"/>
@@ -7403,7 +7590,7 @@
       <c r="C315" s="6"/>
       <c r="D315" s="6"/>
       <c r="E315" s="6"/>
-      <c r="F315" s="6"/>
+      <c r="F315" s="15"/>
       <c r="G315" s="6"/>
       <c r="H315" s="6"/>
       <c r="I315" s="6"/>
@@ -7420,7 +7607,7 @@
       <c r="C316" s="6"/>
       <c r="D316" s="6"/>
       <c r="E316" s="6"/>
-      <c r="F316" s="6"/>
+      <c r="F316" s="15"/>
       <c r="G316" s="6"/>
       <c r="H316" s="6"/>
       <c r="I316" s="6"/>
@@ -7437,7 +7624,7 @@
       <c r="C317" s="6"/>
       <c r="D317" s="6"/>
       <c r="E317" s="6"/>
-      <c r="F317" s="6"/>
+      <c r="F317" s="15"/>
       <c r="G317" s="6"/>
       <c r="H317" s="6"/>
       <c r="I317" s="6"/>
@@ -7454,7 +7641,7 @@
       <c r="C318" s="6"/>
       <c r="D318" s="6"/>
       <c r="E318" s="6"/>
-      <c r="F318" s="6"/>
+      <c r="F318" s="15"/>
       <c r="G318" s="6"/>
       <c r="H318" s="6"/>
       <c r="I318" s="6"/>
@@ -7471,7 +7658,7 @@
       <c r="C319" s="6"/>
       <c r="D319" s="6"/>
       <c r="E319" s="6"/>
-      <c r="F319" s="6"/>
+      <c r="F319" s="15"/>
       <c r="G319" s="6"/>
       <c r="H319" s="6"/>
       <c r="I319" s="6"/>
@@ -7488,7 +7675,7 @@
       <c r="C320" s="6"/>
       <c r="D320" s="6"/>
       <c r="E320" s="6"/>
-      <c r="F320" s="6"/>
+      <c r="F320" s="15"/>
       <c r="G320" s="6"/>
       <c r="H320" s="6"/>
       <c r="I320" s="6"/>
@@ -7505,7 +7692,7 @@
       <c r="C321" s="6"/>
       <c r="D321" s="6"/>
       <c r="E321" s="6"/>
-      <c r="F321" s="6"/>
+      <c r="F321" s="15"/>
       <c r="G321" s="6"/>
       <c r="H321" s="6"/>
       <c r="I321" s="6"/>
@@ -7522,7 +7709,7 @@
       <c r="C322" s="6"/>
       <c r="D322" s="6"/>
       <c r="E322" s="6"/>
-      <c r="F322" s="6"/>
+      <c r="F322" s="15"/>
       <c r="G322" s="6"/>
       <c r="H322" s="6"/>
       <c r="I322" s="6"/>
@@ -7539,7 +7726,7 @@
       <c r="C323" s="6"/>
       <c r="D323" s="6"/>
       <c r="E323" s="6"/>
-      <c r="F323" s="6"/>
+      <c r="F323" s="15"/>
       <c r="G323" s="6"/>
       <c r="H323" s="6"/>
       <c r="I323" s="6"/>
@@ -7556,7 +7743,7 @@
       <c r="C324" s="6"/>
       <c r="D324" s="6"/>
       <c r="E324" s="6"/>
-      <c r="F324" s="6"/>
+      <c r="F324" s="15"/>
       <c r="G324" s="6"/>
       <c r="H324" s="6"/>
       <c r="I324" s="6"/>
@@ -7573,7 +7760,7 @@
       <c r="C325" s="6"/>
       <c r="D325" s="6"/>
       <c r="E325" s="6"/>
-      <c r="F325" s="6"/>
+      <c r="F325" s="15"/>
       <c r="G325" s="6"/>
       <c r="H325" s="6"/>
       <c r="I325" s="6"/>
@@ -7590,7 +7777,7 @@
       <c r="C326" s="6"/>
       <c r="D326" s="6"/>
       <c r="E326" s="6"/>
-      <c r="F326" s="6"/>
+      <c r="F326" s="15"/>
       <c r="G326" s="6"/>
       <c r="H326" s="6"/>
       <c r="I326" s="6"/>
@@ -7607,7 +7794,7 @@
       <c r="C327" s="6"/>
       <c r="D327" s="6"/>
       <c r="E327" s="6"/>
-      <c r="F327" s="6"/>
+      <c r="F327" s="15"/>
       <c r="G327" s="6"/>
       <c r="H327" s="6"/>
       <c r="I327" s="6"/>
@@ -7624,7 +7811,7 @@
       <c r="C328" s="6"/>
       <c r="D328" s="6"/>
       <c r="E328" s="6"/>
-      <c r="F328" s="6"/>
+      <c r="F328" s="15"/>
       <c r="G328" s="6"/>
       <c r="H328" s="6"/>
       <c r="I328" s="6"/>
@@ -7641,7 +7828,7 @@
       <c r="C329" s="6"/>
       <c r="D329" s="6"/>
       <c r="E329" s="6"/>
-      <c r="F329" s="6"/>
+      <c r="F329" s="15"/>
       <c r="G329" s="6"/>
       <c r="H329" s="6"/>
       <c r="I329" s="6"/>
@@ -7658,7 +7845,7 @@
       <c r="C330" s="6"/>
       <c r="D330" s="6"/>
       <c r="E330" s="6"/>
-      <c r="F330" s="6"/>
+      <c r="F330" s="15"/>
       <c r="G330" s="6"/>
       <c r="H330" s="6"/>
       <c r="I330" s="6"/>
@@ -7675,7 +7862,7 @@
       <c r="C331" s="6"/>
       <c r="D331" s="6"/>
       <c r="E331" s="6"/>
-      <c r="F331" s="6"/>
+      <c r="F331" s="15"/>
       <c r="G331" s="6"/>
       <c r="H331" s="6"/>
       <c r="I331" s="6"/>
@@ -7692,7 +7879,7 @@
       <c r="C332" s="6"/>
       <c r="D332" s="6"/>
       <c r="E332" s="6"/>
-      <c r="F332" s="6"/>
+      <c r="F332" s="15"/>
       <c r="G332" s="6"/>
       <c r="H332" s="6"/>
       <c r="I332" s="6"/>
@@ -7709,7 +7896,7 @@
       <c r="C333" s="6"/>
       <c r="D333" s="6"/>
       <c r="E333" s="6"/>
-      <c r="F333" s="6"/>
+      <c r="F333" s="15"/>
       <c r="G333" s="6"/>
       <c r="H333" s="6"/>
       <c r="I333" s="6"/>
@@ -7726,7 +7913,7 @@
       <c r="C334" s="6"/>
       <c r="D334" s="6"/>
       <c r="E334" s="6"/>
-      <c r="F334" s="6"/>
+      <c r="F334" s="15"/>
       <c r="G334" s="6"/>
       <c r="H334" s="6"/>
       <c r="I334" s="6"/>
@@ -7743,7 +7930,7 @@
       <c r="C335" s="6"/>
       <c r="D335" s="6"/>
       <c r="E335" s="6"/>
-      <c r="F335" s="6"/>
+      <c r="F335" s="15"/>
       <c r="G335" s="6"/>
       <c r="H335" s="6"/>
       <c r="I335" s="6"/>
@@ -7760,7 +7947,7 @@
       <c r="C336" s="6"/>
       <c r="D336" s="6"/>
       <c r="E336" s="6"/>
-      <c r="F336" s="6"/>
+      <c r="F336" s="15"/>
       <c r="G336" s="6"/>
       <c r="H336" s="6"/>
       <c r="I336" s="6"/>
@@ -7777,7 +7964,7 @@
       <c r="C337" s="6"/>
       <c r="D337" s="6"/>
       <c r="E337" s="6"/>
-      <c r="F337" s="6"/>
+      <c r="F337" s="15"/>
       <c r="G337" s="6"/>
       <c r="H337" s="6"/>
       <c r="I337" s="6"/>
@@ -7794,7 +7981,7 @@
       <c r="C338" s="6"/>
       <c r="D338" s="6"/>
       <c r="E338" s="6"/>
-      <c r="F338" s="6"/>
+      <c r="F338" s="15"/>
       <c r="G338" s="6"/>
       <c r="H338" s="6"/>
       <c r="I338" s="6"/>
@@ -7811,7 +7998,7 @@
       <c r="C339" s="6"/>
       <c r="D339" s="6"/>
       <c r="E339" s="6"/>
-      <c r="F339" s="6"/>
+      <c r="F339" s="15"/>
       <c r="G339" s="6"/>
       <c r="H339" s="6"/>
       <c r="I339" s="6"/>
@@ -7828,7 +8015,7 @@
       <c r="C340" s="6"/>
       <c r="D340" s="6"/>
       <c r="E340" s="6"/>
-      <c r="F340" s="6"/>
+      <c r="F340" s="15"/>
       <c r="G340" s="6"/>
       <c r="H340" s="6"/>
       <c r="I340" s="6"/>
@@ -7845,7 +8032,7 @@
       <c r="C341" s="6"/>
       <c r="D341" s="6"/>
       <c r="E341" s="6"/>
-      <c r="F341" s="6"/>
+      <c r="F341" s="15"/>
       <c r="G341" s="6"/>
       <c r="H341" s="6"/>
       <c r="I341" s="6"/>
@@ -7862,7 +8049,7 @@
       <c r="C342" s="6"/>
       <c r="D342" s="6"/>
       <c r="E342" s="6"/>
-      <c r="F342" s="6"/>
+      <c r="F342" s="15"/>
       <c r="G342" s="6"/>
       <c r="H342" s="6"/>
       <c r="I342" s="6"/>
@@ -7879,7 +8066,7 @@
       <c r="C343" s="6"/>
       <c r="D343" s="6"/>
       <c r="E343" s="6"/>
-      <c r="F343" s="6"/>
+      <c r="F343" s="15"/>
       <c r="G343" s="6"/>
       <c r="H343" s="6"/>
       <c r="I343" s="6"/>
@@ -7896,7 +8083,7 @@
       <c r="C344" s="6"/>
       <c r="D344" s="6"/>
       <c r="E344" s="6"/>
-      <c r="F344" s="6"/>
+      <c r="F344" s="15"/>
       <c r="G344" s="6"/>
       <c r="H344" s="6"/>
       <c r="I344" s="6"/>
@@ -7913,7 +8100,7 @@
       <c r="C345" s="6"/>
       <c r="D345" s="6"/>
       <c r="E345" s="6"/>
-      <c r="F345" s="6"/>
+      <c r="F345" s="15"/>
       <c r="G345" s="6"/>
       <c r="H345" s="6"/>
       <c r="I345" s="6"/>
@@ -7930,7 +8117,7 @@
       <c r="C346" s="6"/>
       <c r="D346" s="6"/>
       <c r="E346" s="6"/>
-      <c r="F346" s="6"/>
+      <c r="F346" s="15"/>
       <c r="G346" s="6"/>
       <c r="H346" s="6"/>
       <c r="I346" s="6"/>
@@ -7947,7 +8134,7 @@
       <c r="C347" s="6"/>
       <c r="D347" s="6"/>
       <c r="E347" s="6"/>
-      <c r="F347" s="6"/>
+      <c r="F347" s="15"/>
       <c r="G347" s="6"/>
       <c r="H347" s="6"/>
       <c r="I347" s="6"/>
@@ -7964,7 +8151,7 @@
       <c r="C348" s="6"/>
       <c r="D348" s="6"/>
       <c r="E348" s="6"/>
-      <c r="F348" s="6"/>
+      <c r="F348" s="15"/>
       <c r="G348" s="6"/>
       <c r="H348" s="6"/>
       <c r="I348" s="6"/>
@@ -7981,7 +8168,7 @@
       <c r="C349" s="6"/>
       <c r="D349" s="6"/>
       <c r="E349" s="6"/>
-      <c r="F349" s="6"/>
+      <c r="F349" s="15"/>
       <c r="G349" s="6"/>
       <c r="H349" s="6"/>
       <c r="I349" s="6"/>
@@ -7998,7 +8185,7 @@
       <c r="C350" s="6"/>
       <c r="D350" s="6"/>
       <c r="E350" s="6"/>
-      <c r="F350" s="6"/>
+      <c r="F350" s="15"/>
       <c r="G350" s="6"/>
       <c r="H350" s="6"/>
       <c r="I350" s="6"/>
@@ -8015,7 +8202,7 @@
       <c r="C351" s="6"/>
       <c r="D351" s="6"/>
       <c r="E351" s="6"/>
-      <c r="F351" s="6"/>
+      <c r="F351" s="15"/>
       <c r="G351" s="6"/>
       <c r="H351" s="6"/>
       <c r="I351" s="6"/>
@@ -8032,7 +8219,7 @@
       <c r="C352" s="6"/>
       <c r="D352" s="6"/>
       <c r="E352" s="6"/>
-      <c r="F352" s="6"/>
+      <c r="F352" s="15"/>
       <c r="G352" s="6"/>
       <c r="H352" s="6"/>
       <c r="I352" s="6"/>
@@ -8049,7 +8236,7 @@
       <c r="C353" s="6"/>
       <c r="D353" s="6"/>
       <c r="E353" s="6"/>
-      <c r="F353" s="6"/>
+      <c r="F353" s="15"/>
       <c r="G353" s="6"/>
       <c r="H353" s="6"/>
       <c r="I353" s="6"/>
@@ -8066,7 +8253,7 @@
       <c r="C354" s="6"/>
       <c r="D354" s="6"/>
       <c r="E354" s="6"/>
-      <c r="F354" s="6"/>
+      <c r="F354" s="15"/>
       <c r="G354" s="6"/>
       <c r="H354" s="6"/>
       <c r="I354" s="6"/>
@@ -8083,7 +8270,7 @@
       <c r="C355" s="6"/>
       <c r="D355" s="6"/>
       <c r="E355" s="6"/>
-      <c r="F355" s="6"/>
+      <c r="F355" s="15"/>
       <c r="G355" s="6"/>
       <c r="H355" s="6"/>
       <c r="I355" s="6"/>
@@ -8100,7 +8287,7 @@
       <c r="C356" s="6"/>
       <c r="D356" s="6"/>
       <c r="E356" s="6"/>
-      <c r="F356" s="6"/>
+      <c r="F356" s="15"/>
       <c r="G356" s="6"/>
       <c r="H356" s="6"/>
       <c r="I356" s="6"/>
@@ -8117,7 +8304,7 @@
       <c r="C357" s="6"/>
       <c r="D357" s="6"/>
       <c r="E357" s="6"/>
-      <c r="F357" s="6"/>
+      <c r="F357" s="15"/>
       <c r="G357" s="6"/>
       <c r="H357" s="6"/>
       <c r="I357" s="6"/>
@@ -8134,7 +8321,7 @@
       <c r="C358" s="6"/>
       <c r="D358" s="6"/>
       <c r="E358" s="6"/>
-      <c r="F358" s="6"/>
+      <c r="F358" s="15"/>
       <c r="G358" s="6"/>
       <c r="H358" s="6"/>
       <c r="I358" s="6"/>
@@ -8151,7 +8338,7 @@
       <c r="C359" s="6"/>
       <c r="D359" s="6"/>
       <c r="E359" s="6"/>
-      <c r="F359" s="6"/>
+      <c r="F359" s="15"/>
       <c r="G359" s="6"/>
       <c r="H359" s="6"/>
       <c r="I359" s="6"/>
@@ -8168,7 +8355,7 @@
       <c r="C360" s="6"/>
       <c r="D360" s="6"/>
       <c r="E360" s="6"/>
-      <c r="F360" s="6"/>
+      <c r="F360" s="15"/>
       <c r="G360" s="6"/>
       <c r="H360" s="6"/>
       <c r="I360" s="6"/>
@@ -8185,7 +8372,7 @@
       <c r="C361" s="6"/>
       <c r="D361" s="6"/>
       <c r="E361" s="6"/>
-      <c r="F361" s="6"/>
+      <c r="F361" s="15"/>
       <c r="G361" s="6"/>
       <c r="H361" s="6"/>
       <c r="I361" s="6"/>
@@ -8202,7 +8389,7 @@
       <c r="C362" s="6"/>
       <c r="D362" s="6"/>
       <c r="E362" s="6"/>
-      <c r="F362" s="6"/>
+      <c r="F362" s="15"/>
       <c r="G362" s="6"/>
       <c r="H362" s="6"/>
       <c r="I362" s="6"/>
@@ -8219,7 +8406,7 @@
       <c r="C363" s="6"/>
       <c r="D363" s="6"/>
       <c r="E363" s="6"/>
-      <c r="F363" s="6"/>
+      <c r="F363" s="15"/>
       <c r="G363" s="6"/>
       <c r="H363" s="6"/>
       <c r="I363" s="6"/>
@@ -8236,7 +8423,7 @@
       <c r="C364" s="6"/>
       <c r="D364" s="6"/>
       <c r="E364" s="6"/>
-      <c r="F364" s="6"/>
+      <c r="F364" s="15"/>
       <c r="G364" s="6"/>
       <c r="H364" s="6"/>
       <c r="I364" s="6"/>
@@ -8253,7 +8440,7 @@
       <c r="C365" s="6"/>
       <c r="D365" s="6"/>
       <c r="E365" s="6"/>
-      <c r="F365" s="6"/>
+      <c r="F365" s="15"/>
       <c r="G365" s="6"/>
       <c r="H365" s="6"/>
       <c r="I365" s="6"/>
@@ -8270,7 +8457,7 @@
       <c r="C366" s="6"/>
       <c r="D366" s="6"/>
       <c r="E366" s="6"/>
-      <c r="F366" s="6"/>
+      <c r="F366" s="15"/>
       <c r="G366" s="6"/>
       <c r="H366" s="6"/>
       <c r="I366" s="6"/>
@@ -8287,7 +8474,7 @@
       <c r="C367" s="6"/>
       <c r="D367" s="6"/>
       <c r="E367" s="6"/>
-      <c r="F367" s="6"/>
+      <c r="F367" s="15"/>
       <c r="G367" s="6"/>
       <c r="H367" s="6"/>
       <c r="I367" s="6"/>
@@ -8304,7 +8491,7 @@
       <c r="C368" s="6"/>
       <c r="D368" s="6"/>
       <c r="E368" s="6"/>
-      <c r="F368" s="6"/>
+      <c r="F368" s="15"/>
       <c r="G368" s="6"/>
       <c r="H368" s="6"/>
       <c r="I368" s="6"/>
@@ -8321,7 +8508,7 @@
       <c r="C369" s="6"/>
       <c r="D369" s="6"/>
       <c r="E369" s="6"/>
-      <c r="F369" s="6"/>
+      <c r="F369" s="15"/>
       <c r="G369" s="6"/>
       <c r="H369" s="6"/>
       <c r="I369" s="6"/>
@@ -8338,7 +8525,7 @@
       <c r="C370" s="6"/>
       <c r="D370" s="6"/>
       <c r="E370" s="6"/>
-      <c r="F370" s="6"/>
+      <c r="F370" s="15"/>
       <c r="G370" s="6"/>
       <c r="H370" s="6"/>
       <c r="I370" s="6"/>
@@ -8355,7 +8542,7 @@
       <c r="C371" s="6"/>
       <c r="D371" s="6"/>
       <c r="E371" s="6"/>
-      <c r="F371" s="6"/>
+      <c r="F371" s="15"/>
       <c r="G371" s="6"/>
       <c r="H371" s="6"/>
       <c r="I371" s="6"/>
@@ -8372,7 +8559,7 @@
       <c r="C372" s="6"/>
       <c r="D372" s="6"/>
       <c r="E372" s="6"/>
-      <c r="F372" s="6"/>
+      <c r="F372" s="15"/>
       <c r="G372" s="6"/>
       <c r="H372" s="6"/>
       <c r="I372" s="6"/>
@@ -8389,7 +8576,7 @@
       <c r="C373" s="6"/>
       <c r="D373" s="6"/>
       <c r="E373" s="6"/>
-      <c r="F373" s="6"/>
+      <c r="F373" s="15"/>
       <c r="G373" s="6"/>
       <c r="H373" s="6"/>
       <c r="I373" s="6"/>
@@ -8406,7 +8593,7 @@
       <c r="C374" s="6"/>
       <c r="D374" s="6"/>
       <c r="E374" s="6"/>
-      <c r="F374" s="6"/>
+      <c r="F374" s="15"/>
       <c r="G374" s="6"/>
       <c r="H374" s="6"/>
       <c r="I374" s="6"/>
@@ -8423,7 +8610,7 @@
       <c r="C375" s="6"/>
       <c r="D375" s="6"/>
       <c r="E375" s="6"/>
-      <c r="F375" s="6"/>
+      <c r="F375" s="15"/>
       <c r="G375" s="6"/>
       <c r="H375" s="6"/>
       <c r="I375" s="6"/>
@@ -8440,7 +8627,7 @@
       <c r="C376" s="6"/>
       <c r="D376" s="6"/>
       <c r="E376" s="6"/>
-      <c r="F376" s="6"/>
+      <c r="F376" s="15"/>
       <c r="G376" s="6"/>
       <c r="H376" s="6"/>
       <c r="I376" s="6"/>
@@ -8457,7 +8644,7 @@
       <c r="C377" s="6"/>
       <c r="D377" s="6"/>
       <c r="E377" s="6"/>
-      <c r="F377" s="6"/>
+      <c r="F377" s="15"/>
       <c r="G377" s="6"/>
       <c r="H377" s="6"/>
       <c r="I377" s="6"/>
@@ -8474,7 +8661,7 @@
       <c r="C378" s="6"/>
       <c r="D378" s="6"/>
       <c r="E378" s="6"/>
-      <c r="F378" s="6"/>
+      <c r="F378" s="15"/>
       <c r="G378" s="6"/>
       <c r="H378" s="6"/>
       <c r="I378" s="6"/>
@@ -8491,7 +8678,7 @@
       <c r="C379" s="6"/>
       <c r="D379" s="6"/>
       <c r="E379" s="6"/>
-      <c r="F379" s="6"/>
+      <c r="F379" s="15"/>
       <c r="G379" s="6"/>
       <c r="H379" s="6"/>
       <c r="I379" s="6"/>
@@ -8508,7 +8695,7 @@
       <c r="C380" s="6"/>
       <c r="D380" s="6"/>
       <c r="E380" s="6"/>
-      <c r="F380" s="6"/>
+      <c r="F380" s="15"/>
       <c r="G380" s="6"/>
       <c r="H380" s="6"/>
       <c r="I380" s="6"/>
@@ -8525,7 +8712,7 @@
       <c r="C381" s="6"/>
       <c r="D381" s="6"/>
       <c r="E381" s="6"/>
-      <c r="F381" s="6"/>
+      <c r="F381" s="15"/>
       <c r="G381" s="6"/>
       <c r="H381" s="6"/>
       <c r="I381" s="6"/>
@@ -8542,7 +8729,7 @@
       <c r="C382" s="6"/>
       <c r="D382" s="6"/>
       <c r="E382" s="6"/>
-      <c r="F382" s="6"/>
+      <c r="F382" s="15"/>
       <c r="G382" s="6"/>
       <c r="H382" s="6"/>
       <c r="I382" s="6"/>
@@ -8559,7 +8746,7 @@
       <c r="C383" s="6"/>
       <c r="D383" s="6"/>
       <c r="E383" s="6"/>
-      <c r="F383" s="6"/>
+      <c r="F383" s="15"/>
       <c r="G383" s="6"/>
       <c r="H383" s="6"/>
       <c r="I383" s="6"/>
@@ -8576,7 +8763,7 @@
       <c r="C384" s="6"/>
       <c r="D384" s="6"/>
       <c r="E384" s="6"/>
-      <c r="F384" s="6"/>
+      <c r="F384" s="15"/>
       <c r="G384" s="6"/>
       <c r="H384" s="6"/>
       <c r="I384" s="6"/>
@@ -8593,7 +8780,7 @@
       <c r="C385" s="6"/>
       <c r="D385" s="6"/>
       <c r="E385" s="6"/>
-      <c r="F385" s="6"/>
+      <c r="F385" s="15"/>
       <c r="G385" s="6"/>
       <c r="H385" s="6"/>
       <c r="I385" s="6"/>
@@ -8610,7 +8797,7 @@
       <c r="C386" s="6"/>
       <c r="D386" s="6"/>
       <c r="E386" s="6"/>
-      <c r="F386" s="6"/>
+      <c r="F386" s="15"/>
       <c r="G386" s="6"/>
       <c r="H386" s="6"/>
       <c r="I386" s="6"/>
@@ -8627,7 +8814,7 @@
       <c r="C387" s="6"/>
       <c r="D387" s="6"/>
       <c r="E387" s="6"/>
-      <c r="F387" s="6"/>
+      <c r="F387" s="15"/>
       <c r="G387" s="6"/>
       <c r="H387" s="6"/>
       <c r="I387" s="6"/>
@@ -8644,7 +8831,7 @@
       <c r="C388" s="6"/>
       <c r="D388" s="6"/>
       <c r="E388" s="6"/>
-      <c r="F388" s="6"/>
+      <c r="F388" s="15"/>
       <c r="G388" s="6"/>
       <c r="H388" s="6"/>
       <c r="I388" s="6"/>
@@ -8661,7 +8848,7 @@
       <c r="C389" s="6"/>
       <c r="D389" s="6"/>
       <c r="E389" s="6"/>
-      <c r="F389" s="6"/>
+      <c r="F389" s="15"/>
       <c r="G389" s="6"/>
       <c r="H389" s="6"/>
       <c r="I389" s="6"/>
@@ -8678,7 +8865,7 @@
       <c r="C390" s="6"/>
       <c r="D390" s="6"/>
       <c r="E390" s="6"/>
-      <c r="F390" s="6"/>
+      <c r="F390" s="15"/>
       <c r="G390" s="6"/>
       <c r="H390" s="6"/>
       <c r="I390" s="6"/>
@@ -8695,7 +8882,7 @@
       <c r="C391" s="6"/>
       <c r="D391" s="6"/>
       <c r="E391" s="6"/>
-      <c r="F391" s="6"/>
+      <c r="F391" s="15"/>
       <c r="G391" s="6"/>
       <c r="H391" s="6"/>
       <c r="I391" s="6"/>
@@ -8712,7 +8899,7 @@
       <c r="C392" s="6"/>
       <c r="D392" s="6"/>
       <c r="E392" s="6"/>
-      <c r="F392" s="6"/>
+      <c r="F392" s="15"/>
       <c r="G392" s="6"/>
       <c r="H392" s="6"/>
       <c r="I392" s="6"/>
@@ -8729,7 +8916,7 @@
       <c r="C393" s="6"/>
       <c r="D393" s="6"/>
       <c r="E393" s="6"/>
-      <c r="F393" s="6"/>
+      <c r="F393" s="15"/>
       <c r="G393" s="6"/>
       <c r="H393" s="6"/>
       <c r="I393" s="6"/>
@@ -8746,7 +8933,7 @@
       <c r="C394" s="6"/>
       <c r="D394" s="6"/>
       <c r="E394" s="6"/>
-      <c r="F394" s="6"/>
+      <c r="F394" s="15"/>
       <c r="G394" s="6"/>
       <c r="H394" s="6"/>
       <c r="I394" s="6"/>
@@ -8763,7 +8950,7 @@
       <c r="C395" s="6"/>
       <c r="D395" s="6"/>
       <c r="E395" s="6"/>
-      <c r="F395" s="6"/>
+      <c r="F395" s="15"/>
       <c r="G395" s="6"/>
       <c r="H395" s="6"/>
       <c r="I395" s="6"/>
@@ -8780,7 +8967,7 @@
       <c r="C396" s="6"/>
       <c r="D396" s="6"/>
       <c r="E396" s="6"/>
-      <c r="F396" s="6"/>
+      <c r="F396" s="15"/>
       <c r="G396" s="6"/>
       <c r="H396" s="6"/>
       <c r="I396" s="6"/>
@@ -8797,7 +8984,7 @@
       <c r="C397" s="6"/>
       <c r="D397" s="6"/>
       <c r="E397" s="6"/>
-      <c r="F397" s="6"/>
+      <c r="F397" s="15"/>
       <c r="G397" s="6"/>
       <c r="H397" s="6"/>
       <c r="I397" s="6"/>
@@ -8814,7 +9001,7 @@
       <c r="C398" s="6"/>
       <c r="D398" s="6"/>
       <c r="E398" s="6"/>
-      <c r="F398" s="6"/>
+      <c r="F398" s="15"/>
       <c r="G398" s="6"/>
       <c r="H398" s="6"/>
       <c r="I398" s="6"/>
@@ -8831,7 +9018,7 @@
       <c r="C399" s="6"/>
       <c r="D399" s="6"/>
       <c r="E399" s="6"/>
-      <c r="F399" s="6"/>
+      <c r="F399" s="15"/>
       <c r="G399" s="6"/>
       <c r="H399" s="6"/>
       <c r="I399" s="6"/>
@@ -8848,7 +9035,7 @@
       <c r="C400" s="6"/>
       <c r="D400" s="6"/>
       <c r="E400" s="6"/>
-      <c r="F400" s="6"/>
+      <c r="F400" s="15"/>
       <c r="G400" s="6"/>
       <c r="H400" s="6"/>
       <c r="I400" s="6"/>
@@ -8865,7 +9052,7 @@
       <c r="C401" s="6"/>
       <c r="D401" s="6"/>
       <c r="E401" s="6"/>
-      <c r="F401" s="6"/>
+      <c r="F401" s="15"/>
       <c r="G401" s="6"/>
       <c r="H401" s="6"/>
       <c r="I401" s="6"/>
@@ -8882,7 +9069,7 @@
       <c r="C402" s="6"/>
       <c r="D402" s="6"/>
       <c r="E402" s="6"/>
-      <c r="F402" s="6"/>
+      <c r="F402" s="15"/>
       <c r="G402" s="6"/>
       <c r="H402" s="6"/>
       <c r="I402" s="6"/>

</xml_diff>

<commit_message>
Conversation for Nitwit Swen working. Only about a third of doors are rigged up.
</commit_message>
<xml_diff>
--- a/spoilers/conversations.xlsx
+++ b/spoilers/conversations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MYDATA\_GIT_REPOS\mcu4\spoilers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{996C5A6C-AC91-428B-877C-4B5EB2B81D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7938FE42-D55C-452B-A87F-15C7F8AA8A2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="11964" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,12 +16,15 @@
     <sheet name="Legend" sheetId="1" r:id="rId1"/>
     <sheet name="Conversations" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Conversations!$A$1:$O$37</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="214">
   <si>
     <t>Game-Level Conversation List</t>
   </si>
@@ -599,40 +602,70 @@
     <t>I love Johnny Cash!</t>
   </si>
   <si>
-    <t>Hi, my name is SWEN!</t>
-  </si>
-  <si>
-    <t>It'll come in handy at least once, around here.</t>
-  </si>
-  <si>
-    <t>I love the Doors</t>
-  </si>
-  <si>
-    <t>Here's the end of my riddle</t>
-  </si>
-  <si>
-    <t>Here's the start of my riddle</t>
-  </si>
-  <si>
-    <t>A zillion keys but no matching door.</t>
-  </si>
-  <si>
     <t>A zillion doors with no matching key...</t>
   </si>
   <si>
     <t>Cuz I've been "everywhere", man...in Jhelom!</t>
   </si>
   <si>
-    <t>Not the band, but all the doors in Jhelom</t>
-  </si>
-  <si>
-    <t>I love all the doors in Jhelom</t>
-  </si>
-  <si>
-    <t>Riddle 2 there's a zillion keys with no matching door</t>
-  </si>
-  <si>
-    <t>Riddle 1 there's a zillion doors with no matching key</t>
+    <t>I've been everywhere, man…in Jhelom</t>
+  </si>
+  <si>
+    <t>Riddles</t>
+  </si>
+  <si>
+    <t>Roses are red, pressure plates are blue…</t>
+  </si>
+  <si>
+    <t>Here's a riddle I'm working on…</t>
+  </si>
+  <si>
+    <t>…paintings don't speak, but duplicates do.</t>
+  </si>
+  <si>
+    <t>Not the band, but opening doors in Jhelom</t>
+  </si>
+  <si>
+    <t>I love The Doors</t>
+  </si>
+  <si>
+    <t>I've opened all the doors in Jhelom</t>
+  </si>
+  <si>
+    <t>A zillion keys with no matching door…</t>
+  </si>
+  <si>
+    <t>Paintings don't speak, but duplicates do...</t>
+  </si>
+  <si>
+    <t>Here's a joke I'm working on…</t>
+  </si>
+  <si>
+    <t>I looove making up riddles and jokes</t>
+  </si>
+  <si>
+    <t>When is a HELMET a BUCKET…?</t>
+  </si>
+  <si>
+    <t>When is a PUMPKIN a SQUASH…?</t>
+  </si>
+  <si>
+    <t>Folks in Jhelom are valiant but too serious.</t>
+  </si>
+  <si>
+    <t>Folks in Jhelom…</t>
+  </si>
+  <si>
+    <t>are valiant but too serious, IMO.</t>
+  </si>
+  <si>
+    <t>My name SWEN is an acronym for NEWS.</t>
+  </si>
+  <si>
+    <t>I love acronyms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">My name SWEN is an acronym for NEWS. </t>
   </si>
 </sst>
 </file>
@@ -1327,6 +1360,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:O402"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1393,7 +1427,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>58</v>
       </c>
@@ -1436,7 +1470,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>58</v>
       </c>
@@ -1477,7 +1511,7 @@
       </c>
       <c r="O3" s="5"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>58</v>
       </c>
@@ -1518,7 +1552,7 @@
       </c>
       <c r="O4" s="5"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>58</v>
       </c>
@@ -1559,7 +1593,7 @@
       </c>
       <c r="O5" s="5"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>58</v>
       </c>
@@ -1600,7 +1634,7 @@
       </c>
       <c r="O6" s="5"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>58</v>
       </c>
@@ -1641,7 +1675,7 @@
       </c>
       <c r="O7" s="5"/>
     </row>
-    <row r="8" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>58</v>
       </c>
@@ -1688,7 +1722,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>58</v>
       </c>
@@ -1731,7 +1765,7 @@
       </c>
       <c r="O9" s="5"/>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>58</v>
       </c>
@@ -1770,7 +1804,7 @@
       </c>
       <c r="O10" s="5"/>
     </row>
-    <row r="11" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>58</v>
       </c>
@@ -1811,7 +1845,7 @@
       </c>
       <c r="O11" s="5"/>
     </row>
-    <row r="12" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>58</v>
       </c>
@@ -1852,7 +1886,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="13" spans="1:15" s="10" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" s="10" customFormat="1" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
         <v>58</v>
       </c>
@@ -1893,7 +1927,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>58</v>
       </c>
@@ -1934,7 +1968,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>58</v>
       </c>
@@ -1975,7 +2009,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>58</v>
       </c>
@@ -2020,7 +2054,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>58</v>
       </c>
@@ -2061,7 +2095,7 @@
       </c>
       <c r="O17" s="5"/>
     </row>
-    <row r="18" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>58</v>
       </c>
@@ -2102,7 +2136,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>58</v>
       </c>
@@ -2143,7 +2177,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>58</v>
       </c>
@@ -2184,7 +2218,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>58</v>
       </c>
@@ -2225,7 +2259,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="22" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>58</v>
       </c>
@@ -2264,7 +2298,7 @@
       </c>
       <c r="O22" s="5"/>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>58</v>
       </c>
@@ -2304,7 +2338,7 @@
       </c>
       <c r="O23" s="5"/>
     </row>
-    <row r="24" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>58</v>
       </c>
@@ -2344,7 +2378,7 @@
       </c>
       <c r="O24" s="5"/>
     </row>
-    <row r="25" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>58</v>
       </c>
@@ -2384,7 +2418,7 @@
       </c>
       <c r="O25" s="5"/>
     </row>
-    <row r="26" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>58</v>
       </c>
@@ -2424,7 +2458,7 @@
       </c>
       <c r="O26" s="5"/>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>58</v>
       </c>
@@ -2463,7 +2497,7 @@
       </c>
       <c r="O27" s="5"/>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>58</v>
       </c>
@@ -2502,7 +2536,7 @@
       </c>
       <c r="O28" s="5"/>
     </row>
-    <row r="29" spans="1:15" s="12" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:15" s="12" customFormat="1" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
         <v>58</v>
       </c>
@@ -2543,7 +2577,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="30" spans="1:15" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:15" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
         <v>58</v>
       </c>
@@ -2584,7 +2618,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="31" spans="1:15" s="12" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:15" s="12" customFormat="1" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
         <v>58</v>
       </c>
@@ -2624,7 +2658,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="32" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
         <v>58</v>
       </c>
@@ -2690,15 +2724,17 @@
       </c>
       <c r="H33" s="5"/>
       <c r="I33" s="8">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>192</v>
+        <v>209</v>
       </c>
       <c r="K33" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="L33" s="6"/>
+        <v>210</v>
+      </c>
+      <c r="L33" s="6" t="s">
+        <v>208</v>
+      </c>
       <c r="M33" s="6"/>
       <c r="N33" s="6">
         <v>0</v>
@@ -2731,15 +2767,17 @@
       </c>
       <c r="H34" s="5"/>
       <c r="I34" s="8">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>191</v>
+        <v>212</v>
       </c>
       <c r="K34" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="L34" s="6"/>
+        <v>213</v>
+      </c>
+      <c r="L34" s="6" t="s">
+        <v>211</v>
+      </c>
       <c r="M34" s="6"/>
       <c r="N34" s="6">
         <v>0</v>
@@ -2772,16 +2810,16 @@
       </c>
       <c r="H35" s="5"/>
       <c r="I35" s="8">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="J35" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="K35" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="L35" s="6" t="s">
         <v>194</v>
-      </c>
-      <c r="K35" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="L35" s="6" t="s">
-        <v>201</v>
       </c>
       <c r="M35" s="6"/>
       <c r="N35" s="6">
@@ -2815,20 +2853,20 @@
       </c>
       <c r="H36" s="5"/>
       <c r="I36" s="8">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="J36" s="6" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="K36" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L36" s="6" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="M36" s="6"/>
       <c r="N36" s="6">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="O36" s="6" t="s">
         <v>121</v>
@@ -2858,124 +2896,282 @@
       </c>
       <c r="H37" s="5"/>
       <c r="I37" s="8">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="J37" s="6" t="s">
         <v>195</v>
       </c>
       <c r="K37" s="6" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="L37" s="6" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="M37" s="6"/>
       <c r="N37" s="6">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="O37" s="6" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A38" s="6"/>
-      <c r="B38" s="6"/>
-      <c r="C38" s="6"/>
-      <c r="D38" s="6"/>
-      <c r="E38" s="6"/>
-      <c r="F38" s="15"/>
-      <c r="G38" s="6"/>
+      <c r="A38" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F38" s="14">
+        <v>-1</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="H38" s="6"/>
-      <c r="I38" s="6"/>
-      <c r="L38" s="6"/>
+      <c r="I38" s="8">
+        <v>10</v>
+      </c>
+      <c r="J38" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="K38" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="L38" s="6" t="s">
+        <v>192</v>
+      </c>
       <c r="M38" s="6"/>
-      <c r="N38" s="6"/>
-      <c r="O38" s="6"/>
+      <c r="N38" s="6">
+        <v>5</v>
+      </c>
+      <c r="O38" s="6" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A39" s="6"/>
-      <c r="B39" s="6"/>
-      <c r="C39" s="6"/>
-      <c r="D39" s="6"/>
-      <c r="E39" s="6"/>
-      <c r="F39" s="15"/>
-      <c r="G39" s="6"/>
+      <c r="A39" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E39" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F39" s="14">
+        <v>-1</v>
+      </c>
+      <c r="G39" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="H39" s="6"/>
-      <c r="I39" s="6"/>
-      <c r="J39" s="6"/>
-      <c r="K39" s="6"/>
-      <c r="L39" s="6"/>
+      <c r="I39" s="8">
+        <v>5</v>
+      </c>
+      <c r="J39" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="K39" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="L39" s="6" t="s">
+        <v>202</v>
+      </c>
       <c r="M39" s="6"/>
-      <c r="N39" s="6"/>
-      <c r="O39" s="6"/>
+      <c r="N39" s="6">
+        <v>5</v>
+      </c>
+      <c r="O39" s="6" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A40" s="6"/>
-      <c r="B40" s="6"/>
-      <c r="C40" s="6"/>
-      <c r="D40" s="6"/>
-      <c r="E40" s="6"/>
-      <c r="F40" s="15"/>
-      <c r="G40" s="6"/>
+      <c r="A40" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D40" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F40" s="14">
+        <v>-1</v>
+      </c>
+      <c r="G40" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="H40" s="6"/>
-      <c r="I40" s="6"/>
-      <c r="J40" s="6"/>
-      <c r="K40" s="6"/>
-      <c r="L40" s="6"/>
+      <c r="I40" s="8">
+        <v>10</v>
+      </c>
+      <c r="J40" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="K40" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="L40" s="6" t="s">
+        <v>196</v>
+      </c>
       <c r="M40" s="6"/>
-      <c r="N40" s="6"/>
-      <c r="O40" s="6"/>
+      <c r="N40" s="6">
+        <v>5</v>
+      </c>
+      <c r="O40" s="6" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A41" s="6"/>
-      <c r="B41" s="6"/>
-      <c r="C41" s="6"/>
-      <c r="D41" s="6"/>
-      <c r="E41" s="6"/>
-      <c r="F41" s="15"/>
-      <c r="G41" s="6"/>
+      <c r="A41" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D41" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E41" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F41" s="14">
+        <v>-1</v>
+      </c>
+      <c r="G41" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="H41" s="6"/>
-      <c r="I41" s="6"/>
-      <c r="J41" s="6"/>
-      <c r="K41" s="6"/>
-      <c r="L41" s="6"/>
+      <c r="I41" s="8">
+        <v>10</v>
+      </c>
+      <c r="J41" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="K41" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="L41" s="6" t="s">
+        <v>203</v>
+      </c>
       <c r="M41" s="6"/>
-      <c r="N41" s="6"/>
-      <c r="O41" s="6"/>
+      <c r="N41" s="6">
+        <v>5</v>
+      </c>
+      <c r="O41" s="6" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A42" s="6"/>
-      <c r="B42" s="6"/>
-      <c r="C42" s="6"/>
-      <c r="D42" s="6"/>
-      <c r="E42" s="6"/>
-      <c r="F42" s="15"/>
-      <c r="G42" s="6"/>
+      <c r="A42" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D42" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E42" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F42" s="14">
+        <v>-1</v>
+      </c>
+      <c r="G42" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="H42" s="6"/>
-      <c r="I42" s="6"/>
-      <c r="J42" s="6"/>
-      <c r="K42" s="6"/>
-      <c r="L42" s="6"/>
+      <c r="I42" s="8">
+        <v>10</v>
+      </c>
+      <c r="J42" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="K42" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="L42" s="6" t="s">
+        <v>207</v>
+      </c>
       <c r="M42" s="6"/>
-      <c r="N42" s="6"/>
-      <c r="O42" s="6"/>
+      <c r="N42" s="6">
+        <v>5</v>
+      </c>
+      <c r="O42" s="6" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A43" s="6"/>
-      <c r="B43" s="6"/>
-      <c r="C43" s="6"/>
-      <c r="D43" s="6"/>
-      <c r="E43" s="6"/>
-      <c r="F43" s="15"/>
-      <c r="G43" s="6"/>
+      <c r="A43" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D43" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E43" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F43" s="14">
+        <v>-1</v>
+      </c>
+      <c r="G43" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="H43" s="6"/>
-      <c r="I43" s="6"/>
-      <c r="J43" s="6"/>
-      <c r="K43" s="6"/>
-      <c r="L43" s="6"/>
+      <c r="I43" s="8">
+        <v>10</v>
+      </c>
+      <c r="J43" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="K43" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="L43" s="6" t="s">
+        <v>206</v>
+      </c>
       <c r="M43" s="6"/>
-      <c r="N43" s="6"/>
-      <c r="O43" s="6"/>
+      <c r="N43" s="6">
+        <v>5</v>
+      </c>
+      <c r="O43" s="6" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44" s="6"/>
@@ -9081,6 +9277,13 @@
       <c r="O402" s="6"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:O37" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Jhelom"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" sqref="G2:G29 G32:G402" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Statement,Question,Statement-Roll"</formula1>

</xml_diff>

<commit_message>
Hero (Weaponsmith in Lounge) - Tested OK including L1-L3,Question.
</commit_message>
<xml_diff>
--- a/spoilers/conversations.xlsx
+++ b/spoilers/conversations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MYDATA\_GIT_REPOS\mcu4\spoilers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7938FE42-D55C-452B-A87F-15C7F8AA8A2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6407DC3F-51C6-4790-80EA-FAC2F64DAD5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="11964" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,14 +17,14 @@
     <sheet name="Conversations" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Conversations!$A$1:$O$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Conversations!$A$1:$O$48</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="238">
   <si>
     <t>Game-Level Conversation List</t>
   </si>
@@ -608,18 +608,15 @@
     <t>Cuz I've been "everywhere", man...in Jhelom!</t>
   </si>
   <si>
-    <t>I've been everywhere, man…in Jhelom</t>
-  </si>
-  <si>
     <t>Riddles</t>
   </si>
   <si>
+    <t>Here's a riddle…</t>
+  </si>
+  <si>
     <t>Roses are red, pressure plates are blue…</t>
   </si>
   <si>
-    <t>Here's a riddle I'm working on…</t>
-  </si>
-  <si>
     <t>…paintings don't speak, but duplicates do.</t>
   </si>
   <si>
@@ -629,15 +626,9 @@
     <t>I love The Doors</t>
   </si>
   <si>
-    <t>I've opened all the doors in Jhelom</t>
-  </si>
-  <si>
     <t>A zillion keys with no matching door…</t>
   </si>
   <si>
-    <t>Paintings don't speak, but duplicates do...</t>
-  </si>
-  <si>
     <t>Here's a joke I'm working on…</t>
   </si>
   <si>
@@ -650,29 +641,110 @@
     <t>When is a PUMPKIN a SQUASH…?</t>
   </si>
   <si>
-    <t>Folks in Jhelom are valiant but too serious.</t>
-  </si>
-  <si>
     <t>Folks in Jhelom…</t>
   </si>
   <si>
     <t>are valiant but too serious, IMO.</t>
   </si>
   <si>
-    <t>My name SWEN is an acronym for NEWS.</t>
-  </si>
-  <si>
     <t>I love acronyms</t>
   </si>
   <si>
     <t xml:space="preserve">My name SWEN is an acronym for NEWS. </t>
+  </si>
+  <si>
+    <t>Hero</t>
+  </si>
+  <si>
+    <t>Lives in Hero's Lounge</t>
+  </si>
+  <si>
+    <t>I'll trade a trial key for a Goat Horn!</t>
+  </si>
+  <si>
+    <t>Trial keys are hard-earned!</t>
+  </si>
+  <si>
+    <t>Goat Horns are magical!</t>
+  </si>
+  <si>
+    <t>They'll return you to Jhelom's Moongate!</t>
+  </si>
+  <si>
+    <t>Reveals Totem of Undying Trade</t>
+  </si>
+  <si>
+    <t>Swen: Folks in Jhelom are valiant but too serious.</t>
+  </si>
+  <si>
+    <t>Swen: My name SWEN is an acronym for NEWS.</t>
+  </si>
+  <si>
+    <t>Swen: I've been everywhere, man…in Jhelom</t>
+  </si>
+  <si>
+    <t>Swen: I've opened all the doors in Jhelom</t>
+  </si>
+  <si>
+    <t>Swen: I looove making up riddles and jokes</t>
+  </si>
+  <si>
+    <t>Swen: A zillion doors with no matching key...</t>
+  </si>
+  <si>
+    <t>Swen: A zillion keys with no matching door…</t>
+  </si>
+  <si>
+    <t>Swen: Roses are red, pressure plates are blue…</t>
+  </si>
+  <si>
+    <t>Swen: Paintings don't speak, but duplicates do...</t>
+  </si>
+  <si>
+    <t>Swen: When is a PUMPKIN a SQUASH…?</t>
+  </si>
+  <si>
+    <t>Swen: When is a HELMET a BUCKET…?</t>
+  </si>
+  <si>
+    <t>Hero: I'll trade a trial key for a Goat Horn!</t>
+  </si>
+  <si>
+    <t>Hero: Goat Horns return you to Jhelom's Moongate</t>
+  </si>
+  <si>
+    <t>Hero: Return to me with a totem of undying!</t>
+  </si>
+  <si>
+    <t>Hero: Hmm.  I thought you looked kind of pale.</t>
+  </si>
+  <si>
+    <t>Do thou strive to be valiant against evil?</t>
+  </si>
+  <si>
+    <t>L2 Trade or higher</t>
+  </si>
+  <si>
+    <t>A Totem of Undying!</t>
+  </si>
+  <si>
+    <t>The rune is hidden in a corner of this city!</t>
+  </si>
+  <si>
+    <t>Hero: The rune is hidden in a corner of this city!</t>
+  </si>
+  <si>
+    <t>Others will tell of rune too but whatever.</t>
+  </si>
+  <si>
+    <t>Hero doesn’t think much of this guy.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -726,8 +798,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -744,6 +822,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFE8EAF0"/>
         <bgColor rgb="FFE8EAF0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -774,7 +864,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -821,6 +911,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1360,7 +1461,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:O402"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1427,8 +1527,8 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B2" s="5" t="s">
@@ -1470,8 +1570,8 @@
         <v>66</v>
       </c>
     </row>
-    <row r="3" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A3" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B3" s="5" t="s">
@@ -1511,8 +1611,8 @@
       </c>
       <c r="O3" s="5"/>
     </row>
-    <row r="4" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A4" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B4" s="5" t="s">
@@ -1552,8 +1652,8 @@
       </c>
       <c r="O4" s="5"/>
     </row>
-    <row r="5" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A5" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -1593,8 +1693,8 @@
       </c>
       <c r="O5" s="5"/>
     </row>
-    <row r="6" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A6" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B6" s="5" t="s">
@@ -1634,8 +1734,8 @@
       </c>
       <c r="O6" s="5"/>
     </row>
-    <row r="7" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A7" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B7" s="5" t="s">
@@ -1675,8 +1775,8 @@
       </c>
       <c r="O7" s="5"/>
     </row>
-    <row r="8" spans="1:15" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+    <row r="8" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B8" s="5" t="s">
@@ -1722,8 +1822,8 @@
         <v>76</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
+    <row r="9" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B9" s="5" t="s">
@@ -1765,8 +1865,8 @@
       </c>
       <c r="O9" s="5"/>
     </row>
-    <row r="10" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A10" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B10" s="5" t="s">
@@ -1804,8 +1904,8 @@
       </c>
       <c r="O10" s="5"/>
     </row>
-    <row r="11" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
+    <row r="11" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A11" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B11" s="5" t="s">
@@ -1845,8 +1945,8 @@
       </c>
       <c r="O11" s="5"/>
     </row>
-    <row r="12" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
+    <row r="12" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A12" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B12" s="5" t="s">
@@ -1886,8 +1986,8 @@
         <v>89</v>
       </c>
     </row>
-    <row r="13" spans="1:15" s="10" customFormat="1" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
+    <row r="13" spans="1:15" s="10" customFormat="1" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="21" t="s">
         <v>58</v>
       </c>
       <c r="B13" s="7" t="s">
@@ -1927,8 +2027,8 @@
         <v>93</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
+    <row r="14" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A14" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B14" s="5" t="s">
@@ -1968,8 +2068,8 @@
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
+    <row r="15" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A15" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B15" s="5" t="s">
@@ -2009,8 +2109,8 @@
         <v>104</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="39.6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="5" t="s">
+    <row r="16" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B16" s="5" t="s">
@@ -2054,8 +2154,8 @@
         <v>108</v>
       </c>
     </row>
-    <row r="17" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="5" t="s">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A17" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B17" s="5" t="s">
@@ -2095,8 +2195,8 @@
       </c>
       <c r="O17" s="5"/>
     </row>
-    <row r="18" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="5" t="s">
+    <row r="18" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A18" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B18" s="5" t="s">
@@ -2136,8 +2236,8 @@
         <v>115</v>
       </c>
     </row>
-    <row r="19" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A19" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B19" s="5" t="s">
@@ -2177,8 +2277,8 @@
         <v>115</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="5" t="s">
+    <row r="20" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A20" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B20" s="5" t="s">
@@ -2218,8 +2318,8 @@
         <v>123</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
+    <row r="21" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A21" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B21" s="5" t="s">
@@ -2259,8 +2359,8 @@
         <v>123</v>
       </c>
     </row>
-    <row r="22" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="5" t="s">
+    <row r="22" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A22" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B22" s="5" t="s">
@@ -2298,8 +2398,8 @@
       </c>
       <c r="O22" s="5"/>
     </row>
-    <row r="23" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="5" t="s">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A23" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B23" s="5" t="s">
@@ -2338,8 +2438,8 @@
       </c>
       <c r="O23" s="5"/>
     </row>
-    <row r="24" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
+    <row r="24" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A24" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B24" s="5" t="s">
@@ -2378,8 +2478,8 @@
       </c>
       <c r="O24" s="5"/>
     </row>
-    <row r="25" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="5" t="s">
+    <row r="25" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A25" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B25" s="5" t="s">
@@ -2418,8 +2518,8 @@
       </c>
       <c r="O25" s="5"/>
     </row>
-    <row r="26" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="5" t="s">
+    <row r="26" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A26" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B26" s="5" t="s">
@@ -2458,8 +2558,8 @@
       </c>
       <c r="O26" s="5"/>
     </row>
-    <row r="27" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="5" t="s">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A27" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B27" s="5" t="s">
@@ -2497,8 +2597,8 @@
       </c>
       <c r="O27" s="5"/>
     </row>
-    <row r="28" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="5" t="s">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A28" s="20" t="s">
         <v>58</v>
       </c>
       <c r="B28" s="5" t="s">
@@ -2536,8 +2636,8 @@
       </c>
       <c r="O28" s="5"/>
     </row>
-    <row r="29" spans="1:15" s="12" customFormat="1" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="8" t="s">
+    <row r="29" spans="1:15" s="12" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A29" s="22" t="s">
         <v>58</v>
       </c>
       <c r="B29" s="9" t="s">
@@ -2577,8 +2677,8 @@
         <v>111</v>
       </c>
     </row>
-    <row r="30" spans="1:15" s="10" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="8" t="s">
+    <row r="30" spans="1:15" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="22" t="s">
         <v>58</v>
       </c>
       <c r="B30" s="10" t="s">
@@ -2618,8 +2718,8 @@
         <v>115</v>
       </c>
     </row>
-    <row r="31" spans="1:15" s="12" customFormat="1" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="8" t="s">
+    <row r="31" spans="1:15" s="12" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A31" s="22" t="s">
         <v>58</v>
       </c>
       <c r="B31" s="12" t="s">
@@ -2658,8 +2758,8 @@
         <v>115</v>
       </c>
     </row>
-    <row r="32" spans="1:15" ht="26.4" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="7" t="s">
+    <row r="32" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A32" s="21" t="s">
         <v>58</v>
       </c>
       <c r="B32" s="7" t="s">
@@ -2700,8 +2800,8 @@
         <v>183</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A33" s="6" t="s">
+    <row r="33" spans="1:15" s="24" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="23" t="s">
         <v>189</v>
       </c>
       <c r="B33" s="6" t="s">
@@ -2724,16 +2824,16 @@
       </c>
       <c r="H33" s="5"/>
       <c r="I33" s="8">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="K33" s="6" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="L33" s="6" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="M33" s="6"/>
       <c r="N33" s="6">
@@ -2743,8 +2843,8 @@
         <v>121</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A34" s="6" t="s">
+    <row r="34" spans="1:15" s="24" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="23" t="s">
         <v>189</v>
       </c>
       <c r="B34" s="6" t="s">
@@ -2767,16 +2867,16 @@
       </c>
       <c r="H34" s="5"/>
       <c r="I34" s="8">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="K34" s="6" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="L34" s="6" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="M34" s="6"/>
       <c r="N34" s="6">
@@ -2786,8 +2886,8 @@
         <v>121</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A35" s="6" t="s">
+    <row r="35" spans="1:15" s="24" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="23" t="s">
         <v>189</v>
       </c>
       <c r="B35" s="6" t="s">
@@ -2810,7 +2910,7 @@
       </c>
       <c r="H35" s="5"/>
       <c r="I35" s="8">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J35" s="6" t="s">
         <v>191</v>
@@ -2819,7 +2919,7 @@
         <v>193</v>
       </c>
       <c r="L35" s="6" t="s">
-        <v>194</v>
+        <v>218</v>
       </c>
       <c r="M35" s="6"/>
       <c r="N35" s="6">
@@ -2829,8 +2929,8 @@
         <v>121</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A36" s="6" t="s">
+    <row r="36" spans="1:15" s="24" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="23" t="s">
         <v>189</v>
       </c>
       <c r="B36" s="6" t="s">
@@ -2853,16 +2953,16 @@
       </c>
       <c r="H36" s="5"/>
       <c r="I36" s="8">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J36" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K36" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="L36" s="6" t="s">
-        <v>201</v>
+        <v>219</v>
       </c>
       <c r="M36" s="6"/>
       <c r="N36" s="6">
@@ -2872,8 +2972,8 @@
         <v>121</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A37" s="6" t="s">
+    <row r="37" spans="1:15" s="24" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="23" t="s">
         <v>189</v>
       </c>
       <c r="B37" s="6" t="s">
@@ -2896,16 +2996,16 @@
       </c>
       <c r="H37" s="5"/>
       <c r="I37" s="8">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="K37" s="6" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="L37" s="6" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="M37" s="6"/>
       <c r="N37" s="6">
@@ -2915,8 +3015,8 @@
         <v>121</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A38" s="6" t="s">
+    <row r="38" spans="1:15" s="24" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="23" t="s">
         <v>189</v>
       </c>
       <c r="B38" s="6" t="s">
@@ -2939,16 +3039,16 @@
       </c>
       <c r="H38" s="6"/>
       <c r="I38" s="8">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="K38" s="6" t="s">
         <v>192</v>
       </c>
       <c r="L38" s="6" t="s">
-        <v>192</v>
+        <v>221</v>
       </c>
       <c r="M38" s="6"/>
       <c r="N38" s="6">
@@ -2958,8 +3058,8 @@
         <v>121</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A39" s="6" t="s">
+    <row r="39" spans="1:15" s="24" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="23" t="s">
         <v>189</v>
       </c>
       <c r="B39" s="6" t="s">
@@ -2982,16 +3082,16 @@
       </c>
       <c r="H39" s="6"/>
       <c r="I39" s="8">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J39" s="6" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="K39" s="6" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="L39" s="6" t="s">
-        <v>202</v>
+        <v>222</v>
       </c>
       <c r="M39" s="6"/>
       <c r="N39" s="6">
@@ -3001,8 +3101,8 @@
         <v>121</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A40" s="6" t="s">
+    <row r="40" spans="1:15" s="24" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="23" t="s">
         <v>189</v>
       </c>
       <c r="B40" s="6" t="s">
@@ -3025,16 +3125,16 @@
       </c>
       <c r="H40" s="6"/>
       <c r="I40" s="8">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J40" s="6" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="K40" s="6" t="s">
         <v>196</v>
       </c>
       <c r="L40" s="6" t="s">
-        <v>196</v>
+        <v>223</v>
       </c>
       <c r="M40" s="6"/>
       <c r="N40" s="6">
@@ -3044,8 +3144,8 @@
         <v>121</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A41" s="6" t="s">
+    <row r="41" spans="1:15" s="24" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="23" t="s">
         <v>189</v>
       </c>
       <c r="B41" s="6" t="s">
@@ -3068,16 +3168,16 @@
       </c>
       <c r="H41" s="6"/>
       <c r="I41" s="8">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J41" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="K41" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="K41" s="6" t="s">
-        <v>198</v>
-      </c>
       <c r="L41" s="6" t="s">
-        <v>203</v>
+        <v>224</v>
       </c>
       <c r="M41" s="6"/>
       <c r="N41" s="6">
@@ -3087,8 +3187,8 @@
         <v>121</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A42" s="6" t="s">
+    <row r="42" spans="1:15" s="24" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="23" t="s">
         <v>189</v>
       </c>
       <c r="B42" s="6" t="s">
@@ -3111,16 +3211,16 @@
       </c>
       <c r="H42" s="6"/>
       <c r="I42" s="8">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J42" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="K42" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="K42" s="6" t="s">
-        <v>207</v>
-      </c>
       <c r="L42" s="6" t="s">
-        <v>207</v>
+        <v>225</v>
       </c>
       <c r="M42" s="6"/>
       <c r="N42" s="6">
@@ -3130,8 +3230,8 @@
         <v>121</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A43" s="6" t="s">
+    <row r="43" spans="1:15" s="24" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="23" t="s">
         <v>189</v>
       </c>
       <c r="B43" s="6" t="s">
@@ -3154,16 +3254,16 @@
       </c>
       <c r="H43" s="6"/>
       <c r="I43" s="8">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J43" s="6" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="K43" s="6" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="L43" s="6" t="s">
-        <v>206</v>
+        <v>226</v>
       </c>
       <c r="M43" s="6"/>
       <c r="N43" s="6">
@@ -3173,90 +3273,224 @@
         <v>121</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A44" s="6"/>
-      <c r="B44" s="6"/>
-      <c r="C44" s="6"/>
-      <c r="D44" s="6"/>
-      <c r="E44" s="6"/>
-      <c r="F44" s="15"/>
-      <c r="G44" s="6"/>
+    <row r="44" spans="1:15" s="24" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="23" t="s">
+        <v>189</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D44" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E44" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F44" s="14">
+        <v>-1</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="H44" s="6"/>
-      <c r="I44" s="6"/>
-      <c r="J44" s="6"/>
-      <c r="K44" s="6"/>
-      <c r="L44" s="6"/>
+      <c r="I44" s="6">
+        <v>40</v>
+      </c>
+      <c r="J44" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="K44" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="L44" s="6" t="s">
+        <v>227</v>
+      </c>
       <c r="M44" s="6"/>
-      <c r="N44" s="6"/>
-      <c r="O44" s="6"/>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A45" s="6"/>
-      <c r="B45" s="6"/>
-      <c r="C45" s="6"/>
-      <c r="D45" s="6"/>
-      <c r="E45" s="6"/>
-      <c r="F45" s="15"/>
-      <c r="G45" s="6"/>
+      <c r="N44" s="6">
+        <v>5</v>
+      </c>
+      <c r="O44" s="6" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" s="24" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="23" t="s">
+        <v>189</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D45" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E45" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F45" s="14">
+        <v>-1</v>
+      </c>
+      <c r="G45" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="H45" s="6"/>
-      <c r="I45" s="6"/>
-      <c r="J45" s="6"/>
-      <c r="K45" s="6"/>
-      <c r="L45" s="6"/>
+      <c r="I45" s="6">
+        <v>40</v>
+      </c>
+      <c r="J45" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="K45" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="L45" s="6" t="s">
+        <v>228</v>
+      </c>
       <c r="M45" s="6"/>
-      <c r="N45" s="6"/>
-      <c r="O45" s="6"/>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A46" s="6"/>
-      <c r="B46" s="6"/>
-      <c r="C46" s="6"/>
-      <c r="D46" s="6"/>
-      <c r="E46" s="6"/>
-      <c r="F46" s="15"/>
-      <c r="G46" s="6"/>
-      <c r="H46" s="6"/>
-      <c r="I46" s="6"/>
-      <c r="J46" s="6"/>
-      <c r="K46" s="6"/>
-      <c r="L46" s="6"/>
-      <c r="M46" s="6"/>
-      <c r="N46" s="6"/>
-      <c r="O46" s="6"/>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A47" s="6"/>
-      <c r="B47" s="6"/>
-      <c r="C47" s="6"/>
-      <c r="D47" s="6"/>
-      <c r="E47" s="6"/>
-      <c r="F47" s="15"/>
-      <c r="G47" s="6"/>
-      <c r="H47" s="6"/>
-      <c r="I47" s="6"/>
-      <c r="J47" s="6"/>
-      <c r="K47" s="6"/>
-      <c r="L47" s="6"/>
-      <c r="M47" s="6"/>
-      <c r="N47" s="6"/>
-      <c r="O47" s="6"/>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A48" s="6"/>
-      <c r="B48" s="6"/>
-      <c r="C48" s="6"/>
-      <c r="D48" s="6"/>
-      <c r="E48" s="6"/>
-      <c r="F48" s="15"/>
-      <c r="G48" s="6"/>
+      <c r="N45" s="6">
+        <v>5</v>
+      </c>
+      <c r="O45" s="6" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" s="24" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="23" t="s">
+        <v>189</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D46" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E46" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F46" s="14">
+        <v>3</v>
+      </c>
+      <c r="G46" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="H46" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="I46" s="5">
+        <v>20</v>
+      </c>
+      <c r="J46" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="K46" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="L46" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="M46" s="5">
+        <v>100</v>
+      </c>
+      <c r="N46" s="5">
+        <v>20</v>
+      </c>
+      <c r="O46" s="5" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" s="24" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="23" t="s">
+        <v>189</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D47" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E47" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F47" s="14">
+        <v>3</v>
+      </c>
+      <c r="G47" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="H47" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="I47" s="5">
+        <v>20</v>
+      </c>
+      <c r="J47" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="K47" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="L47" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="M47" s="5"/>
+      <c r="N47" s="5">
+        <v>-100</v>
+      </c>
+      <c r="O47" s="6" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" s="24" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A48" s="23" t="s">
+        <v>189</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D48" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="F48" s="14">
+        <v>-1</v>
+      </c>
+      <c r="G48" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="H48" s="6"/>
       <c r="I48" s="6"/>
-      <c r="J48" s="6"/>
-      <c r="K48" s="6"/>
-      <c r="L48" s="6"/>
+      <c r="J48" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="K48" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="L48" s="6" t="s">
+        <v>235</v>
+      </c>
       <c r="M48" s="6"/>
-      <c r="N48" s="6"/>
-      <c r="O48" s="6"/>
+      <c r="N48" s="6">
+        <v>5</v>
+      </c>
+      <c r="O48" s="6" t="s">
+        <v>236</v>
+      </c>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A49" s="6"/>
@@ -9277,13 +9511,7 @@
       <c r="O402" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O37" xr:uid="{00000000-0001-0000-0100-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Jhelom"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:O48" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" sqref="G2:G29 G32:G402" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Statement,Question,Statement-Roll"</formula1>

</xml_diff>

<commit_message>
Added Smith the Talking Horse.
</commit_message>
<xml_diff>
--- a/spoilers/conversations.xlsx
+++ b/spoilers/conversations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MYDATA\_GIT_REPOS\mcu4\spoilers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6407DC3F-51C6-4790-80EA-FAC2F64DAD5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C121753-6C32-43FB-8990-C0589521D940}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="11964" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="250">
   <si>
     <t>Game-Level Conversation List</t>
   </si>
@@ -738,6 +738,42 @@
   </si>
   <si>
     <t>Hero doesn’t think much of this guy.</t>
+  </si>
+  <si>
+    <t>Smith</t>
+  </si>
+  <si>
+    <t>Horse</t>
+  </si>
+  <si>
+    <t>Hi, I'm Mr Ed!</t>
+  </si>
+  <si>
+    <t>Smith: I'm Mr Ed! Neighh, I'm a Smith!</t>
+  </si>
+  <si>
+    <t>Neighh, just kidding. I'm a Smith</t>
+  </si>
+  <si>
+    <t>Smith: Infinity was the final answer in Ultima 4.</t>
+  </si>
+  <si>
+    <t>The Answer to Life is...</t>
+  </si>
+  <si>
+    <t>...Infinity.  Well, it was in Ultima 4.</t>
+  </si>
+  <si>
+    <t>Psst…</t>
+  </si>
+  <si>
+    <t>Mind grabbing me an apple?</t>
+  </si>
+  <si>
+    <t>Smith: Psst! Grab me an apple!</t>
+  </si>
+  <si>
+    <t>A talking horse.</t>
   </si>
 </sst>
 </file>
@@ -3471,7 +3507,7 @@
         <v>-1</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>63</v>
+        <v>81</v>
       </c>
       <c r="H48" s="6"/>
       <c r="I48" s="6"/>
@@ -3493,55 +3529,133 @@
       </c>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A49" s="6"/>
-      <c r="B49" s="6"/>
-      <c r="C49" s="6"/>
-      <c r="D49" s="6"/>
-      <c r="E49" s="6"/>
-      <c r="F49" s="15"/>
-      <c r="G49" s="6"/>
+      <c r="A49" s="23" t="s">
+        <v>189</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D49" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E49" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="F49" s="15">
+        <v>-1</v>
+      </c>
+      <c r="G49" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="H49" s="6"/>
-      <c r="I49" s="6"/>
-      <c r="J49" s="6"/>
-      <c r="K49" s="6"/>
-      <c r="L49" s="6"/>
+      <c r="I49" s="6">
+        <v>30</v>
+      </c>
+      <c r="J49" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="K49" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="L49" s="6" t="s">
+        <v>241</v>
+      </c>
       <c r="M49" s="6"/>
-      <c r="N49" s="6"/>
-      <c r="O49" s="6"/>
+      <c r="N49" s="6">
+        <v>0</v>
+      </c>
+      <c r="O49" s="6" t="s">
+        <v>249</v>
+      </c>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A50" s="6"/>
-      <c r="B50" s="6"/>
-      <c r="C50" s="6"/>
-      <c r="D50" s="6"/>
-      <c r="E50" s="6"/>
-      <c r="F50" s="15"/>
-      <c r="G50" s="6"/>
+      <c r="A50" s="23" t="s">
+        <v>189</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D50" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E50" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="F50" s="15">
+        <v>-1</v>
+      </c>
+      <c r="G50" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="H50" s="6"/>
-      <c r="I50" s="6"/>
-      <c r="J50" s="6"/>
-      <c r="K50" s="6"/>
-      <c r="L50" s="6"/>
+      <c r="I50" s="6">
+        <v>30</v>
+      </c>
+      <c r="J50" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="K50" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="L50" s="6" t="s">
+        <v>243</v>
+      </c>
       <c r="M50" s="6"/>
-      <c r="N50" s="6"/>
-      <c r="O50" s="6"/>
+      <c r="N50" s="6">
+        <v>0</v>
+      </c>
+      <c r="O50" s="6" t="s">
+        <v>249</v>
+      </c>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A51" s="6"/>
-      <c r="B51" s="6"/>
-      <c r="C51" s="6"/>
-      <c r="D51" s="6"/>
-      <c r="E51" s="6"/>
-      <c r="F51" s="15"/>
-      <c r="G51" s="6"/>
+      <c r="A51" s="23" t="s">
+        <v>189</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D51" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E51" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="F51" s="15">
+        <v>-1</v>
+      </c>
+      <c r="G51" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="H51" s="6"/>
-      <c r="I51" s="6"/>
-      <c r="J51" s="6"/>
-      <c r="K51" s="6"/>
-      <c r="L51" s="6"/>
+      <c r="I51" s="6">
+        <v>40</v>
+      </c>
+      <c r="J51" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="K51" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="L51" s="6" t="s">
+        <v>248</v>
+      </c>
       <c r="M51" s="6"/>
-      <c r="N51" s="6"/>
-      <c r="O51" s="6"/>
+      <c r="N51" s="6">
+        <v>0</v>
+      </c>
+      <c r="O51" s="6" t="s">
+        <v>249</v>
+      </c>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52" s="6"/>

</xml_diff>

<commit_message>
Additional testing and polishing in Skara Brae.  Trade and Convos for most NPCs tbd
</commit_message>
<xml_diff>
--- a/spoilers/conversations.xlsx
+++ b/spoilers/conversations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MYDATA\_GIT_REPOS\mcu4\spoilers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C121753-6C32-43FB-8990-C0589521D940}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF6689E9-BB0D-4C7B-8E5B-21BF114C2E6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="11964" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="271">
   <si>
     <t>Game-Level Conversation List</t>
   </si>
@@ -774,6 +774,69 @@
   </si>
   <si>
     <t>A talking horse.</t>
+  </si>
+  <si>
+    <t>Skara Brae</t>
+  </si>
+  <si>
+    <t>Tyrone</t>
+  </si>
+  <si>
+    <t>Innkeeper</t>
+  </si>
+  <si>
+    <t>Welcome, stranger.</t>
+  </si>
+  <si>
+    <t>I rent to only those with some gold to show.</t>
+  </si>
+  <si>
+    <t>Tyrone: I rent to only those with some gold to show.</t>
+  </si>
+  <si>
+    <t>Here's your change.</t>
+  </si>
+  <si>
+    <t>Come back when you'd like a room.</t>
+  </si>
+  <si>
+    <t>Tyrone: Here's your change.</t>
+  </si>
+  <si>
+    <t>Proximity (L2, night only)</t>
+  </si>
+  <si>
+    <t>Would you like a room rental?</t>
+  </si>
+  <si>
+    <t>Tyrone: Then welcome — the room's yours for the night.</t>
+  </si>
+  <si>
+    <t>Opens door; declines if room occupied</t>
+  </si>
+  <si>
+    <t>Tyrone: Suit yourself.</t>
+  </si>
+  <si>
+    <t>Proximity (L2, daytime)</t>
+  </si>
+  <si>
+    <t>(no title)</t>
+  </si>
+  <si>
+    <t>(no subtitle)</t>
+  </si>
+  <si>
+    <t>Tyrone: I don't rent rooms during day!</t>
+  </si>
+  <si>
+    <t>Placeholder text</t>
+  </si>
+  <si>
+    <t>Proximity (L2, occupied)</t>
+  </si>
+  <si>
+    <t>Tyrone: Sorry, the room's occupied right now.</t>
   </si>
 </sst>
 </file>
@@ -841,7 +904,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -869,6 +932,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -900,7 +969,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -941,10 +1010,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -958,6 +1027,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1497,7 +1567,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:O402"/>
+  <dimension ref="A1:O399"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -3658,103 +3728,237 @@
       </c>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A52" s="6"/>
-      <c r="B52" s="6"/>
-      <c r="C52" s="6"/>
-      <c r="D52" s="6"/>
-      <c r="E52" s="6"/>
-      <c r="F52" s="15"/>
-      <c r="G52" s="6"/>
+      <c r="A52" s="25" t="s">
+        <v>250</v>
+      </c>
+      <c r="B52" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E52" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="F52" s="15">
+        <v>-1</v>
+      </c>
+      <c r="G52" s="6" t="s">
+        <v>63</v>
+      </c>
       <c r="H52" s="6"/>
-      <c r="I52" s="6"/>
-      <c r="J52" s="6"/>
-      <c r="K52" s="6"/>
-      <c r="L52" s="6"/>
+      <c r="I52" s="6">
+        <v>100</v>
+      </c>
+      <c r="J52" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="K52" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="L52" s="6" t="s">
+        <v>255</v>
+      </c>
       <c r="M52" s="6"/>
       <c r="N52" s="6"/>
       <c r="O52" s="6"/>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A53" s="6"/>
-      <c r="B53" s="6"/>
-      <c r="C53" s="6"/>
-      <c r="D53" s="6"/>
-      <c r="E53" s="6"/>
-      <c r="F53" s="15"/>
-      <c r="G53" s="6"/>
+      <c r="A53" s="25" t="s">
+        <v>250</v>
+      </c>
+      <c r="B53" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="E53" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F53" s="15">
+        <v>-1</v>
+      </c>
+      <c r="G53" s="6" t="s">
+        <v>63</v>
+      </c>
       <c r="H53" s="6"/>
       <c r="I53" s="6"/>
-      <c r="J53" s="6"/>
-      <c r="K53" s="6"/>
-      <c r="L53" s="6"/>
+      <c r="J53" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="K53" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="L53" s="6" t="s">
+        <v>258</v>
+      </c>
       <c r="M53" s="6"/>
-      <c r="N53" s="6"/>
+      <c r="N53" s="6">
+        <v>5</v>
+      </c>
       <c r="O53" s="6"/>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A54" s="6"/>
-      <c r="B54" s="6"/>
-      <c r="C54" s="6"/>
-      <c r="D54" s="6"/>
-      <c r="E54" s="6"/>
-      <c r="F54" s="15"/>
-      <c r="G54" s="6"/>
-      <c r="H54" s="6"/>
+      <c r="A54" s="25" t="s">
+        <v>250</v>
+      </c>
+      <c r="B54" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="E54" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="F54" s="15">
+        <v>-1</v>
+      </c>
+      <c r="G54" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="H54" s="6" t="s">
+        <v>73</v>
+      </c>
       <c r="I54" s="6"/>
-      <c r="J54" s="6"/>
-      <c r="K54" s="6"/>
-      <c r="L54" s="6"/>
+      <c r="J54" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="K54" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="L54" s="6" t="s">
+        <v>261</v>
+      </c>
       <c r="M54" s="6"/>
-      <c r="N54" s="6"/>
-      <c r="O54" s="6"/>
+      <c r="N54" s="6">
+        <v>20</v>
+      </c>
+      <c r="O54" s="6" t="s">
+        <v>262</v>
+      </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A55" s="6"/>
-      <c r="B55" s="6"/>
-      <c r="C55" s="6"/>
-      <c r="D55" s="6"/>
-      <c r="E55" s="6"/>
-      <c r="F55" s="15"/>
-      <c r="G55" s="6"/>
-      <c r="H55" s="6"/>
+      <c r="A55" s="25" t="s">
+        <v>250</v>
+      </c>
+      <c r="B55" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="E55" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="F55" s="15">
+        <v>-1</v>
+      </c>
+      <c r="G55" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="H55" s="6" t="s">
+        <v>77</v>
+      </c>
       <c r="I55" s="6"/>
-      <c r="J55" s="6"/>
-      <c r="K55" s="6"/>
-      <c r="L55" s="6"/>
+      <c r="J55" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="K55" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="L55" s="6" t="s">
+        <v>263</v>
+      </c>
       <c r="M55" s="6"/>
       <c r="N55" s="6"/>
       <c r="O55" s="6"/>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A56" s="6"/>
-      <c r="B56" s="6"/>
-      <c r="C56" s="6"/>
-      <c r="D56" s="6"/>
-      <c r="E56" s="6"/>
-      <c r="F56" s="15"/>
-      <c r="G56" s="6"/>
+      <c r="A56" s="25" t="s">
+        <v>250</v>
+      </c>
+      <c r="B56" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="D56" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="E56" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="F56" s="15">
+        <v>-1</v>
+      </c>
+      <c r="G56" s="6" t="s">
+        <v>63</v>
+      </c>
       <c r="H56" s="6"/>
       <c r="I56" s="6"/>
-      <c r="J56" s="6"/>
-      <c r="K56" s="6"/>
-      <c r="L56" s="6"/>
+      <c r="J56" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="K56" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="L56" s="6" t="s">
+        <v>267</v>
+      </c>
       <c r="M56" s="6"/>
       <c r="N56" s="6"/>
-      <c r="O56" s="6"/>
+      <c r="O56" s="6" t="s">
+        <v>268</v>
+      </c>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A57" s="6"/>
-      <c r="B57" s="6"/>
-      <c r="C57" s="6"/>
-      <c r="D57" s="6"/>
-      <c r="E57" s="6"/>
-      <c r="F57" s="15"/>
-      <c r="G57" s="6"/>
+      <c r="A57" s="25" t="s">
+        <v>250</v>
+      </c>
+      <c r="B57" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="E57" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="F57" s="15">
+        <v>-1</v>
+      </c>
+      <c r="G57" s="6" t="s">
+        <v>63</v>
+      </c>
       <c r="H57" s="6"/>
       <c r="I57" s="6"/>
-      <c r="J57" s="6"/>
-      <c r="K57" s="6"/>
-      <c r="L57" s="6"/>
+      <c r="J57" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="K57" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="L57" s="6" t="s">
+        <v>270</v>
+      </c>
       <c r="M57" s="6"/>
       <c r="N57" s="6"/>
       <c r="O57" s="6"/>
@@ -9573,67 +9777,16 @@
       <c r="N399" s="6"/>
       <c r="O399" s="6"/>
     </row>
-    <row r="400" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A400" s="6"/>
-      <c r="B400" s="6"/>
-      <c r="C400" s="6"/>
-      <c r="D400" s="6"/>
-      <c r="E400" s="6"/>
-      <c r="F400" s="15"/>
-      <c r="G400" s="6"/>
-      <c r="H400" s="6"/>
-      <c r="I400" s="6"/>
-      <c r="J400" s="6"/>
-      <c r="K400" s="6"/>
-      <c r="L400" s="6"/>
-      <c r="M400" s="6"/>
-      <c r="N400" s="6"/>
-      <c r="O400" s="6"/>
-    </row>
-    <row r="401" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A401" s="6"/>
-      <c r="B401" s="6"/>
-      <c r="C401" s="6"/>
-      <c r="D401" s="6"/>
-      <c r="E401" s="6"/>
-      <c r="F401" s="15"/>
-      <c r="G401" s="6"/>
-      <c r="H401" s="6"/>
-      <c r="I401" s="6"/>
-      <c r="J401" s="6"/>
-      <c r="K401" s="6"/>
-      <c r="L401" s="6"/>
-      <c r="M401" s="6"/>
-      <c r="N401" s="6"/>
-      <c r="O401" s="6"/>
-    </row>
-    <row r="402" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A402" s="6"/>
-      <c r="B402" s="6"/>
-      <c r="C402" s="6"/>
-      <c r="D402" s="6"/>
-      <c r="E402" s="6"/>
-      <c r="F402" s="15"/>
-      <c r="G402" s="6"/>
-      <c r="H402" s="6"/>
-      <c r="I402" s="6"/>
-      <c r="J402" s="6"/>
-      <c r="K402" s="6"/>
-      <c r="L402" s="6"/>
-      <c r="M402" s="6"/>
-      <c r="N402" s="6"/>
-      <c r="O402" s="6"/>
-    </row>
   </sheetData>
   <autoFilter ref="A1:O48" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" sqref="G2:G29 G32:G402" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="G2:G29 G32:G399" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Statement,Question,Statement-Roll"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="G30:G31" xr:uid="{978F0CFC-32AF-4B55-9CBC-7DF8E8F9C2A9}">
       <formula1>"Statement,Question-YN,Question-MultiChoice"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D2:D402" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D2:D399" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Proximity,Trade-completion,Level-reached"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
NPCs set up for Magincia, Minoc, Yew.  XLS updates.
</commit_message>
<xml_diff>
--- a/spoilers/conversations.xlsx
+++ b/spoilers/conversations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MYDATA\_GIT_REPOS\mcu4\spoilers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D73BECF-D7C0-469E-8845-A1501394E242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7FD2239-7E2D-4CC2-B72A-397F949A4545}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="11964" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,14 +21,14 @@
     <externalReference r:id="rId4"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Conversations!$A$1:$O$144</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Conversations!$A$1:$O$147</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1329" uniqueCount="509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1339" uniqueCount="515">
   <si>
     <t>Game-Level Conversation List</t>
   </si>
@@ -654,9 +654,6 @@
     <t>I love acronyms</t>
   </si>
   <si>
-    <t xml:space="preserve">My name SWEN is an acronym for NEWS. </t>
-  </si>
-  <si>
     <t>Hero</t>
   </si>
   <si>
@@ -679,9 +676,6 @@
   </si>
   <si>
     <t>Swen: Folks in Jhelom are valiant but too serious.</t>
-  </si>
-  <si>
-    <t>Swen: My name SWEN is an acronym for NEWS.</t>
   </si>
   <si>
     <t>Swen: I've been everywhere, man…in Jhelom</t>
@@ -1579,6 +1573,30 @@
   </si>
   <si>
     <t>Fires after "I teach Enlightenment"</t>
+  </si>
+  <si>
+    <t>My name SWEN is an acronym for NEWS.  Or, NESW…</t>
+  </si>
+  <si>
+    <t>Swen: My name SWEN is an acronym for NEWS. Or, NESW…</t>
+  </si>
+  <si>
+    <t>Yew</t>
+  </si>
+  <si>
+    <t>Minoc</t>
+  </si>
+  <si>
+    <t>Magincia</t>
+  </si>
+  <si>
+    <t>ALL NPCs tagged but no conversation yet - Aug 30</t>
+  </si>
+  <si>
+    <t>Lycaeum</t>
+  </si>
+  <si>
+    <t>TBD - no NPCs set up yet - Aug 30</t>
   </si>
 </sst>
 </file>
@@ -1693,7 +1711,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1736,6 +1754,12 @@
         <bgColor rgb="FF2F5233"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1764,7 +1788,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1866,6 +1890,15 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -12523,7 +12556,7 @@
             <v>MANT</v>
           </cell>
           <cell r="F528" t="str">
-            <v>The mantra of valor is ’RA’ use it in the shrine on the next isle!</v>
+            <v>The mantra of valor is ’RA’.</v>
           </cell>
         </row>
         <row r="529">
@@ -13928,7 +13961,7 @@
         </row>
         <row r="599">
           <cell r="A599" t="str">
-            <v>Jhelom|Sir William|HEALTH</v>
+            <v>Jhelom|Sir William|VALOR</v>
           </cell>
           <cell r="B599" t="str">
             <v>Towns</v>
@@ -13940,10 +13973,10 @@
             <v>Sir William</v>
           </cell>
           <cell r="E599" t="str">
-            <v>HEALTH</v>
+            <v>VALOR</v>
           </cell>
           <cell r="F599" t="str">
-            <v>Very well.</v>
+            <v>True valor is seen not in the force of arms, but in the force of will!</v>
           </cell>
         </row>
         <row r="600">
@@ -31503,7 +31536,7 @@
             <v>FELO</v>
           </cell>
           <cell r="F1477" t="str">
-            <v>He is a mean nasty ugly villain!</v>
+            <v>That other felon is a mean nasty ugly villain!</v>
           </cell>
         </row>
         <row r="1478">
@@ -31523,7 +31556,7 @@
             <v>HEALTH</v>
           </cell>
           <cell r="F1478" t="str">
-            <v>Well treated.</v>
+            <v>They treat me judicially, here, though.</v>
           </cell>
         </row>
         <row r="1479">
@@ -31588,7 +31621,7 @@
         </row>
         <row r="1482">
           <cell r="A1482" t="str">
-            <v>Yew|Beggar|SINE</v>
+            <v>Yew|Beggar|I have sinned.</v>
           </cell>
           <cell r="B1482" t="str">
             <v>Towns</v>
@@ -31600,7 +31633,7 @@
             <v>Beggar</v>
           </cell>
           <cell r="E1482" t="str">
-            <v>SINE</v>
+            <v>I have sinned.</v>
           </cell>
           <cell r="F1482" t="str">
             <v>I have gotten chests in the townes and killed non-evil creatures.</v>
@@ -32263,7 +32296,7 @@
             <v>JOB</v>
           </cell>
           <cell r="F1515" t="str">
-            <v>See my poor baby I beg for him.</v>
+            <v>I beg and live hand-to-mouth every day.</v>
           </cell>
         </row>
         <row r="1516">
@@ -32583,7 +32616,7 @@
             <v>FELO</v>
           </cell>
           <cell r="F1531" t="str">
-            <v>That’ll be the right hand cell. careful in there!</v>
+            <v>Felons are jailed in the right hand cell.</v>
           </cell>
         </row>
         <row r="1532">
@@ -32663,7 +32696,7 @@
             <v>MISD</v>
           </cell>
           <cell r="F1535" t="str">
-            <v>That’ll be the left cell.</v>
+            <v>Misdemeanors are jailed in the the left cell.</v>
           </cell>
         </row>
         <row r="1536">
@@ -32808,7 +32841,7 @@
         </row>
         <row r="1543">
           <cell r="A1543" t="str">
-            <v>Yew|Ranger|HEALTH</v>
+            <v>Yew|Ranger Rick|HEALTH</v>
           </cell>
           <cell r="B1543" t="str">
             <v>Towns</v>
@@ -32817,7 +32850,7 @@
             <v>Yew</v>
           </cell>
           <cell r="D1543" t="str">
-            <v>Ranger</v>
+            <v>Ranger Rick</v>
           </cell>
           <cell r="E1543" t="str">
             <v>HEALTH</v>
@@ -32828,7 +32861,7 @@
         </row>
         <row r="1544">
           <cell r="A1544" t="str">
-            <v>Yew|Ranger|HOME</v>
+            <v>Yew|Ranger Rick|HOME</v>
           </cell>
           <cell r="B1544" t="str">
             <v>Towns</v>
@@ -32837,7 +32870,7 @@
             <v>Yew</v>
           </cell>
           <cell r="D1544" t="str">
-            <v>Ranger</v>
+            <v>Ranger Rick</v>
           </cell>
           <cell r="E1544" t="str">
             <v>HOME</v>
@@ -32848,7 +32881,7 @@
         </row>
         <row r="1545">
           <cell r="A1545" t="str">
-            <v>Yew|Ranger|JOB</v>
+            <v>Yew|Ranger Rick|JOB</v>
           </cell>
           <cell r="B1545" t="str">
             <v>Towns</v>
@@ -32857,7 +32890,7 @@
             <v>Yew</v>
           </cell>
           <cell r="D1545" t="str">
-            <v>Ranger</v>
+            <v>Ranger Rick</v>
           </cell>
           <cell r="E1545" t="str">
             <v>JOB</v>
@@ -32868,7 +32901,7 @@
         </row>
         <row r="1546">
           <cell r="A1546" t="str">
-            <v>Yew|Ranger|LOOK</v>
+            <v>Yew|Ranger Rick|LOOK</v>
           </cell>
           <cell r="B1546" t="str">
             <v>Towns</v>
@@ -32877,7 +32910,7 @@
             <v>Yew</v>
           </cell>
           <cell r="D1546" t="str">
-            <v>Ranger</v>
+            <v>Ranger Rick</v>
           </cell>
           <cell r="E1546" t="str">
             <v>LOOK</v>
@@ -32888,7 +32921,7 @@
         </row>
         <row r="1547">
           <cell r="A1547" t="str">
-            <v>Yew|Ranger|NAME</v>
+            <v>Yew|Ranger Rick|NAME</v>
           </cell>
           <cell r="B1547" t="str">
             <v>Towns</v>
@@ -32897,7 +32930,7 @@
             <v>Yew</v>
           </cell>
           <cell r="D1547" t="str">
-            <v>Ranger</v>
+            <v>Ranger Rick</v>
           </cell>
           <cell r="E1547" t="str">
             <v>NAME</v>
@@ -32908,7 +32941,7 @@
         </row>
         <row r="1548">
           <cell r="A1548" t="str">
-            <v>Yew|Ranger|RANG</v>
+            <v>Yew|Ranger Rick|RANG</v>
           </cell>
           <cell r="B1548" t="str">
             <v>Towns</v>
@@ -32917,7 +32950,7 @@
             <v>Yew</v>
           </cell>
           <cell r="D1548" t="str">
-            <v>Ranger</v>
+            <v>Ranger Rick</v>
           </cell>
           <cell r="E1548" t="str">
             <v>RANG</v>
@@ -33203,7 +33236,7 @@
             <v>JUST</v>
           </cell>
           <cell r="F1562" t="str">
-            <v>Justice is truth in action!</v>
+            <v>The virtue of justice draws its nature from the principles of Trust and Wisdom!</v>
           </cell>
         </row>
         <row r="1563">
@@ -35592,7 +35625,7 @@
         <v>206</v>
       </c>
       <c r="L33" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="M33" s="5"/>
       <c r="N33" s="5">
@@ -35632,10 +35665,10 @@
         <v>207</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>208</v>
+        <v>507</v>
       </c>
       <c r="L34" s="5" t="s">
-        <v>217</v>
+        <v>508</v>
       </c>
       <c r="M34" s="5"/>
       <c r="N34" s="5">
@@ -35678,7 +35711,7 @@
         <v>193</v>
       </c>
       <c r="L35" s="5" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="M35" s="5"/>
       <c r="N35" s="5">
@@ -35721,7 +35754,7 @@
         <v>198</v>
       </c>
       <c r="L36" s="5" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="M36" s="5"/>
       <c r="N36" s="5">
@@ -35764,7 +35797,7 @@
         <v>202</v>
       </c>
       <c r="L37" s="5" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="M37" s="5"/>
       <c r="N37" s="5">
@@ -35807,7 +35840,7 @@
         <v>192</v>
       </c>
       <c r="L38" s="5" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="M38" s="5"/>
       <c r="N38" s="5">
@@ -35850,7 +35883,7 @@
         <v>200</v>
       </c>
       <c r="L39" s="5" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="M39" s="5"/>
       <c r="N39" s="5">
@@ -35893,7 +35926,7 @@
         <v>196</v>
       </c>
       <c r="L40" s="5" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="M40" s="5"/>
       <c r="N40" s="5">
@@ -35936,7 +35969,7 @@
         <v>197</v>
       </c>
       <c r="L41" s="5" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="M41" s="5"/>
       <c r="N41" s="5">
@@ -35979,7 +36012,7 @@
         <v>204</v>
       </c>
       <c r="L42" s="5" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="M42" s="5"/>
       <c r="N42" s="5">
@@ -36022,7 +36055,7 @@
         <v>203</v>
       </c>
       <c r="L43" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="M43" s="5"/>
       <c r="N43" s="5">
@@ -36037,7 +36070,7 @@
         <v>189</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C44" s="5" t="s">
         <v>142</v>
@@ -36059,20 +36092,20 @@
         <v>40</v>
       </c>
       <c r="J44" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="K44" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="L44" s="5" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="M44" s="5"/>
       <c r="N44" s="5">
         <v>5</v>
       </c>
       <c r="O44" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="45" spans="1:15" s="22" customFormat="1" x14ac:dyDescent="0.3">
@@ -36080,7 +36113,7 @@
         <v>189</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C45" s="5" t="s">
         <v>142</v>
@@ -36102,20 +36135,20 @@
         <v>40</v>
       </c>
       <c r="J45" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="K45" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="K45" s="5" t="s">
-        <v>214</v>
-      </c>
       <c r="L45" s="5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="M45" s="5"/>
       <c r="N45" s="5">
         <v>5</v>
       </c>
       <c r="O45" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="46" spans="1:15" s="22" customFormat="1" x14ac:dyDescent="0.3">
@@ -36123,7 +36156,7 @@
         <v>189</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C46" s="5" t="s">
         <v>142</v>
@@ -36150,10 +36183,10 @@
         <v>74</v>
       </c>
       <c r="K46" s="4" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="L46" s="4" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="M46" s="4">
         <v>100</v>
@@ -36162,7 +36195,7 @@
         <v>20</v>
       </c>
       <c r="O46" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="47" spans="1:15" s="22" customFormat="1" x14ac:dyDescent="0.3">
@@ -36170,7 +36203,7 @@
         <v>189</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C47" s="5" t="s">
         <v>142</v>
@@ -36197,17 +36230,17 @@
         <v>74</v>
       </c>
       <c r="K47" s="4" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="L47" s="4" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="M47" s="4"/>
       <c r="N47" s="4">
         <v>-100</v>
       </c>
       <c r="O47" s="5" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="48" spans="1:15" s="22" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
@@ -36215,7 +36248,7 @@
         <v>189</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>142</v>
@@ -36224,7 +36257,7 @@
         <v>79</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="F48" s="13">
         <v>-1</v>
@@ -36235,20 +36268,20 @@
       <c r="H48" s="5"/>
       <c r="I48" s="5"/>
       <c r="J48" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="K48" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="L48" s="5" t="s">
         <v>233</v>
-      </c>
-      <c r="K48" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="L48" s="5" t="s">
-        <v>235</v>
       </c>
       <c r="M48" s="5"/>
       <c r="N48" s="5">
         <v>5</v>
       </c>
       <c r="O48" s="5" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.3">
@@ -36256,10 +36289,10 @@
         <v>189</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D49" s="7" t="s">
         <v>61</v>
@@ -36278,20 +36311,20 @@
         <v>30</v>
       </c>
       <c r="J49" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="K49" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="K49" s="5" t="s">
-        <v>242</v>
-      </c>
       <c r="L49" s="5" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="M49" s="5"/>
       <c r="N49" s="5">
         <v>0</v>
       </c>
       <c r="O49" s="5" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.3">
@@ -36299,10 +36332,10 @@
         <v>189</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D50" s="7" t="s">
         <v>61</v>
@@ -36321,20 +36354,20 @@
         <v>30</v>
       </c>
       <c r="J50" s="5" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="K50" s="5" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="L50" s="5" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="M50" s="5"/>
       <c r="N50" s="5">
         <v>0</v>
       </c>
       <c r="O50" s="5" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.3">
@@ -36342,10 +36375,10 @@
         <v>189</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D51" s="7" t="s">
         <v>61</v>
@@ -36364,31 +36397,31 @@
         <v>40</v>
       </c>
       <c r="J51" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="K51" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="L51" s="5" t="s">
         <v>246</v>
-      </c>
-      <c r="K51" s="5" t="s">
-        <v>247</v>
-      </c>
-      <c r="L51" s="5" t="s">
-        <v>248</v>
       </c>
       <c r="M51" s="5"/>
       <c r="N51" s="5">
         <v>0</v>
       </c>
       <c r="O51" s="5" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52" s="23" t="s">
+        <v>248</v>
+      </c>
+      <c r="B52" s="10" t="s">
+        <v>249</v>
+      </c>
+      <c r="C52" s="5" t="s">
         <v>250</v>
-      </c>
-      <c r="B52" s="10" t="s">
-        <v>251</v>
-      </c>
-      <c r="C52" s="5" t="s">
-        <v>252</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>61</v>
@@ -36407,13 +36440,13 @@
         <v>100</v>
       </c>
       <c r="J52" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="K52" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="L52" s="5" t="s">
         <v>253</v>
-      </c>
-      <c r="K52" s="5" t="s">
-        <v>254</v>
-      </c>
-      <c r="L52" s="5" t="s">
-        <v>255</v>
       </c>
       <c r="M52" s="5"/>
       <c r="N52" s="5"/>
@@ -36421,13 +36454,13 @@
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A53" s="23" t="s">
+        <v>248</v>
+      </c>
+      <c r="B53" s="10" t="s">
+        <v>249</v>
+      </c>
+      <c r="C53" s="5" t="s">
         <v>250</v>
-      </c>
-      <c r="B53" s="10" t="s">
-        <v>251</v>
-      </c>
-      <c r="C53" s="5" t="s">
-        <v>252</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>79</v>
@@ -36443,17 +36476,17 @@
       </c>
       <c r="H53" s="5"/>
       <c r="I53" s="5">
-        <f>INT((1/COUNTIF(B:B,B53))*100)</f>
+        <f t="shared" ref="I53:I91" si="0">INT((1/COUNTIF(B:B,B53))*100)</f>
         <v>16</v>
       </c>
       <c r="J53" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="K53" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="L53" s="5" t="s">
         <v>256</v>
-      </c>
-      <c r="K53" s="5" t="s">
-        <v>257</v>
-      </c>
-      <c r="L53" s="5" t="s">
-        <v>258</v>
       </c>
       <c r="M53" s="5"/>
       <c r="N53" s="5">
@@ -36463,16 +36496,16 @@
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A54" s="23" t="s">
+        <v>248</v>
+      </c>
+      <c r="B54" s="10" t="s">
+        <v>249</v>
+      </c>
+      <c r="C54" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="B54" s="10" t="s">
-        <v>251</v>
-      </c>
-      <c r="C54" s="5" t="s">
-        <v>252</v>
-      </c>
       <c r="D54" s="5" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E54" s="5" t="s">
         <v>154</v>
@@ -36487,38 +36520,38 @@
         <v>73</v>
       </c>
       <c r="I54" s="5">
-        <f>INT((1/COUNTIF(B:B,B54))*100)</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="J54" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="K54" s="5" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="L54" s="5" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="M54" s="5"/>
       <c r="N54" s="5">
         <v>20</v>
       </c>
       <c r="O54" s="5" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A55" s="23" t="s">
+        <v>248</v>
+      </c>
+      <c r="B55" s="10" t="s">
+        <v>249</v>
+      </c>
+      <c r="C55" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="B55" s="10" t="s">
-        <v>251</v>
-      </c>
-      <c r="C55" s="5" t="s">
-        <v>252</v>
-      </c>
       <c r="D55" s="5" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E55" s="5" t="s">
         <v>154</v>
@@ -36533,17 +36566,17 @@
         <v>77</v>
       </c>
       <c r="I55" s="5">
-        <f>INT((1/COUNTIF(B:B,B55))*100)</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="J55" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="K55" s="5" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="L55" s="5" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="M55" s="5"/>
       <c r="N55" s="5"/>
@@ -36551,16 +36584,16 @@
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A56" s="23" t="s">
+        <v>248</v>
+      </c>
+      <c r="B56" s="10" t="s">
+        <v>249</v>
+      </c>
+      <c r="C56" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="B56" s="10" t="s">
-        <v>251</v>
-      </c>
-      <c r="C56" s="5" t="s">
-        <v>252</v>
-      </c>
       <c r="D56" s="5" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="E56" s="5" t="s">
         <v>154</v>
@@ -36573,36 +36606,36 @@
       </c>
       <c r="H56" s="5"/>
       <c r="I56" s="5">
-        <f>INT((1/COUNTIF(B:B,B56))*100)</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="J56" s="5" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="K56" s="5" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="L56" s="5" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="M56" s="5"/>
       <c r="N56" s="5"/>
       <c r="O56" s="5" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A57" s="23" t="s">
+        <v>248</v>
+      </c>
+      <c r="B57" s="10" t="s">
+        <v>249</v>
+      </c>
+      <c r="C57" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="B57" s="10" t="s">
-        <v>251</v>
-      </c>
-      <c r="C57" s="5" t="s">
-        <v>252</v>
-      </c>
       <c r="D57" s="5" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="E57" s="5" t="s">
         <v>154</v>
@@ -36615,17 +36648,17 @@
       </c>
       <c r="H57" s="5"/>
       <c r="I57" s="5">
-        <f>INT((1/COUNTIF(B:B,B57))*100)</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="J57" s="5" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="K57" s="5" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="L57" s="5" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="M57" s="5"/>
       <c r="N57" s="5"/>
@@ -36633,10 +36666,10 @@
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A58" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B58" s="25" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C58" s="28" t="str">
         <f>VLOOKUP(A58&amp;"|"&amp;B58&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -36656,14 +36689,14 @@
       </c>
       <c r="H58" s="5"/>
       <c r="I58" s="5">
-        <f>INT((1/COUNTIF(B:B,B58))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J58" s="24" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="K58" s="24" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="L58" s="5" t="str">
         <f>B58&amp;": "&amp;K58</f>
@@ -36675,10 +36708,10 @@
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A59" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B59" s="25" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C59" s="28" t="str">
         <f>VLOOKUP(A59&amp;"|"&amp;B59&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -36698,17 +36731,17 @@
       </c>
       <c r="H59" s="5"/>
       <c r="I59" s="5">
-        <f>INT((1/COUNTIF(B:B,B59))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J59" s="24" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="K59" s="24" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="L59" s="5" t="str">
-        <f t="shared" ref="L59:L98" si="0">B59&amp;": "&amp;K59</f>
+        <f t="shared" ref="L59:L98" si="1">B59&amp;": "&amp;K59</f>
         <v>Browning: I strive to live an honest life!</v>
       </c>
       <c r="M59" s="5"/>
@@ -36717,10 +36750,10 @@
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A60" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B60" s="25" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C60" s="28" t="str">
         <f>VLOOKUP(A60&amp;"|"&amp;B60&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -36740,17 +36773,17 @@
       </c>
       <c r="H60" s="5"/>
       <c r="I60" s="5">
-        <f>INT((1/COUNTIF(B:B,B60))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J60" s="24" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="K60" s="24" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="L60" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Browning: It is rooted in Knowledge and Courage.</v>
       </c>
       <c r="M60" s="5"/>
@@ -36759,10 +36792,10 @@
     </row>
     <row r="61" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A61" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B61" s="25" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C61" s="28" t="str">
         <f>VLOOKUP(A61&amp;"|"&amp;B61&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -36782,17 +36815,17 @@
       </c>
       <c r="H61" s="5"/>
       <c r="I61" s="5">
-        <f>INT((1/COUNTIF(B:B,B61))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J61" s="25" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="K61" s="25" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="L61" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Calabrini: Yes several types of potions are sold here!</v>
       </c>
       <c r="M61" s="5"/>
@@ -36801,10 +36834,10 @@
     </row>
     <row r="62" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A62" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B62" s="25" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C62" s="28" t="str">
         <f>VLOOKUP(A62&amp;"|"&amp;B62&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -36824,17 +36857,17 @@
       </c>
       <c r="H62" s="5"/>
       <c r="I62" s="5">
-        <f>INT((1/COUNTIF(B:B,B62))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J62" s="24" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="K62" s="24" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="L62" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Calabrini: The housekeeper at the inn is very chatty.</v>
       </c>
       <c r="M62" s="5"/>
@@ -36843,10 +36876,10 @@
     </row>
     <row r="63" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A63" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B63" s="25" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C63" s="28" t="str">
         <f>VLOOKUP(A63&amp;"|"&amp;B63&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -36866,17 +36899,17 @@
       </c>
       <c r="H63" s="5"/>
       <c r="I63" s="5">
-        <f>INT((1/COUNTIF(B:B,B63))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J63" s="24" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="K63" s="25" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="L63" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Calabrini: I bear greetings from the HONEST town of Moonglow.</v>
       </c>
       <c r="M63" s="5"/>
@@ -36885,10 +36918,10 @@
     </row>
     <row r="64" spans="1:15" ht="21.6" x14ac:dyDescent="0.3">
       <c r="A64" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B64" s="25" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C64" s="28" t="str">
         <f>VLOOKUP(A64&amp;"|"&amp;B64&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -36908,17 +36941,17 @@
       </c>
       <c r="H64" s="5"/>
       <c r="I64" s="5">
-        <f>INT((1/COUNTIF(B:B,B64))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J64" s="25" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="K64" s="25" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="L64" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Christen: Honest friends are few!</v>
       </c>
       <c r="M64" s="5"/>
@@ -36927,10 +36960,10 @@
     </row>
     <row r="65" spans="1:15" ht="21.6" x14ac:dyDescent="0.3">
       <c r="A65" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B65" s="25" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C65" s="28" t="str">
         <f>VLOOKUP(A65&amp;"|"&amp;B65&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -36950,17 +36983,17 @@
       </c>
       <c r="H65" s="5"/>
       <c r="I65" s="5">
-        <f>INT((1/COUNTIF(B:B,B65))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J65" s="24" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="K65" s="24" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="L65" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Christen: Imma feeling gooood!</v>
       </c>
       <c r="M65" s="5"/>
@@ -36969,10 +37002,10 @@
     </row>
     <row r="66" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A66" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B66" s="25" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C66" s="28" t="str">
         <f>VLOOKUP(A66&amp;"|"&amp;B66&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -36992,17 +37025,17 @@
       </c>
       <c r="H66" s="5"/>
       <c r="I66" s="5">
-        <f>INT((1/COUNTIF(B:B,B66))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J66" s="24" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="K66" s="25" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="L66" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Christen: My friend William knows where the rune of honesty is.</v>
       </c>
       <c r="M66" s="5"/>
@@ -37011,10 +37044,10 @@
     </row>
     <row r="67" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A67" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B67" s="25" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C67" s="28" t="str">
         <f>VLOOKUP(A67&amp;"|"&amp;B67&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37034,17 +37067,17 @@
       </c>
       <c r="H67" s="5"/>
       <c r="I67" s="5">
-        <f>INT((1/COUNTIF(B:B,B67))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J67" s="24" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="K67" s="29" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="L67" s="26" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Christen: Hey, don't open Rebelias' personal chests. That's not honest!</v>
       </c>
       <c r="M67" s="5"/>
@@ -37053,10 +37086,10 @@
     </row>
     <row r="68" spans="1:15" ht="21.6" x14ac:dyDescent="0.3">
       <c r="A68" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B68" s="25" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C68" s="28" t="str">
         <f>VLOOKUP(A68&amp;"|"&amp;B68&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37076,17 +37109,17 @@
       </c>
       <c r="H68" s="5"/>
       <c r="I68" s="5">
-        <f>INT((1/COUNTIF(B:B,B68))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J68" s="24" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="K68" s="24" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="L68" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Christen: The housekeeping nitwit.</v>
       </c>
       <c r="M68" s="5"/>
@@ -37095,10 +37128,10 @@
     </row>
     <row r="69" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A69" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B69" s="25" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C69" s="28" t="str">
         <f>VLOOKUP(A69&amp;"|"&amp;B69&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37118,17 +37151,17 @@
       </c>
       <c r="H69" s="5"/>
       <c r="I69" s="5">
-        <f>INT((1/COUNTIF(B:B,B69))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J69" s="24" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="K69" s="24" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="L69" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Cromwell: A few honest men are better than numbers!</v>
       </c>
       <c r="M69" s="5"/>
@@ -37137,10 +37170,10 @@
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A70" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B70" s="25" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C70" s="28" t="str">
         <f>VLOOKUP(A70&amp;"|"&amp;B70&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37160,17 +37193,17 @@
       </c>
       <c r="H70" s="5"/>
       <c r="I70" s="5">
-        <f>INT((1/COUNTIF(B:B,B70))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J70" s="24" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="K70" s="24" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="L70" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Cromwell: I speak of the virtues of honesty!</v>
       </c>
       <c r="M70" s="5"/>
@@ -37179,10 +37212,10 @@
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A71" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B71" s="25" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C71" s="28" t="str">
         <f>VLOOKUP(A71&amp;"|"&amp;B71&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37202,17 +37235,17 @@
       </c>
       <c r="H71" s="5"/>
       <c r="I71" s="5">
-        <f>INT((1/COUNTIF(B:B,B71))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J71" s="24" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="K71" s="24" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="L71" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Cromwell: The mantra for Honesty is ’AHM’.</v>
       </c>
       <c r="M71" s="5"/>
@@ -37221,10 +37254,10 @@
     </row>
     <row r="72" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A72" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B72" s="25" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C72" s="28" t="str">
         <f>VLOOKUP(A72&amp;"|"&amp;B72&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37244,17 +37277,17 @@
       </c>
       <c r="H72" s="5"/>
       <c r="I72" s="5">
-        <f>INT((1/COUNTIF(B:B,B72))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J72" s="24" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="K72" s="24" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="L72" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Mariah: Yes, I hope to go on a great quest, one day!</v>
       </c>
       <c r="M72" s="5"/>
@@ -37263,10 +37296,10 @@
     </row>
     <row r="73" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A73" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B73" s="25" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C73" s="28" t="str">
         <f>VLOOKUP(A73&amp;"|"&amp;B73&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37286,17 +37319,17 @@
       </c>
       <c r="H73" s="5"/>
       <c r="I73" s="5">
-        <f>INT((1/COUNTIF(B:B,B73))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J73" s="24" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="K73" s="24" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="L73" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Mariah: I tend to the pond fish. It's honest work.</v>
       </c>
       <c r="M73" s="5"/>
@@ -37305,10 +37338,10 @@
     </row>
     <row r="74" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A74" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B74" s="25" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C74" s="28" t="str">
         <f>VLOOKUP(A74&amp;"|"&amp;B74&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37328,17 +37361,17 @@
       </c>
       <c r="H74" s="5"/>
       <c r="I74" s="5">
-        <f>INT((1/COUNTIF(B:B,B74))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J74" s="24" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="K74" s="24" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="L74" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Mariah: The quest of the avatar is noble indeed!</v>
       </c>
       <c r="M74" s="5"/>
@@ -37347,10 +37380,10 @@
     </row>
     <row r="75" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A75" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B75" s="25" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C75" s="28" t="str">
         <f>VLOOKUP(A75&amp;"|"&amp;B75&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37370,17 +37403,17 @@
       </c>
       <c r="H75" s="5"/>
       <c r="I75" s="5">
-        <f>INT((1/COUNTIF(B:B,B75))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J75" s="24" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="K75" s="24" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="L75" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Patric the Humble Shepherd: Humility is not derived from any of the four principles.</v>
       </c>
       <c r="M75" s="5"/>
@@ -37389,10 +37422,10 @@
     </row>
     <row r="76" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A76" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B76" s="25" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C76" s="28" t="str">
         <f>VLOOKUP(A76&amp;"|"&amp;B76&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37412,17 +37445,17 @@
       </c>
       <c r="H76" s="5"/>
       <c r="I76" s="5">
-        <f>INT((1/COUNTIF(B:B,B76))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J76" s="24" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="K76" s="24" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="L76" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Patric the Humble Shepherd: Humility is to act while remaining humble.</v>
       </c>
       <c r="M76" s="5"/>
@@ -37431,10 +37464,10 @@
     </row>
     <row r="77" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A77" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B77" s="25" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C77" s="28" t="str">
         <f>VLOOKUP(A77&amp;"|"&amp;B77&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37454,17 +37487,17 @@
       </c>
       <c r="H77" s="5"/>
       <c r="I77" s="5">
-        <f>INT((1/COUNTIF(B:B,B77))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J77" s="24" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="K77" s="24" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="L77" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Patric the Humble Shepherd: I am a meek shepherd.</v>
       </c>
       <c r="M77" s="5"/>
@@ -37473,10 +37506,10 @@
     </row>
     <row r="78" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A78" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B78" s="25" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C78" s="28" t="str">
         <f>VLOOKUP(A78&amp;"|"&amp;B78&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37496,17 +37529,17 @@
       </c>
       <c r="H78" s="5"/>
       <c r="I78" s="5">
-        <f>INT((1/COUNTIF(B:B,B78))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J78" s="24" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="K78" s="24" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="L78" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Rebelias: Evil still exists in our hearts and souls!</v>
       </c>
       <c r="M78" s="5"/>
@@ -37515,10 +37548,10 @@
     </row>
     <row r="79" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A79" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B79" s="25" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C79" s="28" t="str">
         <f>VLOOKUP(A79&amp;"|"&amp;B79&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37538,17 +37571,17 @@
       </c>
       <c r="H79" s="5"/>
       <c r="I79" s="5">
-        <f>INT((1/COUNTIF(B:B,B79))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J79" s="24" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="K79" s="24" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="L79" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Rebelias: Speak the truth always and shame evil forces!</v>
       </c>
       <c r="M79" s="5"/>
@@ -37557,10 +37590,10 @@
     </row>
     <row r="80" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A80" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B80" s="25" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C80" s="28" t="str">
         <f>VLOOKUP(A80&amp;"|"&amp;B80&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37580,17 +37613,17 @@
       </c>
       <c r="H80" s="5"/>
       <c r="I80" s="5">
-        <f>INT((1/COUNTIF(B:B,B80))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J80" s="24" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="K80" s="24" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="L80" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Rebelias: I live an honest life as a mystic wizard.</v>
       </c>
       <c r="M80" s="5"/>
@@ -37599,10 +37632,10 @@
     </row>
     <row r="81" spans="1:15" ht="21.6" x14ac:dyDescent="0.3">
       <c r="A81" s="29" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B81" s="29" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C81" s="28" t="str">
         <f>VLOOKUP(A81&amp;"|"&amp;B81&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37622,17 +37655,17 @@
       </c>
       <c r="H81" s="5"/>
       <c r="I81" s="5">
-        <f>INT((1/COUNTIF(B:B,B81))*100)</f>
+        <f t="shared" si="0"/>
         <v>100</v>
       </c>
       <c r="J81" s="29" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="K81" s="29" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="L81" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Scatu: I am the Proprietor of Inn</v>
       </c>
       <c r="M81" s="5"/>
@@ -37641,10 +37674,10 @@
     </row>
     <row r="82" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A82" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B82" s="25" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C82" s="28" t="str">
         <f>VLOOKUP(A82&amp;"|"&amp;B82&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37664,17 +37697,17 @@
       </c>
       <c r="H82" s="5"/>
       <c r="I82" s="5">
-        <f>INT((1/COUNTIF(B:B,B82))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J82" s="24" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="K82" s="24" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="L82" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shakespeare: Corruption wins not more than honesty!</v>
       </c>
       <c r="M82" s="5"/>
@@ -37683,10 +37716,10 @@
     </row>
     <row r="83" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A83" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B83" s="25" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C83" s="28" t="str">
         <f>VLOOKUP(A83&amp;"|"&amp;B83&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37706,17 +37739,17 @@
       </c>
       <c r="H83" s="5"/>
       <c r="I83" s="5">
-        <f>INT((1/COUNTIF(B:B,B83))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J83" s="24" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="K83" s="24" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="L83" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shakespeare: Remember, there is no terror in threats for I am strong in honesty!</v>
       </c>
       <c r="M83" s="5"/>
@@ -37725,10 +37758,10 @@
     </row>
     <row r="84" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A84" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B84" s="25" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C84" s="28" t="str">
         <f>VLOOKUP(A84&amp;"|"&amp;B84&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37748,17 +37781,17 @@
       </c>
       <c r="H84" s="5"/>
       <c r="I84" s="5">
-        <f>INT((1/COUNTIF(B:B,B84))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J84" s="24" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="K84" s="24" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="L84" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shakespeare: I create tales of honesty.</v>
       </c>
       <c r="M84" s="5"/>
@@ -37767,10 +37800,10 @@
     </row>
     <row r="85" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A85" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B85" s="25" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C85" s="28" t="str">
         <f>VLOOKUP(A85&amp;"|"&amp;B85&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37790,17 +37823,17 @@
       </c>
       <c r="H85" s="5"/>
       <c r="I85" s="5">
-        <f>INT((1/COUNTIF(B:B,B85))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J85" s="29" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="K85" s="24" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="L85" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shakespeare: A wise wizard.</v>
       </c>
       <c r="M85" s="5"/>
@@ -37809,10 +37842,10 @@
     </row>
     <row r="86" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A86" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B86" s="25" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C86" s="28" t="str">
         <f>VLOOKUP(A86&amp;"|"&amp;B86&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37832,17 +37865,17 @@
       </c>
       <c r="H86" s="5"/>
       <c r="I86" s="5">
-        <f>INT((1/COUNTIF(B:B,B86))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J86" s="24" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="K86" s="24" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="L86" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shakespeare: Shakespeare</v>
       </c>
       <c r="M86" s="5"/>
@@ -37851,10 +37884,10 @@
     </row>
     <row r="87" spans="1:15" ht="21.6" x14ac:dyDescent="0.3">
       <c r="A87" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B87" s="25" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C87" s="28" t="str">
         <f>VLOOKUP(A87&amp;"|"&amp;B87&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37874,17 +37907,17 @@
       </c>
       <c r="H87" s="5"/>
       <c r="I87" s="5">
-        <f>INT((1/COUNTIF(B:B,B87))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J87" s="24" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K87" s="24" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="L87" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shazom: I will soon die.</v>
       </c>
       <c r="M87" s="5"/>
@@ -37893,10 +37926,10 @@
     </row>
     <row r="88" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A88" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B88" s="25" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C88" s="28" t="str">
         <f>VLOOKUP(A88&amp;"|"&amp;B88&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37916,17 +37949,17 @@
       </c>
       <c r="H88" s="5"/>
       <c r="I88" s="5">
-        <f>INT((1/COUNTIF(B:B,B88))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J88" s="24" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="K88" s="24" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="L88" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shazom: I am apprentice to the great wizard Nigel!</v>
       </c>
       <c r="M88" s="5"/>
@@ -37935,10 +37968,10 @@
     </row>
     <row r="89" spans="1:15" ht="21.6" x14ac:dyDescent="0.3">
       <c r="A89" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B89" s="25" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C89" s="28" t="str">
         <f>VLOOKUP(A89&amp;"|"&amp;B89&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -37958,17 +37991,17 @@
       </c>
       <c r="H89" s="5"/>
       <c r="I89" s="5">
-        <f>INT((1/COUNTIF(B:B,B89))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J89" s="29" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="K89" s="24" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="L89" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shazom: A dying young wizard.</v>
       </c>
       <c r="M89" s="5"/>
@@ -37977,10 +38010,10 @@
     </row>
     <row r="90" spans="1:15" ht="21.6" x14ac:dyDescent="0.3">
       <c r="A90" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B90" s="25" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C90" s="28" t="str">
         <f>VLOOKUP(A90&amp;"|"&amp;B90&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -38000,17 +38033,17 @@
       </c>
       <c r="H90" s="5"/>
       <c r="I90" s="5">
-        <f>INT((1/COUNTIF(B:B,B90))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J90" s="24" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="K90" s="24" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="L90" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shazom: Shazom</v>
       </c>
       <c r="M90" s="5"/>
@@ -38019,10 +38052,10 @@
     </row>
     <row r="91" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A91" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B91" s="25" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C91" s="28" t="str">
         <f>VLOOKUP(A91&amp;"|"&amp;B91&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -38042,17 +38075,17 @@
       </c>
       <c r="H91" s="5"/>
       <c r="I91" s="5">
-        <f>INT((1/COUNTIF(B:B,B91))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J91" s="24" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="K91" s="24" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="L91" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shazom: I will soon need to use the spell he calls ’recall’.</v>
       </c>
       <c r="M91" s="5"/>
@@ -38061,10 +38094,10 @@
     </row>
     <row r="92" spans="1:15" ht="21.6" x14ac:dyDescent="0.3">
       <c r="A92" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B92" s="25" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C92" s="28" t="str">
         <f>VLOOKUP(A92&amp;"|"&amp;B92&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -38087,13 +38120,13 @@
         <v>20</v>
       </c>
       <c r="J92" s="24" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="K92" s="24" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="L92" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>William: Pretty good.</v>
       </c>
       <c r="M92" s="5"/>
@@ -38102,10 +38135,10 @@
     </row>
     <row r="93" spans="1:15" ht="21.6" x14ac:dyDescent="0.3">
       <c r="A93" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B93" s="25" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C93" s="28" t="str">
         <f>VLOOKUP(A93&amp;"|"&amp;B93&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -38128,13 +38161,13 @@
         <v>30</v>
       </c>
       <c r="J93" s="29" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="K93" s="25" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="L93" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>William: A Nitwit eating a sandwich.</v>
       </c>
       <c r="M93" s="5"/>
@@ -38143,10 +38176,10 @@
     </row>
     <row r="94" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A94" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B94" s="25" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C94" s="28" t="str">
         <f>VLOOKUP(A94&amp;"|"&amp;B94&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -38169,13 +38202,13 @@
         <v>20</v>
       </c>
       <c r="J94" s="24" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="K94" s="24" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="L94" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>William: Search for the rune of honesty near Mariah’s gold chest!</v>
       </c>
       <c r="M94" s="5"/>
@@ -38184,10 +38217,10 @@
     </row>
     <row r="95" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A95" s="24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B95" s="25" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C95" s="28" t="str">
         <f>VLOOKUP(A95&amp;"|"&amp;B95&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -38210,13 +38243,13 @@
         <v>30</v>
       </c>
       <c r="J95" s="24" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="K95" s="24" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="L95" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>William: It’s a peanut butter and grape jelly on lightly toasted bread!</v>
       </c>
       <c r="M95" s="5"/>
@@ -38225,10 +38258,10 @@
     </row>
     <row r="96" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A96" s="29" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B96" s="29" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C96" s="28" t="str">
         <f>VLOOKUP(A96&amp;"|"&amp;B96&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -38252,13 +38285,13 @@
         <v>100</v>
       </c>
       <c r="J96" s="29" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="K96" s="29" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="L96" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shaman: I am the Proprietor of Sage Deli, here.</v>
       </c>
       <c r="M96" s="5"/>
@@ -38267,10 +38300,10 @@
     </row>
     <row r="97" spans="1:15" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A97" s="29" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B97" s="29" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C97" s="28" t="str">
         <f>VLOOKUP(A97&amp;"|"&amp;B97&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -38294,13 +38327,13 @@
         <v>100</v>
       </c>
       <c r="J97" s="29" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="K97" s="29" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="L97" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Harmony: I am the Proprietor of The Healer shoppe.</v>
       </c>
       <c r="M97" s="5"/>
@@ -38309,10 +38342,10 @@
     </row>
     <row r="98" spans="1:15" ht="21.6" x14ac:dyDescent="0.3">
       <c r="A98" s="27" t="s">
+        <v>277</v>
+      </c>
+      <c r="B98" s="29" t="s">
         <v>279</v>
-      </c>
-      <c r="B98" s="29" t="s">
-        <v>281</v>
       </c>
       <c r="C98" s="28" t="str">
         <f>VLOOKUP(A98&amp;"|"&amp;B98&amp;"|"&amp;"LOOK",'[1]NPC Dialogue'!$A:$F,6,FALSE)</f>
@@ -38336,13 +38369,13 @@
         <v>100</v>
       </c>
       <c r="J98" s="29" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="K98" s="27" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="L98" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Margot: I am the Propriety of Magical Herbs</v>
       </c>
       <c r="M98" s="5"/>
@@ -38351,13 +38384,13 @@
     </row>
     <row r="99" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A99" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B99" s="5" t="s">
+        <v>351</v>
+      </c>
+      <c r="C99" s="5" t="s">
         <v>352</v>
-      </c>
-      <c r="B99" s="5" t="s">
-        <v>353</v>
-      </c>
-      <c r="C99" s="5" t="s">
-        <v>354</v>
       </c>
       <c r="D99" s="5" t="s">
         <v>61</v>
@@ -38376,13 +38409,13 @@
         <v>25</v>
       </c>
       <c r="J99" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="K99" s="5" t="s">
+        <v>354</v>
+      </c>
+      <c r="L99" s="5" t="s">
         <v>355</v>
-      </c>
-      <c r="K99" s="5" t="s">
-        <v>356</v>
-      </c>
-      <c r="L99" s="5" t="s">
-        <v>357</v>
       </c>
       <c r="M99" s="5"/>
       <c r="N99" s="5"/>
@@ -38390,13 +38423,13 @@
     </row>
     <row r="100" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A100" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B100" s="5" t="s">
+        <v>351</v>
+      </c>
+      <c r="C100" s="5" t="s">
         <v>352</v>
-      </c>
-      <c r="B100" s="5" t="s">
-        <v>353</v>
-      </c>
-      <c r="C100" s="5" t="s">
-        <v>354</v>
       </c>
       <c r="D100" s="5" t="s">
         <v>61</v>
@@ -38415,13 +38448,13 @@
         <v>25</v>
       </c>
       <c r="J100" s="5" t="s">
+        <v>356</v>
+      </c>
+      <c r="K100" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="L100" s="5" t="s">
         <v>358</v>
-      </c>
-      <c r="K100" s="5" t="s">
-        <v>359</v>
-      </c>
-      <c r="L100" s="5" t="s">
-        <v>360</v>
       </c>
       <c r="M100" s="5"/>
       <c r="N100" s="5"/>
@@ -38429,13 +38462,13 @@
     </row>
     <row r="101" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A101" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B101" s="5" t="s">
+        <v>351</v>
+      </c>
+      <c r="C101" s="5" t="s">
         <v>352</v>
-      </c>
-      <c r="B101" s="5" t="s">
-        <v>353</v>
-      </c>
-      <c r="C101" s="5" t="s">
-        <v>354</v>
       </c>
       <c r="D101" s="5" t="s">
         <v>61</v>
@@ -38454,13 +38487,13 @@
         <v>25</v>
       </c>
       <c r="J101" s="5" t="s">
+        <v>359</v>
+      </c>
+      <c r="K101" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="L101" s="5" t="s">
         <v>361</v>
-      </c>
-      <c r="K101" s="5" t="s">
-        <v>362</v>
-      </c>
-      <c r="L101" s="5" t="s">
-        <v>363</v>
       </c>
       <c r="M101" s="5"/>
       <c r="N101" s="5"/>
@@ -38468,13 +38501,13 @@
     </row>
     <row r="102" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A102" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B102" s="5" t="s">
+        <v>351</v>
+      </c>
+      <c r="C102" s="5" t="s">
         <v>352</v>
-      </c>
-      <c r="B102" s="5" t="s">
-        <v>353</v>
-      </c>
-      <c r="C102" s="5" t="s">
-        <v>354</v>
       </c>
       <c r="D102" s="5" t="s">
         <v>61</v>
@@ -38493,13 +38526,13 @@
         <v>25</v>
       </c>
       <c r="J102" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="K102" s="5" t="s">
+        <v>363</v>
+      </c>
+      <c r="L102" s="5" t="s">
         <v>364</v>
-      </c>
-      <c r="K102" s="5" t="s">
-        <v>365</v>
-      </c>
-      <c r="L102" s="5" t="s">
-        <v>366</v>
       </c>
       <c r="M102" s="5"/>
       <c r="N102" s="5"/>
@@ -38507,13 +38540,13 @@
     </row>
     <row r="103" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A103" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B103" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="C103" s="5" t="s">
         <v>352</v>
-      </c>
-      <c r="B103" s="5" t="s">
-        <v>368</v>
-      </c>
-      <c r="C103" s="5" t="s">
-        <v>354</v>
       </c>
       <c r="D103" s="5" t="s">
         <v>61</v>
@@ -38532,13 +38565,13 @@
         <v>20</v>
       </c>
       <c r="J103" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="K103" s="5" t="s">
         <v>497</v>
       </c>
-      <c r="K103" s="5" t="s">
-        <v>499</v>
-      </c>
       <c r="L103" s="5" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="M103" s="5"/>
       <c r="N103" s="5">
@@ -38548,13 +38581,13 @@
     </row>
     <row r="104" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A104" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B104" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="C104" s="5" t="s">
         <v>352</v>
-      </c>
-      <c r="B104" s="5" t="s">
-        <v>368</v>
-      </c>
-      <c r="C104" s="5" t="s">
-        <v>354</v>
       </c>
       <c r="D104" s="5" t="s">
         <v>61</v>
@@ -38573,13 +38606,13 @@
         <v>20</v>
       </c>
       <c r="J104" s="5" t="s">
+        <v>370</v>
+      </c>
+      <c r="K104" s="5" t="s">
+        <v>371</v>
+      </c>
+      <c r="L104" s="5" t="s">
         <v>372</v>
-      </c>
-      <c r="K104" s="5" t="s">
-        <v>373</v>
-      </c>
-      <c r="L104" s="5" t="s">
-        <v>374</v>
       </c>
       <c r="M104" s="5"/>
       <c r="N104" s="5"/>
@@ -38587,13 +38620,13 @@
     </row>
     <row r="105" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A105" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B105" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="C105" s="5" t="s">
         <v>352</v>
-      </c>
-      <c r="B105" s="5" t="s">
-        <v>368</v>
-      </c>
-      <c r="C105" s="5" t="s">
-        <v>354</v>
       </c>
       <c r="D105" s="5" t="s">
         <v>61</v>
@@ -38612,13 +38645,13 @@
         <v>20</v>
       </c>
       <c r="J105" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="K105" s="5" t="s">
+        <v>368</v>
+      </c>
+      <c r="L105" s="5" t="s">
         <v>369</v>
-      </c>
-      <c r="K105" s="5" t="s">
-        <v>370</v>
-      </c>
-      <c r="L105" s="5" t="s">
-        <v>371</v>
       </c>
       <c r="M105" s="5"/>
       <c r="N105" s="5">
@@ -38628,13 +38661,13 @@
     </row>
     <row r="106" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A106" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B106" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="C106" s="5" t="s">
         <v>352</v>
-      </c>
-      <c r="B106" s="5" t="s">
-        <v>368</v>
-      </c>
-      <c r="C106" s="5" t="s">
-        <v>354</v>
       </c>
       <c r="D106" s="5" t="s">
         <v>61</v>
@@ -38653,13 +38686,13 @@
         <v>20</v>
       </c>
       <c r="J106" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="K106" s="5" t="s">
         <v>437</v>
       </c>
-      <c r="K106" s="5" t="s">
-        <v>439</v>
-      </c>
       <c r="L106" s="5" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="M106" s="5"/>
       <c r="N106" s="5">
@@ -38669,13 +38702,13 @@
     </row>
     <row r="107" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A107" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B107" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="C107" s="5" t="s">
         <v>352</v>
-      </c>
-      <c r="B107" s="5" t="s">
-        <v>368</v>
-      </c>
-      <c r="C107" s="5" t="s">
-        <v>354</v>
       </c>
       <c r="D107" s="5" t="s">
         <v>61</v>
@@ -38694,13 +38727,13 @@
         <v>20</v>
       </c>
       <c r="J107" s="5" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="K107" s="5" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="L107" s="5" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="M107" s="5"/>
       <c r="N107" s="5">
@@ -38710,13 +38743,13 @@
     </row>
     <row r="108" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A108" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C108" s="5" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D108" s="5" t="s">
         <v>61</v>
@@ -38735,13 +38768,13 @@
         <v>25</v>
       </c>
       <c r="J108" s="5" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="K108" s="5" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="L108" s="5" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="M108" s="5"/>
       <c r="N108" s="5"/>
@@ -38749,13 +38782,13 @@
     </row>
     <row r="109" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A109" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C109" s="5" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D109" s="5" t="s">
         <v>61</v>
@@ -38774,13 +38807,13 @@
         <v>25</v>
       </c>
       <c r="J109" s="5" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="K109" s="5" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="L109" s="5" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="M109" s="5"/>
       <c r="N109" s="5"/>
@@ -38788,13 +38821,13 @@
     </row>
     <row r="110" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A110" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C110" s="5" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D110" s="5" t="s">
         <v>61</v>
@@ -38813,29 +38846,29 @@
         <v>25</v>
       </c>
       <c r="J110" s="5" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="K110" s="5" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="L110" s="5" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="M110" s="5"/>
       <c r="N110" s="5"/>
       <c r="O110" s="5" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="111" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A111" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C111" s="5" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D111" s="5" t="s">
         <v>61</v>
@@ -38854,13 +38887,13 @@
         <v>25</v>
       </c>
       <c r="J111" s="5" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="K111" s="5" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="L111" s="5" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="M111" s="5"/>
       <c r="N111" s="5"/>
@@ -38868,13 +38901,13 @@
     </row>
     <row r="112" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A112" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C112" s="5" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D112" s="5" t="s">
         <v>61</v>
@@ -38893,29 +38926,29 @@
       </c>
       <c r="I112" s="5"/>
       <c r="J112" s="5" t="s">
+        <v>498</v>
+      </c>
+      <c r="K112" s="5" t="s">
+        <v>499</v>
+      </c>
+      <c r="L112" s="5" t="s">
         <v>500</v>
-      </c>
-      <c r="K112" s="5" t="s">
-        <v>501</v>
-      </c>
-      <c r="L112" s="5" t="s">
-        <v>502</v>
       </c>
       <c r="M112" s="5"/>
       <c r="N112" s="5"/>
       <c r="O112" s="5" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
     </row>
     <row r="113" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A113" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B113" s="5" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C113" s="5" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D113" s="5" t="s">
         <v>61</v>
@@ -38934,29 +38967,29 @@
       </c>
       <c r="I113" s="5"/>
       <c r="J113" s="5" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="K113" s="5" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="L113" s="5" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="M113" s="5"/>
       <c r="N113" s="5"/>
       <c r="O113" s="5" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
     </row>
     <row r="114" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A114" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B114" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="C114" s="5" t="s">
         <v>352</v>
-      </c>
-      <c r="B114" s="5" t="s">
-        <v>380</v>
-      </c>
-      <c r="C114" s="5" t="s">
-        <v>354</v>
       </c>
       <c r="D114" s="5" t="s">
         <v>61</v>
@@ -38975,29 +39008,29 @@
         <v>25</v>
       </c>
       <c r="J114" s="5" t="s">
+        <v>379</v>
+      </c>
+      <c r="K114" s="5" t="s">
+        <v>380</v>
+      </c>
+      <c r="L114" s="5" t="s">
         <v>381</v>
-      </c>
-      <c r="K114" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="L114" s="5" t="s">
-        <v>383</v>
       </c>
       <c r="M114" s="5"/>
       <c r="N114" s="5"/>
       <c r="O114" s="5" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="115" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A115" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B115" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="C115" s="5" t="s">
         <v>352</v>
-      </c>
-      <c r="B115" s="5" t="s">
-        <v>380</v>
-      </c>
-      <c r="C115" s="5" t="s">
-        <v>354</v>
       </c>
       <c r="D115" s="5" t="s">
         <v>61</v>
@@ -39016,13 +39049,13 @@
         <v>25</v>
       </c>
       <c r="J115" s="5" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="K115" s="5" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="L115" s="5" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="M115" s="5"/>
       <c r="N115" s="5"/>
@@ -39030,13 +39063,13 @@
     </row>
     <row r="116" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A116" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B116" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="C116" s="5" t="s">
         <v>352</v>
-      </c>
-      <c r="B116" s="5" t="s">
-        <v>380</v>
-      </c>
-      <c r="C116" s="5" t="s">
-        <v>354</v>
       </c>
       <c r="D116" s="5" t="s">
         <v>61</v>
@@ -39055,13 +39088,13 @@
         <v>25</v>
       </c>
       <c r="J116" s="5" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="K116" s="5" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="L116" s="5" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="M116" s="5"/>
       <c r="N116" s="5"/>
@@ -39069,13 +39102,13 @@
     </row>
     <row r="117" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A117" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B117" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="C117" s="5" t="s">
         <v>352</v>
-      </c>
-      <c r="B117" s="5" t="s">
-        <v>380</v>
-      </c>
-      <c r="C117" s="5" t="s">
-        <v>354</v>
       </c>
       <c r="D117" s="5" t="s">
         <v>61</v>
@@ -39094,29 +39127,29 @@
         <v>25</v>
       </c>
       <c r="J117" s="5" t="s">
+        <v>385</v>
+      </c>
+      <c r="K117" s="5" t="s">
+        <v>386</v>
+      </c>
+      <c r="L117" s="5" t="s">
         <v>387</v>
-      </c>
-      <c r="K117" s="5" t="s">
-        <v>388</v>
-      </c>
-      <c r="L117" s="5" t="s">
-        <v>389</v>
       </c>
       <c r="M117" s="5"/>
       <c r="N117" s="5"/>
       <c r="O117" s="5" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="118" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A118" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B118" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="C118" s="5" t="s">
         <v>352</v>
-      </c>
-      <c r="B118" s="5" t="s">
-        <v>380</v>
-      </c>
-      <c r="C118" s="5" t="s">
-        <v>354</v>
       </c>
       <c r="D118" s="5" t="s">
         <v>61</v>
@@ -39135,31 +39168,31 @@
       </c>
       <c r="I118" s="5"/>
       <c r="J118" s="5" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="K118" s="5" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="L118" s="5" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="M118" s="5"/>
       <c r="N118" s="5">
         <v>20</v>
       </c>
       <c r="O118" s="5" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="119" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A119" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B119" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="C119" s="5" t="s">
         <v>352</v>
-      </c>
-      <c r="B119" s="5" t="s">
-        <v>380</v>
-      </c>
-      <c r="C119" s="5" t="s">
-        <v>354</v>
       </c>
       <c r="D119" s="5" t="s">
         <v>61</v>
@@ -39178,13 +39211,13 @@
       </c>
       <c r="I119" s="5"/>
       <c r="J119" s="5" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="K119" s="5" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="L119" s="5" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="M119" s="5"/>
       <c r="N119" s="5">
@@ -39194,19 +39227,19 @@
     </row>
     <row r="120" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A120" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B120" s="10" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C120" s="10" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="D120" s="10" t="s">
         <v>61</v>
       </c>
       <c r="E120" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F120" s="34">
         <v>-1</v>
@@ -39219,13 +39252,13 @@
         <v>15</v>
       </c>
       <c r="J120" s="10" t="s">
+        <v>456</v>
+      </c>
+      <c r="K120" s="10" t="s">
         <v>458</v>
       </c>
-      <c r="K120" s="10" t="s">
-        <v>460</v>
-      </c>
       <c r="L120" s="10" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="M120" s="10"/>
       <c r="N120" s="10"/>
@@ -39233,19 +39266,19 @@
     </row>
     <row r="121" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A121" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B121" s="10" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C121" s="10" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="D121" s="10" t="s">
         <v>61</v>
       </c>
       <c r="E121" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F121" s="34">
         <v>-1</v>
@@ -39258,13 +39291,13 @@
         <v>20</v>
       </c>
       <c r="J121" s="10" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="K121" s="10" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="L121" s="10" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="M121" s="10"/>
       <c r="N121" s="10"/>
@@ -39272,19 +39305,19 @@
     </row>
     <row r="122" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A122" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B122" s="10" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C122" s="10" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="D122" s="10" t="s">
         <v>61</v>
       </c>
       <c r="E122" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F122" s="34">
         <v>-1</v>
@@ -39297,13 +39330,13 @@
         <v>20</v>
       </c>
       <c r="J122" s="10" t="s">
+        <v>460</v>
+      </c>
+      <c r="K122" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="L122" s="10" t="s">
         <v>462</v>
-      </c>
-      <c r="K122" s="10" t="s">
-        <v>463</v>
-      </c>
-      <c r="L122" s="10" t="s">
-        <v>464</v>
       </c>
       <c r="M122" s="10"/>
       <c r="N122" s="10"/>
@@ -39311,19 +39344,19 @@
     </row>
     <row r="123" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A123" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B123" s="10" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C123" s="10" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="D123" s="10" t="s">
         <v>61</v>
       </c>
       <c r="E123" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F123" s="34">
         <v>-1</v>
@@ -39336,35 +39369,35 @@
         <v>15</v>
       </c>
       <c r="J123" s="10" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="K123" s="10" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="L123" s="10" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="M123" s="10"/>
       <c r="N123" s="10"/>
       <c r="O123" s="5" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="124" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A124" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B124" s="10" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C124" s="10" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E124" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F124" s="14">
         <v>-1</v>
@@ -39377,13 +39410,13 @@
       </c>
       <c r="I124" s="5"/>
       <c r="J124" s="5" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="K124" s="5" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="L124" s="5" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="M124" s="5">
         <v>10</v>
@@ -39394,19 +39427,19 @@
     </row>
     <row r="125" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A125" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B125" s="10" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C125" s="10" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="D125" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E125" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F125" s="14">
         <v>-1</v>
@@ -39419,13 +39452,13 @@
       </c>
       <c r="I125" s="5"/>
       <c r="J125" s="5" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="K125" s="5" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="L125" s="5" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="M125" s="5"/>
       <c r="N125" s="5">
@@ -39435,19 +39468,19 @@
     </row>
     <row r="126" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A126" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B126" s="10" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C126" s="10" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="D126" s="10" t="s">
         <v>61</v>
       </c>
       <c r="E126" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F126" s="34">
         <v>-1</v>
@@ -39460,13 +39493,13 @@
         <v>15</v>
       </c>
       <c r="J126" s="10" t="s">
+        <v>416</v>
+      </c>
+      <c r="K126" s="10" t="s">
+        <v>417</v>
+      </c>
+      <c r="L126" s="10" t="s">
         <v>418</v>
-      </c>
-      <c r="K126" s="10" t="s">
-        <v>419</v>
-      </c>
-      <c r="L126" s="10" t="s">
-        <v>420</v>
       </c>
       <c r="M126" s="10"/>
       <c r="N126" s="10"/>
@@ -39474,13 +39507,13 @@
     </row>
     <row r="127" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A127" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B127" s="10" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C127" s="10" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="D127" s="10" t="s">
         <v>61</v>
@@ -39499,13 +39532,13 @@
         <v>15</v>
       </c>
       <c r="J127" s="10" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="K127" s="10" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="L127" s="10" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="M127" s="10"/>
       <c r="N127" s="10"/>
@@ -39513,10 +39546,10 @@
     </row>
     <row r="128" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A128" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B128" s="10" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="C128" s="10" t="s">
         <v>121</v>
@@ -39525,7 +39558,7 @@
         <v>61</v>
       </c>
       <c r="E128" s="10" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F128" s="34">
         <v>-1</v>
@@ -39538,13 +39571,13 @@
         <v>20</v>
       </c>
       <c r="J128" s="10" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="K128" s="10" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="L128" s="10" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="M128" s="10"/>
       <c r="N128" s="10"/>
@@ -39552,10 +39585,10 @@
     </row>
     <row r="129" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A129" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B129" s="10" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="C129" s="10" t="s">
         <v>121</v>
@@ -39564,7 +39597,7 @@
         <v>61</v>
       </c>
       <c r="E129" s="10" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F129" s="34">
         <v>-1</v>
@@ -39577,13 +39610,13 @@
         <v>20</v>
       </c>
       <c r="J129" s="10" t="s">
+        <v>426</v>
+      </c>
+      <c r="K129" s="10" t="s">
+        <v>427</v>
+      </c>
+      <c r="L129" s="10" t="s">
         <v>428</v>
-      </c>
-      <c r="K129" s="10" t="s">
-        <v>429</v>
-      </c>
-      <c r="L129" s="10" t="s">
-        <v>430</v>
       </c>
       <c r="M129" s="10"/>
       <c r="N129" s="10"/>
@@ -39591,10 +39624,10 @@
     </row>
     <row r="130" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A130" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B130" s="10" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="C130" s="10" t="s">
         <v>121</v>
@@ -39603,7 +39636,7 @@
         <v>61</v>
       </c>
       <c r="E130" s="10" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F130" s="34">
         <v>-1</v>
@@ -39616,13 +39649,13 @@
         <v>20</v>
       </c>
       <c r="J130" s="10" t="s">
+        <v>477</v>
+      </c>
+      <c r="K130" s="10" t="s">
+        <v>478</v>
+      </c>
+      <c r="L130" s="10" t="s">
         <v>479</v>
-      </c>
-      <c r="K130" s="10" t="s">
-        <v>480</v>
-      </c>
-      <c r="L130" s="10" t="s">
-        <v>481</v>
       </c>
       <c r="M130" s="10"/>
       <c r="N130" s="10"/>
@@ -39630,10 +39663,10 @@
     </row>
     <row r="131" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A131" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B131" s="10" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="C131" s="10" t="s">
         <v>121</v>
@@ -39642,7 +39675,7 @@
         <v>61</v>
       </c>
       <c r="E131" s="10" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F131" s="34">
         <v>-1</v>
@@ -39655,13 +39688,13 @@
         <v>20</v>
       </c>
       <c r="J131" s="10" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="K131" s="10" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="L131" s="10" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="M131" s="10"/>
       <c r="N131" s="10"/>
@@ -39669,10 +39702,10 @@
     </row>
     <row r="132" spans="1:15" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A132" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B132" s="10" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="C132" s="10" t="s">
         <v>121</v>
@@ -39681,7 +39714,7 @@
         <v>61</v>
       </c>
       <c r="E132" s="10" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F132" s="34">
         <v>-1</v>
@@ -39694,13 +39727,13 @@
         <v>20</v>
       </c>
       <c r="J132" s="10" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="K132" s="10" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="L132" s="10" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="M132" s="10"/>
       <c r="N132" s="10"/>
@@ -39708,19 +39741,19 @@
     </row>
     <row r="133" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A133" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B133" s="5" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C133" s="5" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="D133" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E133" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F133" s="14">
         <v>-1</v>
@@ -39733,13 +39766,13 @@
         <v>25</v>
       </c>
       <c r="J133" s="5" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="K133" s="5" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="L133" s="5" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="M133" s="5"/>
       <c r="N133" s="5"/>
@@ -39747,19 +39780,19 @@
     </row>
     <row r="134" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A134" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B134" s="5" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C134" s="5" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="D134" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E134" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F134" s="14">
         <v>-1</v>
@@ -39772,13 +39805,13 @@
         <v>25</v>
       </c>
       <c r="J134" s="5" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="K134" s="5" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="L134" s="5" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="M134" s="5"/>
       <c r="N134" s="5"/>
@@ -39786,19 +39819,19 @@
     </row>
     <row r="135" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A135" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B135" s="5" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C135" s="5" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="D135" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E135" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F135" s="14">
         <v>-1</v>
@@ -39811,13 +39844,13 @@
         <v>25</v>
       </c>
       <c r="J135" s="5" t="s">
+        <v>405</v>
+      </c>
+      <c r="K135" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="L135" s="5" t="s">
         <v>407</v>
-      </c>
-      <c r="K135" s="5" t="s">
-        <v>408</v>
-      </c>
-      <c r="L135" s="5" t="s">
-        <v>409</v>
       </c>
       <c r="M135" s="5"/>
       <c r="N135" s="5"/>
@@ -39825,19 +39858,19 @@
     </row>
     <row r="136" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A136" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B136" s="5" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C136" s="5" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="D136" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E136" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F136" s="14">
         <v>-1</v>
@@ -39850,35 +39883,35 @@
         <v>25</v>
       </c>
       <c r="J136" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="K136" s="5" t="s">
+        <v>409</v>
+      </c>
+      <c r="L136" s="5" t="s">
         <v>410</v>
-      </c>
-      <c r="K136" s="5" t="s">
-        <v>411</v>
-      </c>
-      <c r="L136" s="5" t="s">
-        <v>412</v>
       </c>
       <c r="M136" s="5"/>
       <c r="N136" s="5"/>
       <c r="O136" s="5" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="137" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A137" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C137" s="5" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="D137" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E137" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F137" s="14">
         <v>-1</v>
@@ -39891,37 +39924,37 @@
       </c>
       <c r="I137" s="5"/>
       <c r="J137" s="5" t="s">
+        <v>421</v>
+      </c>
+      <c r="K137" s="5" t="s">
         <v>423</v>
       </c>
-      <c r="K137" s="5" t="s">
-        <v>425</v>
-      </c>
       <c r="L137" s="5" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="M137" s="5"/>
       <c r="N137" s="5">
         <v>2</v>
       </c>
       <c r="O137" s="5" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="138" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A138" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B138" s="5" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C138" s="5" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="D138" s="5" t="s">
         <v>61</v>
       </c>
       <c r="E138" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F138" s="14">
         <v>-1</v>
@@ -39934,13 +39967,13 @@
       </c>
       <c r="I138" s="5"/>
       <c r="J138" s="5" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="K138" s="5" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="L138" s="5" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="M138" s="5"/>
       <c r="N138" s="5">
@@ -39950,10 +39983,10 @@
     </row>
     <row r="139" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A139" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B139" s="31" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="C139" s="32" t="s">
         <v>142</v>
@@ -39975,10 +40008,10 @@
         <v>100</v>
       </c>
       <c r="J139" s="5" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="K139" s="30" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="L139" s="5" t="str">
         <f>B139&amp;": "&amp;K139</f>
@@ -39990,10 +40023,10 @@
     </row>
     <row r="140" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A140" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B140" s="31" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="C140" s="33" t="s">
         <v>134</v>
@@ -40015,13 +40048,13 @@
         <v>100</v>
       </c>
       <c r="J140" s="5" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="K140" s="30" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="L140" s="5" t="str">
-        <f t="shared" ref="L140:L142" si="1">B140&amp;": "&amp;K140</f>
+        <f t="shared" ref="L140:L142" si="2">B140&amp;": "&amp;K140</f>
         <v>Jumar: I am the Proprietor of Duelling Armour.</v>
       </c>
       <c r="M140" s="5"/>
@@ -40030,10 +40063,10 @@
     </row>
     <row r="141" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A141" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B141" s="31" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="C141" s="32" t="s">
         <v>91</v>
@@ -40055,13 +40088,13 @@
         <v>100</v>
       </c>
       <c r="J141" s="5" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="K141" s="30" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="L141" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>Terran: I am the Proprietor of The Keg Tap.</v>
       </c>
       <c r="M141" s="5"/>
@@ -40070,10 +40103,10 @@
     </row>
     <row r="142" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A142" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B142" s="31" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="C142" s="32" t="s">
         <v>111</v>
@@ -40095,13 +40128,13 @@
         <v>100</v>
       </c>
       <c r="J142" s="5" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="K142" s="30" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="L142" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>Zajac: I am the Proprietor of the Honorable Inn.</v>
       </c>
       <c r="M142" s="5"/>
@@ -40110,10 +40143,10 @@
     </row>
     <row r="143" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A143" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B143" s="31" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="C143" s="32" t="s">
         <v>111</v>
@@ -40135,28 +40168,28 @@
       </c>
       <c r="I143" s="5"/>
       <c r="J143" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="K143" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="L143" s="5" t="s">
         <v>452</v>
-      </c>
-      <c r="K143" s="5" t="s">
-        <v>453</v>
-      </c>
-      <c r="L143" s="5" t="s">
-        <v>454</v>
       </c>
       <c r="M143" s="5"/>
       <c r="N143" s="5">
         <v>50</v>
       </c>
       <c r="O143" s="5" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="144" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A144" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B144" s="31" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="C144" s="32" t="s">
         <v>111</v>
@@ -40178,13 +40211,13 @@
       </c>
       <c r="I144" s="5"/>
       <c r="J144" s="5" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="K144" s="5" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="L144" s="5" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="M144" s="5"/>
       <c r="N144" s="5">
@@ -40193,12 +40226,16 @@
       <c r="O144" s="5"/>
     </row>
     <row r="145" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A145" s="5"/>
-      <c r="B145" s="5"/>
-      <c r="C145" s="5"/>
-      <c r="D145" s="5"/>
-      <c r="E145" s="5"/>
-      <c r="F145" s="14"/>
+      <c r="A145" s="43" t="s">
+        <v>248</v>
+      </c>
+      <c r="B145" s="43" t="s">
+        <v>512</v>
+      </c>
+      <c r="C145" s="43"/>
+      <c r="D145" s="43"/>
+      <c r="E145" s="43"/>
+      <c r="F145" s="44"/>
       <c r="G145" s="5"/>
       <c r="H145" s="5"/>
       <c r="I145" s="5"/>
@@ -40210,12 +40247,16 @@
       <c r="O145" s="5"/>
     </row>
     <row r="146" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A146" s="5"/>
-      <c r="B146" s="5"/>
-      <c r="C146" s="5"/>
-      <c r="D146" s="5"/>
-      <c r="E146" s="5"/>
-      <c r="F146" s="14"/>
+      <c r="A146" s="43" t="s">
+        <v>509</v>
+      </c>
+      <c r="B146" s="43" t="s">
+        <v>512</v>
+      </c>
+      <c r="C146" s="43"/>
+      <c r="D146" s="43"/>
+      <c r="E146" s="43"/>
+      <c r="F146" s="44"/>
       <c r="G146" s="5"/>
       <c r="H146" s="5"/>
       <c r="I146" s="5"/>
@@ -40227,12 +40268,16 @@
       <c r="O146" s="5"/>
     </row>
     <row r="147" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A147" s="5"/>
-      <c r="B147" s="5"/>
-      <c r="C147" s="5"/>
-      <c r="D147" s="5"/>
-      <c r="E147" s="5"/>
-      <c r="F147" s="14"/>
+      <c r="A147" s="43" t="s">
+        <v>510</v>
+      </c>
+      <c r="B147" s="43" t="s">
+        <v>512</v>
+      </c>
+      <c r="C147" s="43"/>
+      <c r="D147" s="43"/>
+      <c r="E147" s="43"/>
+      <c r="F147" s="44"/>
       <c r="G147" s="5"/>
       <c r="H147" s="5"/>
       <c r="I147" s="5"/>
@@ -40244,12 +40289,16 @@
       <c r="O147" s="5"/>
     </row>
     <row r="148" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A148" s="5"/>
-      <c r="B148" s="5"/>
-      <c r="C148" s="5"/>
-      <c r="D148" s="5"/>
-      <c r="E148" s="5"/>
-      <c r="F148" s="14"/>
+      <c r="A148" s="43" t="s">
+        <v>511</v>
+      </c>
+      <c r="B148" s="43" t="s">
+        <v>512</v>
+      </c>
+      <c r="C148" s="43"/>
+      <c r="D148" s="43"/>
+      <c r="E148" s="43"/>
+      <c r="F148" s="44"/>
       <c r="G148" s="5"/>
       <c r="H148" s="5"/>
       <c r="I148" s="5"/>
@@ -40261,12 +40310,16 @@
       <c r="O148" s="5"/>
     </row>
     <row r="149" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A149" s="5"/>
-      <c r="B149" s="5"/>
-      <c r="C149" s="5"/>
-      <c r="D149" s="5"/>
-      <c r="E149" s="5"/>
-      <c r="F149" s="14"/>
+      <c r="A149" s="45" t="s">
+        <v>513</v>
+      </c>
+      <c r="B149" s="47" t="s">
+        <v>514</v>
+      </c>
+      <c r="C149" s="46"/>
+      <c r="D149" s="46"/>
+      <c r="E149" s="46"/>
+      <c r="F149" s="46"/>
       <c r="G149" s="5"/>
       <c r="H149" s="5"/>
       <c r="I149" s="5"/>
@@ -44511,8 +44564,8 @@
       <c r="O398" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O144" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
-  <conditionalFormatting sqref="K144:K1048576 K110:K111 K113:K142 K1:K105">
+  <autoFilter ref="A1:O147" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <conditionalFormatting sqref="K1:K105 K110:K111 K113:K142 K144:K1048576">
     <cfRule type="expression" dxfId="8" priority="15">
       <formula>"&gt;len(20)"</formula>
     </cfRule>
@@ -44522,49 +44575,49 @@
       <formula>"&gt;len(20)"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="K112:L112">
+    <cfRule type="expression" dxfId="6" priority="1">
+      <formula>"&gt;len(20)"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L111">
+    <cfRule type="expression" dxfId="5" priority="3">
+      <formula>"&gt;len(20)"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L113">
+    <cfRule type="expression" dxfId="4" priority="2">
+      <formula>"&gt;len(20)"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="L122">
-    <cfRule type="expression" dxfId="6" priority="10">
+    <cfRule type="expression" dxfId="3" priority="10">
       <formula>"&gt;len(20)"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L124:L125">
-    <cfRule type="expression" dxfId="5" priority="6">
+    <cfRule type="expression" dxfId="2" priority="6">
       <formula>"&gt;len(20)"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L130">
-    <cfRule type="expression" dxfId="4" priority="7">
+    <cfRule type="expression" dxfId="1" priority="7">
       <formula>"&gt;len(20)"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L144">
-    <cfRule type="expression" dxfId="3" priority="11">
+    <cfRule type="expression" dxfId="0" priority="11">
       <formula>"&gt;len(20)"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L111">
-    <cfRule type="expression" dxfId="2" priority="3">
-      <formula>"&gt;len(20)"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L113">
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>"&gt;len(20)"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K112:L112">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>"&gt;len(20)"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="3">
+  <dataValidations disablePrompts="1" count="3">
     <dataValidation type="list" allowBlank="1" sqref="G2:G29 G32:G398" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Statement,Question,Statement-Roll"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="G30:G31" xr:uid="{978F0CFC-32AF-4B55-9CBC-7DF8E8F9C2A9}">
       <formula1>"Statement,Question-YN,Question-MultiChoice"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D2:D398" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D2:D148 D150:D398" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Proximity,Trade-completion,Level-reached"</formula1>
     </dataValidation>
   </dataValidations>
@@ -44588,16 +44641,16 @@
   <sheetData>
     <row r="1" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="35" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="B1" s="35" t="s">
+        <v>471</v>
+      </c>
+      <c r="C1" s="35" t="s">
+        <v>488</v>
+      </c>
+      <c r="D1" s="37" t="s">
         <v>473</v>
-      </c>
-      <c r="C1" s="35" t="s">
-        <v>490</v>
-      </c>
-      <c r="D1" s="37" t="s">
-        <v>475</v>
       </c>
       <c r="E1" s="37">
         <v>2</v>
@@ -44611,30 +44664,30 @@
     </row>
     <row r="2" spans="1:7" s="36" customFormat="1" ht="81.599999999999994" x14ac:dyDescent="0.3">
       <c r="A2" s="36" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="B2" s="36" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="D2" s="38" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="E2" s="38" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="F2" s="38" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="36" customFormat="1" ht="193.8" x14ac:dyDescent="0.3">
       <c r="A3" s="36" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="B3" s="36" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C3" s="38" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="D3" s="38"/>
       <c r="E3" s="38"/>

</xml_diff>